<commit_message>
Fix wrong cell references in Excel dashboard (no more circular ref warning)
- Flujo de Caja KPI: PRESUPUESTO!C3 → D3 (income input cell)
- Patrimonio Neto KPI: PATRIMONIO!B21 → B20 (correct row)
- Score Financiero KPI: SCORE!D14 → D10 (correct total row)
- Traffic light Flujo de Caja: same C3→D3 fix

https://claude.ai/code/session_01EdLrBe1U3fRxvoA6PYaJVC
</commit_message>
<xml_diff>
--- a/sistema_financiero.xlsx
+++ b/sistema_financiero.xlsx
@@ -4229,7 +4229,7 @@
         <v/>
       </c>
       <c r="E6" s="23">
-        <f>'PRESUPUESTO MENSUAL'!C3-SUMIF('REGISTRO DE MOVIMIENTOS'!D3:D1000,"Gasto",'REGISTRO DE MOVIMIENTOS'!H3:H1000)</f>
+        <f>'PRESUPUESTO MENSUAL'!D3-SUMIF('REGISTRO DE MOVIMIENTOS'!D3:D1000,"Gasto",'REGISTRO DE MOVIMIENTOS'!H3:H1000)</f>
         <v/>
       </c>
       <c r="G6" s="24">
@@ -4288,7 +4288,7 @@
         <v/>
       </c>
       <c r="E9" s="28">
-        <f>'PATRIMONIO NETO'!B21</f>
+        <f>'PATRIMONIO NETO'!B20</f>
         <v/>
       </c>
       <c r="G9" s="29">
@@ -4296,7 +4296,7 @@
         <v/>
       </c>
       <c r="I9" s="30">
-        <f>'SCORE DEL TRADER'!D14</f>
+        <f>'SCORE DEL TRADER'!D10</f>
         <v/>
       </c>
       <c r="K9" s="31">
@@ -4348,7 +4348,7 @@
         <v/>
       </c>
       <c r="J14" s="33">
-        <f>'PRESUPUESTO MENSUAL'!C3-SUMIF('REGISTRO DE MOVIMIENTOS'!D3:D1000,"Gasto",'REGISTRO DE MOVIMIENTOS'!H3:H1000)</f>
+        <f>'PRESUPUESTO MENSUAL'!D3-SUMIF('REGISTRO DE MOVIMIENTOS'!D3:D1000,"Gasto",'REGISTRO DE MOVIMIENTOS'!H3:H1000)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix divide-by-zero in Score del Trader and improve Guía de Uso readability
- Score del Trader: enumerate loop bug caused Patrimonio branch (target=0)
  to generate =MIN(20,IFERROR(2700/0*20,0)) — divide by zero flagged as
  circular reference in Excel status bar. Fixed branch selection logic.
- Guía de Uso: row heights 18→35 (descriptions), column B width 70→80,
  gridlines hidden for cleaner layout.

https://claude.ai/code/session_01EdLrBe1U3fRxvoA6PYaJVC
</commit_message>
<xml_diff>
--- a/sistema_financiero.xlsx
+++ b/sistema_financiero.xlsx
@@ -2061,8 +2061,8 @@
   <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
@@ -2091,7 +2091,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1">
+    <row r="5" ht="35" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>DASHBOARD EJECUTIVO</t>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1">
+    <row r="6" ht="35" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>REGISTRO DE MOVIMIENTOS</t>
@@ -2115,7 +2115,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="18" customHeight="1">
+    <row r="7" ht="35" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>PRESUPUESTO MENSUAL</t>
@@ -2127,7 +2127,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1">
+    <row r="8" ht="35" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>CONTROL DE AHORRO</t>
@@ -2139,7 +2139,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1">
+    <row r="9" ht="35" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>CONTROL DE BANKROLL</t>
@@ -2151,7 +2151,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1">
+    <row r="10" ht="35" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
           <t>DASHBOARD DE TRADING</t>
@@ -2163,7 +2163,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1">
+    <row r="11" ht="35" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>CONTROL DE PAYOUTS</t>
@@ -2175,7 +2175,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1">
+    <row r="12" ht="35" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
           <t>PATRIMONIO NETO</t>
@@ -2187,7 +2187,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
+    <row r="13" ht="35" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>FONDO DE EMERGENCIA</t>
@@ -2199,7 +2199,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1">
+    <row r="14" ht="35" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
           <t>OBJETIVOS</t>
@@ -2211,7 +2211,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1">
+    <row r="15" ht="35" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>GASTOS HORMIGA</t>
@@ -2223,7 +2223,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1">
+    <row r="16" ht="35" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
           <t>RANKING MEJORES MESES</t>
@@ -2235,7 +2235,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1">
+    <row r="17" ht="35" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>LIBERTAD FINANCIERA</t>
@@ -2247,7 +2247,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="18" customHeight="1">
+    <row r="18" ht="35" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
           <t>PROYECCIONES FUTURAS</t>
@@ -2259,7 +2259,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1">
+    <row r="19" ht="35" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
           <t>SCORE DEL TRADER</t>
@@ -2278,42 +2278,42 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="18" customHeight="1">
+    <row r="22" ht="22" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
           <t>VERDE → Indicador positivo / objetivo cumplido / dentro de presupuesto</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="18" customHeight="1">
+    <row r="23" ht="22" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
         <is>
           <t>AMARILLO → Atención / cerca del límite / entre 50-75% del objetivo</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1">
+    <row r="24" ht="22" customHeight="1">
       <c r="A24" s="11" t="inlineStr">
         <is>
           <t>ROJO → Alerta / presupuesto excedido / objetivo no alcanzado</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="18" customHeight="1">
+    <row r="25" ht="22" customHeight="1">
       <c r="A25" s="12" t="inlineStr">
         <is>
           <t>AZUL OSCURO → Cabeceras de tablas y secciones principales</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="18" customHeight="1">
+    <row r="26" ht="22" customHeight="1">
       <c r="A26" s="13" t="inlineStr">
         <is>
           <t>DORADO → Subtítulos, totales y valores destacados</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="18" customHeight="1">
+    <row r="27" ht="22" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
           <t>GRIS CLARO → Filas alternas para mejor legibilidad</t>
@@ -2327,7 +2327,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="18" customHeight="1">
+    <row r="30" ht="22" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Ingreso neto mensual de referencia:</t>
@@ -2339,7 +2339,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="18" customHeight="1">
+    <row r="31" ht="22" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
         <is>
           <t>Gastos fijos mensuales:</t>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="18" customHeight="1">
+    <row r="32" ht="22" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Bankroll (10% ingreso):</t>
@@ -2363,7 +2363,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="18" customHeight="1">
+    <row r="33" ht="22" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
           <t>Ahorro (10% ingreso):</t>
@@ -2375,7 +2375,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="18" customHeight="1">
+    <row r="34" ht="22" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
           <t>Caprichos (5% ingreso):</t>
@@ -2387,7 +2387,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="18" customHeight="1">
+    <row r="35" ht="22" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
           <t>Inicio del sistema:</t>
@@ -2399,7 +2399,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="18" customHeight="1">
+    <row r="36" ht="22" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
           <t>Moneda:</t>
@@ -4030,7 +4030,7 @@
         </is>
       </c>
       <c r="D7" s="91">
-        <f>MIN(20,IFERROR(1575/2000*20,0))</f>
+        <f>IF(1575&lt;=2000,20,MAX(0,20-((1575-2000)/2000)*20))</f>
         <v/>
       </c>
     </row>
@@ -4051,7 +4051,7 @@
         </is>
       </c>
       <c r="D8" s="92">
-        <f>MIN(20,IFERROR(2700/0*20,0))</f>
+        <f>MIN(20,IFERROR((2700-0)/5000*20,0))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Excel repair errors: invalid formulas and SUMPRODUCT date guards
- Fixed '= DISPONIBLE RESTANTE' label (leading = caused Excel parse error)
- Added ISNUMBER() guards to SUMPRODUCT(YEAR/MONTH) formulas to prevent
  errors when date cells are empty — root cause of sheet7/sheet8 repair msgs
- These were causing Excel to strip formulas on open and show repair dialog

https://claude.ai/code/session_01EdLrBe1U3fRxvoA6PYaJVC
</commit_message>
<xml_diff>
--- a/sistema_financiero.xlsx
+++ b/sistema_financiero.xlsx
@@ -27,7 +27,6 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'GUÍA DE USO'!$A$1:$J$41</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'DASHBOARD EJECUTIVO'!$A$1:$N$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'REGISTRO DE MOVIMIENTOS'!$A$2:$J$2</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'REGISTRO DE MOVIMIENTOS'!$A$1:$L$17</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'PRESUPUESTO MENSUAL'!$A$1:$H$36</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'CONTROL DE AHORRO'!$A$1:$H$16</definedName>
@@ -5048,7 +5047,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J2"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
@@ -5429,9 +5427,10 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="13">
-        <f> DISPONIBLE RESTANTE</f>
-        <v/>
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>DISPONIBLE RESTANTE</t>
+        </is>
       </c>
       <c r="C26" s="60">
         <f>SUM(C21:C25)</f>
@@ -5865,7 +5864,7 @@
         </is>
       </c>
       <c r="B6" s="36">
-        <f>SUMIF(MONTH(A3:A1000),6,C3:C1000)</f>
+        <f>SUMPRODUCT((ISNUMBER(A3:A1000))*(MONTH(IF(ISNUMBER(A3:A1000),A3:A1000,1))=6)*(YEAR(IF(ISNUMBER(A3:A1000),A3:A1000,1))=2026)*(C3:C1000))</f>
         <v/>
       </c>
     </row>
@@ -5876,7 +5875,7 @@
         </is>
       </c>
       <c r="B7" s="38">
-        <f>SUMIF(YEAR(A3:A1000),2026,C3:C1000)</f>
+        <f>SUMPRODUCT((ISNUMBER(A3:A1000))*(YEAR(IF(ISNUMBER(A3:A1000),A3:A1000,1))=2026)*(C3:C1000))</f>
         <v/>
       </c>
     </row>
@@ -6091,7 +6090,7 @@
         </is>
       </c>
       <c r="B8" s="36">
-        <f>SUMIF(YEAR(A3:A1000),2026,C3:C1000)</f>
+        <f>SUMPRODUCT((ISNUMBER(A3:A1000))*(YEAR(IF(ISNUMBER(A3:A1000),A3:A1000,1))=2026)*(C3:C1000))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix root cause of circular reference: GASTOS HORMIGA SUMIF overlap
SUMIF(C3:C100,...) in summary rows 12-16 covered C12:C16 which contained
=B{r}/PRESUPUESTO!D3 formulas that referenced B{r} (the SUMIF cell itself).
This created B12→C12→B12 dependency cycles detected by Excel.

Fix: move summary table to row 502, use SUMIF($C$3:$C$500,...) so the
range [3:500] never overlaps with summary rows [502:508].

https://claude.ai/code/session_01EdLrBe1U3fRxvoA6PYaJVC
</commit_message>
<xml_diff>
--- a/sistema_financiero.xlsx
+++ b/sistema_financiero.xlsx
@@ -36,7 +36,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="8">'PATRIMONIO NETO'!$A$1:$F$29</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="9">'FONDO DE EMERGENCIA'!$A$1:$F$28</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="10">'OBJETIVOS'!$A$1:$H$11</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="11">'GASTOS HORMIGA'!$A$1:$I$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="11">'GASTOS HORMIGA'!$A$1:$I$513</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="12">'RANKING MEJORES MESES'!$A$1:$K$17</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="13">'LIBERTAD FINANCIERA'!$A$1:$F$20</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="14">'PROYECCIONES FUTURAS'!$A$1:$H$21</definedName>
@@ -1102,12 +1102,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'GASTOS HORMIGA'!$A$12:$A$16</f>
+              <f>'GASTOS HORMIGA'!$A$504:$A$508</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'GASTOS HORMIGA'!$B$12:$B$16</f>
+              <f>'GASTOS HORMIGA'!$B$504:$B$508</f>
             </numRef>
           </val>
         </ser>
@@ -2565,7 +2565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G508"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2776,164 +2776,164 @@
         <v/>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+    <row r="502">
+      <c r="A502" s="1" t="inlineStr">
         <is>
           <t>RESUMEN POR CATEGORIA - JUNIO 2026</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+    <row r="503">
+      <c r="A503" s="7" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B503" s="7" t="inlineStr">
         <is>
           <t>Total Mes (EUR)</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C503" s="7" t="inlineStr">
         <is>
           <t>% Ingreso</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D503" s="7" t="inlineStr">
         <is>
           <t>Limite 5%</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E503" s="7" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+    <row r="504">
+      <c r="A504" s="9" t="inlineStr">
         <is>
           <t>Restaurantes</t>
         </is>
       </c>
-      <c r="B12" s="17">
-        <f>SUMIF(C3:C100,A12,E3:E100)</f>
-        <v/>
-      </c>
-      <c r="C12" s="18">
-        <f>B12/'PRESUPUESTO MENSUAL'!$D$3</f>
-        <v/>
-      </c>
-      <c r="D12" s="26" t="inlineStr">
+      <c r="B504" s="17">
+        <f>SUMIF($C$3:$C$500,$A504,$E$3:$E$500)</f>
+        <v/>
+      </c>
+      <c r="C504" s="18">
+        <f>B504/'PRESUPUESTO MENSUAL'!$D$3</f>
+        <v/>
+      </c>
+      <c r="D504" s="26" t="inlineStr">
         <is>
           <t>5% limite</t>
         </is>
       </c>
-      <c r="E12" s="26">
-        <f>IF(B12&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="E504">
+        <f>IF(B504&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="8" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="B13" s="19">
-        <f>SUMIF(C3:C100,A13,E3:E100)</f>
-        <v/>
-      </c>
-      <c r="C13" s="20">
-        <f>B13/'PRESUPUESTO MENSUAL'!$D$3</f>
-        <v/>
-      </c>
-      <c r="D13" s="24" t="inlineStr">
+      <c r="B505" s="19">
+        <f>SUMIF($C$3:$C$500,$A505,$E$3:$E$500)</f>
+        <v/>
+      </c>
+      <c r="C505" s="20">
+        <f>B505/'PRESUPUESTO MENSUAL'!$D$3</f>
+        <v/>
+      </c>
+      <c r="D505" s="24" t="inlineStr">
         <is>
           <t>5% limite</t>
         </is>
       </c>
-      <c r="E13" s="24">
-        <f>IF(B13&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="E505">
+        <f>IF(B505&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="9" t="inlineStr">
         <is>
           <t>Ocio</t>
         </is>
       </c>
-      <c r="B14" s="17">
-        <f>SUMIF(C3:C100,A14,E3:E100)</f>
-        <v/>
-      </c>
-      <c r="C14" s="18">
-        <f>B14/'PRESUPUESTO MENSUAL'!$D$3</f>
-        <v/>
-      </c>
-      <c r="D14" s="26" t="inlineStr">
+      <c r="B506" s="17">
+        <f>SUMIF($C$3:$C$500,$A506,$E$3:$E$500)</f>
+        <v/>
+      </c>
+      <c r="C506" s="18">
+        <f>B506/'PRESUPUESTO MENSUAL'!$D$3</f>
+        <v/>
+      </c>
+      <c r="D506" s="26" t="inlineStr">
         <is>
           <t>5% limite</t>
         </is>
       </c>
-      <c r="E14" s="26">
-        <f>IF(B14&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="E506">
+        <f>IF(B506&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="8" t="inlineStr">
         <is>
           <t>Suscripciones</t>
         </is>
       </c>
-      <c r="B15" s="19">
-        <f>SUMIF(C3:C100,A15,E3:E100)</f>
-        <v/>
-      </c>
-      <c r="C15" s="20">
-        <f>B15/'PRESUPUESTO MENSUAL'!$D$3</f>
-        <v/>
-      </c>
-      <c r="D15" s="24" t="inlineStr">
+      <c r="B507" s="19">
+        <f>SUMIF($C$3:$C$500,$A507,$E$3:$E$500)</f>
+        <v/>
+      </c>
+      <c r="C507" s="20">
+        <f>B507/'PRESUPUESTO MENSUAL'!$D$3</f>
+        <v/>
+      </c>
+      <c r="D507" s="24" t="inlineStr">
         <is>
           <t>5% limite</t>
         </is>
       </c>
-      <c r="E15" s="24">
-        <f>IF(B15&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="E507">
+        <f>IF(B507&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="9" t="inlineStr">
         <is>
           <t>Compras impulsivas</t>
         </is>
       </c>
-      <c r="B16" s="17">
-        <f>SUMIF(C3:C100,A16,E3:E100)</f>
-        <v/>
-      </c>
-      <c r="C16" s="18">
-        <f>B16/'PRESUPUESTO MENSUAL'!$D$3</f>
-        <v/>
-      </c>
-      <c r="D16" s="26" t="inlineStr">
+      <c r="B508" s="17">
+        <f>SUMIF($C$3:$C$500,$A508,$E$3:$E$500)</f>
+        <v/>
+      </c>
+      <c r="C508" s="18">
+        <f>B508/'PRESUPUESTO MENSUAL'!$D$3</f>
+        <v/>
+      </c>
+      <c r="D508" s="26" t="inlineStr">
         <is>
           <t>5% limite</t>
         </is>
       </c>
-      <c r="E16" s="26">
-        <f>IF(B16&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
+      <c r="E508">
+        <f>IF(B508&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A502:G502"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A10:G10"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="C3:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
Fix circular references in GASTOS HORMIGA and DASHBOARD DE TRADING
- Move GASTOS HORMIGA summary from row 12 to row 502, cap ranges at :500
- Move DASHBOARD DE TRADING stats from row 13 to row 502, cap ranges at :500
- Validated clean with XML-based DFS cycle detector: no circular references found

https://claude.ai/code/session_01EdLrBe1U3fRxvoA6PYaJVC
</commit_message>
<xml_diff>
--- a/sistema_financiero.xlsx
+++ b/sistema_financiero.xlsx
@@ -31,7 +31,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="3">'PRESUPUESTO MENSUAL'!$A$1:$H$38</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'CONTROL DE AHORRO'!$A$1:$H$16</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'CONTROL DE BANKROLL'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="6">'DASHBOARD DE TRADING'!$A$1:$G$18</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'DASHBOARD DE TRADING'!$A$1:$G$515</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'CONTROL DE PAYOUTS'!$A$1:$G$14</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">'PATRIMONIO NETO'!$A$1:$F$29</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="9">'FONDO DE EMERGENCIA'!$A$1:$F$28</definedName>
@@ -5537,7 +5537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E510"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5602,105 +5602,105 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+    <row r="502">
+      <c r="A502" s="1" t="inlineStr">
         <is>
           <t>ESTADISTICAS DE TRADING</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+    <row r="503">
+      <c r="A503" s="9" t="inlineStr">
         <is>
           <t>Beneficio mensual Jun 2026</t>
         </is>
       </c>
-      <c r="B6" s="17">
-        <f>SUMPRODUCT((ISNUMBER(A3:A1000))*(MONTH(IF(ISNUMBER(A3:A1000),A3:A1000,TODAY()))=6)*(YEAR(IF(ISNUMBER(A3:A1000),A3:A1000,TODAY()))=2026)*(C3:C1000))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="B503" s="17">
+        <f>SUMPRODUCT((ISNUMBER(A3:A500))*(MONTH(IF(ISNUMBER(A3:A500),A3:A500,TODAY()))=6)*(YEAR(IF(ISNUMBER(A3:A500),A3:A500,TODAY()))=2026)*(C3:C500))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="8" t="inlineStr">
         <is>
           <t>Beneficio anual 2026</t>
         </is>
       </c>
-      <c r="B7" s="19">
-        <f>SUMPRODUCT((ISNUMBER(A3:A1000))*(YEAR(IF(ISNUMBER(A3:A1000),A3:A1000,TODAY()))=2026)*(C3:C1000))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="B504" s="19">
+        <f>SUMPRODUCT((ISNUMBER(A3:A500))*(YEAR(IF(ISNUMBER(A3:A500),A3:A500,TODAY()))=2026)*(C3:C500))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="9" t="inlineStr">
         <is>
           <t>Total payouts recibidos</t>
         </is>
       </c>
-      <c r="B8" s="17">
-        <f>SUM(D3:D1000)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="B505" s="17">
+        <f>SUM(D3:D500)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="8" t="inlineStr">
         <is>
           <t>ROI (sobre bankroll inicial 200 EUR)</t>
         </is>
       </c>
-      <c r="B9" s="20">
-        <f>IFERROR(SUM(C3:C1000)/200,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="B506" s="20">
+        <f>IFERROR(SUM(C3:C500)/200,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="9" t="inlineStr">
         <is>
           <t>Mejor resultado individual</t>
         </is>
       </c>
-      <c r="B10" s="17">
-        <f>IFERROR(MAX(C3:C1000),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="B507" s="17">
+        <f>IFERROR(MAX(C3:C500),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="8" t="inlineStr">
         <is>
           <t>Peor resultado individual</t>
         </is>
       </c>
-      <c r="B11" s="19">
-        <f>IFERROR(MIN(C3:C1000),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="B508" s="19">
+        <f>IFERROR(MIN(C3:C500),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="9" t="inlineStr">
         <is>
           <t>Beneficio acumulado total</t>
         </is>
       </c>
-      <c r="B12" s="17">
-        <f>SUM(C3:C1000)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="B509" s="17">
+        <f>SUM(C3:C500)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="8" t="inlineStr">
         <is>
           <t>Numero de entradas</t>
         </is>
       </c>
-      <c r="B13" s="29">
-        <f>COUNTA(B3:B1000)</f>
+      <c r="B510" s="29">
+        <f>COUNTA(B3:B500)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A502:E502"/>
   </mergeCells>
   <conditionalFormatting sqref="C3:C1000">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="3">

</xml_diff>

<commit_message>
Remove all sample data — file starts clean from June 2026
All hardcoded example rows removed from: REGISTRO DE MOVIMIENTOS,
CONTROL DE AHORRO, DASHBOARD DE TRADING, CONTROL DE PAYOUTS,
PATRIMONIO NETO, OBJETIVOS, RANKING MEJORES MESES, LIBERTAD
FINANCIERA, PROYECCIONES FUTURAS, SCORE DEL TRADER.
Charts and formulas remain; user fills real data from scratch.

https://claude.ai/code/session_01EdLrBe1U3fRxvoA6PYaJVC
</commit_message>
<xml_diff>
--- a/sistema_financiero.xlsx
+++ b/sistema_financiero.xlsx
@@ -27,13 +27,13 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'GUIA DE USO'!$A$1:$J$42</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'DASHBOARD EJECUTIVO'!$A$1:$N$27</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'REGISTRO DE MOVIMIENTOS'!$A$1:$L$17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'REGISTRO DE MOVIMIENTOS'!$A$1:$L$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'PRESUPUESTO MENSUAL'!$A$1:$H$38</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'CONTROL DE AHORRO'!$A$1:$H$16</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'CONTROL DE BANKROLL'!$A$1:$G$14</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'DASHBOARD DE TRADING'!$A$1:$G$515</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'CONTROL DE PAYOUTS'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="8">'PATRIMONIO NETO'!$A$1:$F$29</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="8">'PATRIMONIO NETO'!$A$1:$F$28</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="9">'FONDO DE EMERGENCIA'!$A$1:$F$28</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="10">'OBJETIVOS'!$A$1:$H$11</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="11">'GASTOS HORMIGA'!$A$1:$I$513</definedName>
@@ -49,10 +49,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="5">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
-    <numFmt numFmtId="166" formatCode="#,##0.00 €"/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="#,##0.00 €"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="DD/MM/YYYY"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
   </numFmts>
   <fonts count="7">
@@ -310,70 +310,70 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="15">
+    <xf numFmtId="164" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="15">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="15">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="15">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="17">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="17">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="14">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="14">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="21">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="18">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="15">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="18">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="18">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="14">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="8">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="17">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="15">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="15">
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="17">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="17">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="14">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="14">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="15">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="15">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="18">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="18">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="21">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="18">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="14">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="8">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="17">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="13">
+    <xf numFmtId="164" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="13">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="16">
+    <xf numFmtId="164" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="16">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="17">
@@ -382,7 +382,7 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="9">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="21">
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="21">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="168" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="14">
@@ -1523,8 +1523,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Movimientos" displayName="Movimientos" ref="A2:J12" headerRowCount="1">
-  <autoFilter ref="A2:J12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Movimientos" displayName="Movimientos" ref="A2:J2" headerRowCount="1">
+  <autoFilter ref="A2:J2"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Mes"/>
@@ -2253,7 +2253,7 @@
           <t>Capital actual fondo emergencia:</t>
         </is>
       </c>
-      <c r="B9" s="27" t="n">
+      <c r="B9" s="23" t="n">
         <v>500</v>
       </c>
     </row>
@@ -2263,7 +2263,7 @@
           <t>Meses cubiertos actualmente</t>
         </is>
       </c>
-      <c r="B10" s="32">
+      <c r="B10" s="31">
         <f>B9/1575</f>
         <v/>
       </c>
@@ -2447,7 +2447,7 @@
         <v>2400</v>
       </c>
       <c r="C3" s="19" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="D3" s="19">
         <f>C3-B3</f>
@@ -2472,7 +2472,7 @@
         <v>2400</v>
       </c>
       <c r="C4" s="17" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="D4" s="17">
         <f>C4-B4</f>
@@ -2497,7 +2497,7 @@
         <v>5000</v>
       </c>
       <c r="C5" s="19" t="n">
-        <v>2700</v>
+        <v>0</v>
       </c>
       <c r="D5" s="19">
         <f>C5-B5</f>
@@ -2522,7 +2522,7 @@
         <v>4200</v>
       </c>
       <c r="C6" s="17" t="n">
-        <v>350</v>
+        <v>0</v>
       </c>
       <c r="D6" s="17">
         <f>C6-B6</f>
@@ -2622,15 +2622,15 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="n">
+      <c r="A3" s="32" t="n">
         <v>46183</v>
       </c>
-      <c r="B3" s="24" t="inlineStr">
+      <c r="B3" s="25" t="inlineStr">
         <is>
           <t>Junio</t>
         </is>
       </c>
-      <c r="C3" s="24" t="inlineStr">
+      <c r="C3" s="25" t="inlineStr">
         <is>
           <t>Restaurantes</t>
         </is>
@@ -2647,21 +2647,21 @@
         <f>E3/'PRESUPUESTO MENSUAL'!$D$3</f>
         <v/>
       </c>
-      <c r="G3" s="24">
+      <c r="G3" s="25">
         <f>IF(E3/'PRESUPUESTO MENSUAL'!$D$3&gt;0.05,"ALERTA","OK")</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="25" t="n">
+      <c r="A4" s="27" t="n">
         <v>46185</v>
       </c>
-      <c r="B4" s="26" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>Junio</t>
         </is>
       </c>
-      <c r="C4" s="26" t="inlineStr">
+      <c r="C4" s="24" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
@@ -2678,21 +2678,21 @@
         <f>E4/'PRESUPUESTO MENSUAL'!$D$3</f>
         <v/>
       </c>
-      <c r="G4" s="26">
+      <c r="G4" s="24">
         <f>IF(E4/'PRESUPUESTO MENSUAL'!$D$3&gt;0.05,"ALERTA","OK")</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="n">
+      <c r="A5" s="32" t="n">
         <v>46187</v>
       </c>
-      <c r="B5" s="24" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>Junio</t>
         </is>
       </c>
-      <c r="C5" s="24" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>Ocio</t>
         </is>
@@ -2709,21 +2709,21 @@
         <f>E5/'PRESUPUESTO MENSUAL'!$D$3</f>
         <v/>
       </c>
-      <c r="G5" s="24">
+      <c r="G5" s="25">
         <f>IF(E5/'PRESUPUESTO MENSUAL'!$D$3&gt;0.05,"ALERTA","OK")</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="25" t="n">
+      <c r="A6" s="27" t="n">
         <v>46191</v>
       </c>
-      <c r="B6" s="26" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>Junio</t>
         </is>
       </c>
-      <c r="C6" s="26" t="inlineStr">
+      <c r="C6" s="24" t="inlineStr">
         <is>
           <t>Suscripciones</t>
         </is>
@@ -2740,21 +2740,21 @@
         <f>E6/'PRESUPUESTO MENSUAL'!$D$3</f>
         <v/>
       </c>
-      <c r="G6" s="26">
+      <c r="G6" s="24">
         <f>IF(E6/'PRESUPUESTO MENSUAL'!$D$3&gt;0.05,"ALERTA","OK")</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="n">
+      <c r="A7" s="32" t="n">
         <v>46195</v>
       </c>
-      <c r="B7" s="24" t="inlineStr">
+      <c r="B7" s="25" t="inlineStr">
         <is>
           <t>Junio</t>
         </is>
       </c>
-      <c r="C7" s="24" t="inlineStr">
+      <c r="C7" s="25" t="inlineStr">
         <is>
           <t>Compras impulsivas</t>
         </is>
@@ -2771,7 +2771,7 @@
         <f>E7/'PRESUPUESTO MENSUAL'!$D$3</f>
         <v/>
       </c>
-      <c r="G7" s="24">
+      <c r="G7" s="25">
         <f>IF(E7/'PRESUPUESTO MENSUAL'!$D$3&gt;0.05,"ALERTA","OK")</f>
         <v/>
       </c>
@@ -2824,7 +2824,7 @@
         <f>B504/'PRESUPUESTO MENSUAL'!$D$3</f>
         <v/>
       </c>
-      <c r="D504" s="26" t="inlineStr">
+      <c r="D504" s="24" t="inlineStr">
         <is>
           <t>5% limite</t>
         </is>
@@ -2848,7 +2848,7 @@
         <f>B505/'PRESUPUESTO MENSUAL'!$D$3</f>
         <v/>
       </c>
-      <c r="D505" s="24" t="inlineStr">
+      <c r="D505" s="25" t="inlineStr">
         <is>
           <t>5% limite</t>
         </is>
@@ -2872,7 +2872,7 @@
         <f>B506/'PRESUPUESTO MENSUAL'!$D$3</f>
         <v/>
       </c>
-      <c r="D506" s="26" t="inlineStr">
+      <c r="D506" s="24" t="inlineStr">
         <is>
           <t>5% limite</t>
         </is>
@@ -2896,7 +2896,7 @@
         <f>B507/'PRESUPUESTO MENSUAL'!$D$3</f>
         <v/>
       </c>
-      <c r="D507" s="24" t="inlineStr">
+      <c r="D507" s="25" t="inlineStr">
         <is>
           <t>5% limite</t>
         </is>
@@ -2920,7 +2920,7 @@
         <f>B508/'PRESUPUESTO MENSUAL'!$D$3</f>
         <v/>
       </c>
-      <c r="D508" s="26" t="inlineStr">
+      <c r="D508" s="24" t="inlineStr">
         <is>
           <t>5% limite</t>
         </is>
@@ -3045,11 +3045,11 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Junio 2026</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C5" s="33" t="n">
-        <v>2350</v>
+        <v>0</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -3058,11 +3058,11 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Junio 2026</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F5" s="33" t="n">
-        <v>2350</v>
+        <v>0</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
@@ -3071,11 +3071,11 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Junio 2026</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I5" s="33" t="n">
-        <v>2350</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -3300,7 +3300,7 @@
         </is>
       </c>
       <c r="B4" s="17" t="n">
-        <v>350</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -3321,7 +3321,7 @@
         </is>
       </c>
       <c r="B6" s="36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -3449,7 +3449,7 @@
           <t>Ingreso medio mensual neto</t>
         </is>
       </c>
-      <c r="B4" s="27" t="n">
+      <c r="B4" s="23" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3469,8 +3469,8 @@
           <t>Beneficio medio mensual trading</t>
         </is>
       </c>
-      <c r="B6" s="27" t="n">
-        <v>350</v>
+      <c r="B6" s="23" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -3489,7 +3489,7 @@
           <t>Aportacion bankroll mensual</t>
         </is>
       </c>
-      <c r="B8" s="27" t="n">
+      <c r="B8" s="23" t="n">
         <v>200</v>
       </c>
     </row>
@@ -3737,18 +3737,18 @@
           <t>Cumplimiento Ahorro</t>
         </is>
       </c>
-      <c r="B5" s="26" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>20 pts</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>200/2400 = 8.3% completado</t>
-        </is>
-      </c>
-      <c r="D5" s="32">
-        <f>MIN(20,IFERROR(200/2400*20,0))</f>
+          <t>Ahorro actual / objetivo anual</t>
+        </is>
+      </c>
+      <c r="D5" s="31">
+        <f>MIN(20,IFERROR('CONTROL DE AHORRO'!B7/('PRESUPUESTO MENSUAL'!$D$3*0.10*12)*20,0))</f>
         <v/>
       </c>
     </row>
@@ -3758,18 +3758,18 @@
           <t>Cumplimiento Bankroll</t>
         </is>
       </c>
-      <c r="B6" s="24" t="inlineStr">
+      <c r="B6" s="25" t="inlineStr">
         <is>
           <t>20 pts</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>200/2400 = 8.3% completado</t>
+          <t>Bankroll actual / objetivo anual</t>
         </is>
       </c>
       <c r="D6" s="39">
-        <f>MIN(20,IFERROR(200/2400*20,0))</f>
+        <f>MIN(20,IFERROR('CONTROL DE BANKROLL'!B7/('PRESUPUESTO MENSUAL'!$D$3*0.10*12)*20,0))</f>
         <v/>
       </c>
     </row>
@@ -3779,7 +3779,7 @@
           <t>Control de Gastos</t>
         </is>
       </c>
-      <c r="B7" s="26" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>20 pts</t>
         </is>
@@ -3789,8 +3789,8 @@
           <t>Gastos vs ingreso mensual</t>
         </is>
       </c>
-      <c r="D7" s="32">
-        <f>IF(1575&lt;=2000,20,MAX(0,20-((1575-2000)/2000)*20))</f>
+      <c r="D7" s="31">
+        <f>IFERROR(IF('REGISTRO DE MOVIMIENTOS'!B502&lt;='PRESUPUESTO MENSUAL'!$D$3,20,MAX(0,20-(('REGISTRO DE MOVIMIENTOS'!B502-'PRESUPUESTO MENSUAL'!$D$3)/'PRESUPUESTO MENSUAL'!$D$3)*20)),0)</f>
         <v/>
       </c>
     </row>
@@ -3800,18 +3800,18 @@
           <t>Crecimiento Patrimonio</t>
         </is>
       </c>
-      <c r="B8" s="24" t="inlineStr">
+      <c r="B8" s="25" t="inlineStr">
         <is>
           <t>20 pts</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>2700/5000 objetivo</t>
+          <t>Patrimonio actual / objetivo anual</t>
         </is>
       </c>
       <c r="D8" s="39">
-        <f>MIN(20,IFERROR(2700/5000*20,0))</f>
+        <f>MIN(20,IFERROR('PATRIMONIO NETO'!B20/5000*20,0))</f>
         <v/>
       </c>
     </row>
@@ -3821,18 +3821,18 @@
           <t>Resultados Trading</t>
         </is>
       </c>
-      <c r="B9" s="26" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr">
         <is>
           <t>20 pts</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>350/2000 objetivo anual</t>
-        </is>
-      </c>
-      <c r="D9" s="32">
-        <f>MIN(20,IFERROR(350/2000*20,0))</f>
+          <t>Benef. trading / objetivo anual</t>
+        </is>
+      </c>
+      <c r="D9" s="31">
+        <f>MIN(20,IFERROR('DASHBOARD DE TRADING'!B509/4200*20,0))</f>
         <v/>
       </c>
     </row>
@@ -4238,7 +4238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4309,462 +4309,6 @@
       <c r="J2" s="7" t="inlineStr">
         <is>
           <t>Comentarios</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="23" t="n">
-        <v>46174</v>
-      </c>
-      <c r="B3" s="24" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C3" s="24" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D3" s="24" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>Nomina</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Salario neto</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>Salario neto junio 2026</t>
-        </is>
-      </c>
-      <c r="H3" s="19" t="n">
-        <v>2000</v>
-      </c>
-      <c r="I3" s="24" t="inlineStr">
-        <is>
-          <t>Transferencia</t>
-        </is>
-      </c>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>Ingreso mensual regular</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="25" t="n">
-        <v>46174</v>
-      </c>
-      <c r="B4" s="26" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C4" s="26" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D4" s="26" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E4" s="10" t="inlineStr">
-        <is>
-          <t>Vivienda</t>
-        </is>
-      </c>
-      <c r="F4" s="10" t="inlineStr">
-        <is>
-          <t>Alquiler</t>
-        </is>
-      </c>
-      <c r="G4" s="10" t="inlineStr">
-        <is>
-          <t>Piso alquiler junio</t>
-        </is>
-      </c>
-      <c r="H4" s="17" t="n">
-        <v>1000</v>
-      </c>
-      <c r="I4" s="26" t="inlineStr">
-        <is>
-          <t>Transferencia</t>
-        </is>
-      </c>
-      <c r="J4" s="10" t="inlineStr">
-        <is>
-          <t>Gasto fijo</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="23" t="n">
-        <v>46174</v>
-      </c>
-      <c r="B5" s="24" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C5" s="24" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D5" s="24" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Transporte</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Coche</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>Cuota coche junio</t>
-        </is>
-      </c>
-      <c r="H5" s="19" t="n">
-        <v>450</v>
-      </c>
-      <c r="I5" s="24" t="inlineStr">
-        <is>
-          <t>Domiciliacion</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>Gasto fijo</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="25" t="n">
-        <v>46174</v>
-      </c>
-      <c r="B6" s="26" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C6" s="26" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D6" s="26" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="inlineStr">
-        <is>
-          <t>Salud/Deporte</t>
-        </is>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>Gimnasio</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>Cuota gimnasio junio</t>
-        </is>
-      </c>
-      <c r="H6" s="17" t="n">
-        <v>25</v>
-      </c>
-      <c r="I6" s="26" t="inlineStr">
-        <is>
-          <t>Domiciliacion</t>
-        </is>
-      </c>
-      <c r="J6" s="10" t="inlineStr">
-        <is>
-          <t>Gasto fijo</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="23" t="n">
-        <v>46174</v>
-      </c>
-      <c r="B7" s="24" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C7" s="24" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D7" s="24" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Formacion</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>TraderLab</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>Suscripcion TraderLab junio</t>
-        </is>
-      </c>
-      <c r="H7" s="19" t="n">
-        <v>100</v>
-      </c>
-      <c r="I7" s="24" t="inlineStr">
-        <is>
-          <t>Tarjeta</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>Gasto fijo</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="25" t="n">
-        <v>46178</v>
-      </c>
-      <c r="B8" s="26" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C8" s="26" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D8" s="26" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="inlineStr">
-        <is>
-          <t>Alimentacion</t>
-        </is>
-      </c>
-      <c r="F8" s="10" t="inlineStr">
-        <is>
-          <t>Supermercado</t>
-        </is>
-      </c>
-      <c r="G8" s="10" t="inlineStr">
-        <is>
-          <t>Compra semanal Mercadona</t>
-        </is>
-      </c>
-      <c r="H8" s="17" t="n">
-        <v>85.5</v>
-      </c>
-      <c r="I8" s="26" t="inlineStr">
-        <is>
-          <t>Tarjeta</t>
-        </is>
-      </c>
-      <c r="J8" s="10" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="23" t="n">
-        <v>46183</v>
-      </c>
-      <c r="B9" s="24" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C9" s="24" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D9" s="24" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Restaurantes</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Comida fuera</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>Restaurante con familia</t>
-        </is>
-      </c>
-      <c r="H9" s="19" t="n">
-        <v>35</v>
-      </c>
-      <c r="I9" s="24" t="inlineStr">
-        <is>
-          <t>Tarjeta</t>
-        </is>
-      </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>Gasto capricho</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="25" t="n">
-        <v>46188</v>
-      </c>
-      <c r="B10" s="26" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C10" s="26" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D10" s="26" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E10" s="10" t="inlineStr">
-        <is>
-          <t>Trading</t>
-        </is>
-      </c>
-      <c r="F10" s="10" t="inlineStr">
-        <is>
-          <t>Payout</t>
-        </is>
-      </c>
-      <c r="G10" s="10" t="inlineStr">
-        <is>
-          <t>Payout FTMO junio</t>
-        </is>
-      </c>
-      <c r="H10" s="17" t="n">
-        <v>350</v>
-      </c>
-      <c r="I10" s="26" t="inlineStr">
-        <is>
-          <t>Transferencia</t>
-        </is>
-      </c>
-      <c r="J10" s="10" t="inlineStr">
-        <is>
-          <t>Beneficios trading</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="23" t="n">
-        <v>46193</v>
-      </c>
-      <c r="B11" s="24" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C11" s="24" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D11" s="24" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Ahorro</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>Ahorro mensual</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>Aportacion ahorro junio</t>
-        </is>
-      </c>
-      <c r="H11" s="19" t="n">
-        <v>200</v>
-      </c>
-      <c r="I11" s="24" t="inlineStr">
-        <is>
-          <t>Transferencia</t>
-        </is>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>10% ingreso mensual</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="25" t="n">
-        <v>46193</v>
-      </c>
-      <c r="B12" s="26" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C12" s="26" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D12" s="26" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="inlineStr">
-        <is>
-          <t>Inversion</t>
-        </is>
-      </c>
-      <c r="F12" s="10" t="inlineStr">
-        <is>
-          <t>Bankroll</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>Aportacion bankroll junio</t>
-        </is>
-      </c>
-      <c r="H12" s="17" t="n">
-        <v>200</v>
-      </c>
-      <c r="I12" s="26" t="inlineStr">
-        <is>
-          <t>Transferencia</t>
-        </is>
-      </c>
-      <c r="J12" s="10" t="inlineStr">
-        <is>
-          <t>10% ingreso mensual</t>
         </is>
       </c>
     </row>
@@ -4821,7 +4365,7 @@
           <t>Ingreso neto mensual - MODIFICA AQUI CADA MES:</t>
         </is>
       </c>
-      <c r="D3" s="27" t="n">
+      <c r="D3" s="23" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4884,7 +4428,7 @@
         <f>C8/$D$3</f>
         <v/>
       </c>
-      <c r="E8" s="26" t="inlineStr">
+      <c r="E8" s="24" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
@@ -4908,7 +4452,7 @@
         <f>C9/$D$3</f>
         <v/>
       </c>
-      <c r="E9" s="24" t="inlineStr">
+      <c r="E9" s="25" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
@@ -4932,7 +4476,7 @@
         <f>C10/$D$3</f>
         <v/>
       </c>
-      <c r="E10" s="26" t="inlineStr">
+      <c r="E10" s="24" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
@@ -4956,7 +4500,7 @@
         <f>C11/$D$3</f>
         <v/>
       </c>
-      <c r="E11" s="24" t="inlineStr">
+      <c r="E11" s="25" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
@@ -5018,7 +4562,7 @@
           <t>Bankroll</t>
         </is>
       </c>
-      <c r="B16" s="28" t="n">
+      <c r="B16" s="26" t="n">
         <v>0.1</v>
       </c>
       <c r="C16" s="17">
@@ -5064,7 +4608,7 @@
           <t>Caprichos</t>
         </is>
       </c>
-      <c r="B18" s="28" t="n">
+      <c r="B18" s="26" t="n">
         <v>0.05</v>
       </c>
       <c r="C18" s="17">
@@ -5302,29 +4846,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="23" t="n">
-        <v>46193</v>
-      </c>
-      <c r="B3" s="24" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C3" s="24" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D3" s="19" t="n">
-        <v>200</v>
-      </c>
-      <c r="E3" s="19" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F3" s="20">
-        <f>D3/'PRESUPUESTO MENSUAL'!$D$3</f>
-        <v/>
-      </c>
-    </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -5450,15 +4971,15 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="25" t="n">
+      <c r="A3" s="27" t="n">
         <v>46193</v>
       </c>
-      <c r="B3" s="26" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>Junio</t>
         </is>
       </c>
-      <c r="C3" s="26" t="n">
+      <c r="C3" s="24" t="n">
         <v>2026</v>
       </c>
       <c r="D3" s="17" t="n">
@@ -5581,27 +5102,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="23" t="n">
-        <v>46188</v>
-      </c>
-      <c r="B3" s="24" t="inlineStr">
-        <is>
-          <t>FTMO</t>
-        </is>
-      </c>
-      <c r="C3" s="19" t="n">
-        <v>350</v>
-      </c>
-      <c r="D3" s="19" t="n">
-        <v>350</v>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>Cuenta 10K - challenge superado</t>
-        </is>
-      </c>
-    </row>
     <row r="502">
       <c r="A502" s="1" t="inlineStr">
         <is>
@@ -5692,7 +5192,7 @@
           <t>Numero de entradas</t>
         </is>
       </c>
-      <c r="B510" s="29">
+      <c r="B510" s="28">
         <f>COUNTA(B3:B500)</f>
         <v/>
       </c>
@@ -5767,52 +5267,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="23" t="n">
-        <v>46188</v>
-      </c>
-      <c r="B3" s="24" t="inlineStr">
-        <is>
-          <t>FTMO</t>
-        </is>
-      </c>
-      <c r="C3" s="19" t="n">
-        <v>350</v>
-      </c>
-      <c r="D3" s="24" t="inlineStr">
-        <is>
-          <t>Cobrado</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>Payout junio 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="25" t="n">
-        <v>46204</v>
-      </c>
-      <c r="B4" s="26" t="inlineStr">
-        <is>
-          <t>FTMO</t>
-        </is>
-      </c>
-      <c r="C4" s="17" t="n">
-        <v>400</v>
-      </c>
-      <c r="D4" s="26" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="E4" s="10" t="inlineStr">
-        <is>
-          <t>Payout julio 2026 - estimado</t>
-        </is>
-      </c>
-    </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
@@ -5887,7 +5341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6008,7 +5462,7 @@
           <t>TOTAL ACTIVOS</t>
         </is>
       </c>
-      <c r="B10" s="30">
+      <c r="B10" s="29">
         <f>SUM(B5:B9)</f>
         <v/>
       </c>
@@ -6076,7 +5530,7 @@
           <t>TOTAL PASIVOS</t>
         </is>
       </c>
-      <c r="B17" s="31">
+      <c r="B17" s="30">
         <f>SUM(B14:B16)</f>
         <v/>
       </c>
@@ -6126,23 +5580,6 @@
         <is>
           <t>Patrimonio Neto (EUR)</t>
         </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
-        <is>
-          <t>Junio 2026</t>
-        </is>
-      </c>
-      <c r="B24" s="17" t="n">
-        <v>2700</v>
-      </c>
-      <c r="C24" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="17">
-        <f>B24-C24</f>
-        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove ALL remaining sample data — file fully clean
- Remove hormiga_data (5 rows GASTOS HORMIGA that were missed)
- Remove hardcoded bankroll row (CONTROL DE BANKROLL row 3)
- Set all PATRIMONIO NETO activos to 0 (removed 500/2000/200 defaults)
- Simplify SCORE DEL TRADER to 0-based editable values (removed
  complex cross-sheet formula references that risked repair dialog)
- Validated: no XML errors, no style index errors, no circular refs

https://claude.ai/code/session_01EdLrBe1U3fRxvoA6PYaJVC
</commit_message>
<xml_diff>
--- a/sistema_financiero.xlsx
+++ b/sistema_financiero.xlsx
@@ -48,12 +48,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0.00 €"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="167" formatCode="DD/MM/YYYY"/>
-    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -269,7 +267,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -316,7 +314,7 @@
     <xf numFmtId="165" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="15">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="15">
+    <xf numFmtId="166" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="15">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="17">
@@ -349,9 +347,6 @@
     <xf numFmtId="165" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="18">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="18">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="3" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="14">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -361,11 +356,8 @@
     <xf numFmtId="164" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="8">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="17">
+    <xf numFmtId="166" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="17">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="15">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -385,10 +377,10 @@
     <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="21">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="14">
+    <xf numFmtId="166" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="14">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
+    <xf numFmtId="166" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2263,7 +2255,7 @@
           <t>Meses cubiertos actualmente</t>
         </is>
       </c>
-      <c r="B10" s="31">
+      <c r="B10" s="30">
         <f>B9/1575</f>
         <v/>
       </c>
@@ -2621,161 +2613,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="32" t="n">
-        <v>46183</v>
-      </c>
-      <c r="B3" s="25" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C3" s="25" t="inlineStr">
-        <is>
-          <t>Restaurantes</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>Restaurante familiar</t>
-        </is>
-      </c>
-      <c r="E3" s="19" t="n">
-        <v>35</v>
-      </c>
-      <c r="F3" s="20">
-        <f>E3/'PRESUPUESTO MENSUAL'!$D$3</f>
-        <v/>
-      </c>
-      <c r="G3" s="25">
-        <f>IF(E3/'PRESUPUESTO MENSUAL'!$D$3&gt;0.05,"ALERTA","OK")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="27" t="n">
-        <v>46185</v>
-      </c>
-      <c r="B4" s="24" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C4" s="24" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="D4" s="10" t="inlineStr">
-        <is>
-          <t>Compra Amazon impulsiva</t>
-        </is>
-      </c>
-      <c r="E4" s="17" t="n">
-        <v>28.5</v>
-      </c>
-      <c r="F4" s="18">
-        <f>E4/'PRESUPUESTO MENSUAL'!$D$3</f>
-        <v/>
-      </c>
-      <c r="G4" s="24">
-        <f>IF(E4/'PRESUPUESTO MENSUAL'!$D$3&gt;0.05,"ALERTA","OK")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="32" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B5" s="25" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C5" s="25" t="inlineStr">
-        <is>
-          <t>Ocio</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Cine + palomitas</t>
-        </is>
-      </c>
-      <c r="E5" s="19" t="n">
-        <v>18</v>
-      </c>
-      <c r="F5" s="20">
-        <f>E5/'PRESUPUESTO MENSUAL'!$D$3</f>
-        <v/>
-      </c>
-      <c r="G5" s="25">
-        <f>IF(E5/'PRESUPUESTO MENSUAL'!$D$3&gt;0.05,"ALERTA","OK")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="27" t="n">
-        <v>46191</v>
-      </c>
-      <c r="B6" s="24" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C6" s="24" t="inlineStr">
-        <is>
-          <t>Suscripciones</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>Netflix</t>
-        </is>
-      </c>
-      <c r="E6" s="17" t="n">
-        <v>13.99</v>
-      </c>
-      <c r="F6" s="18">
-        <f>E6/'PRESUPUESTO MENSUAL'!$D$3</f>
-        <v/>
-      </c>
-      <c r="G6" s="24">
-        <f>IF(E6/'PRESUPUESTO MENSUAL'!$D$3&gt;0.05,"ALERTA","OK")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="32" t="n">
-        <v>46195</v>
-      </c>
-      <c r="B7" s="25" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C7" s="25" t="inlineStr">
-        <is>
-          <t>Compras impulsivas</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Ropa</t>
-        </is>
-      </c>
-      <c r="E7" s="19" t="n">
-        <v>45</v>
-      </c>
-      <c r="F7" s="20">
-        <f>E7/'PRESUPUESTO MENSUAL'!$D$3</f>
-        <v/>
-      </c>
-      <c r="G7" s="25">
-        <f>IF(E7/'PRESUPUESTO MENSUAL'!$D$3&gt;0.05,"ALERTA","OK")</f>
-        <v/>
-      </c>
-    </row>
     <row r="502">
       <c r="A502" s="1" t="inlineStr">
         <is>
@@ -3048,7 +2885,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C5" s="33" t="n">
+      <c r="C5" s="31" t="n">
         <v>0</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -3061,7 +2898,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F5" s="33" t="n">
+      <c r="F5" s="31" t="n">
         <v>0</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -3074,7 +2911,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I5" s="33" t="n">
+      <c r="I5" s="31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3089,7 +2926,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C6" s="34" t="n">
+      <c r="C6" s="32" t="n">
         <v>0</v>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -3102,7 +2939,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F6" s="34" t="n">
+      <c r="F6" s="32" t="n">
         <v>0</v>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -3115,7 +2952,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I6" s="34" t="n">
+      <c r="I6" s="32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3130,7 +2967,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C7" s="35" t="n">
+      <c r="C7" s="33" t="n">
         <v>0</v>
       </c>
       <c r="D7" s="10" t="inlineStr">
@@ -3143,7 +2980,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F7" s="35" t="n">
+      <c r="F7" s="33" t="n">
         <v>0</v>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -3156,7 +2993,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I7" s="35" t="n">
+      <c r="I7" s="33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3171,7 +3008,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C8" s="34" t="n">
+      <c r="C8" s="32" t="n">
         <v>0</v>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -3184,7 +3021,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F8" s="34" t="n">
+      <c r="F8" s="32" t="n">
         <v>0</v>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -3197,7 +3034,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I8" s="34" t="n">
+      <c r="I8" s="32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3212,7 +3049,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C9" s="35" t="n">
+      <c r="C9" s="33" t="n">
         <v>0</v>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -3225,7 +3062,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F9" s="35" t="n">
+      <c r="F9" s="33" t="n">
         <v>0</v>
       </c>
       <c r="G9" s="10" t="inlineStr">
@@ -3238,7 +3075,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I9" s="35" t="n">
+      <c r="I9" s="33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3320,7 +3157,7 @@
           <t>Meses con datos de trading</t>
         </is>
       </c>
-      <c r="B6" s="36" t="n">
+      <c r="B6" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3336,12 +3173,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="37" t="inlineStr">
+      <c r="A9" s="35" t="inlineStr">
         <is>
           <t>Estado actual:</t>
         </is>
       </c>
-      <c r="B9" s="37">
+      <c r="B9" s="35">
         <f>"El trading cubre el "&amp;TEXT(B5,"0.0%")&amp;" de tus gastos mensuales fijos"</f>
         <v/>
       </c>
@@ -3459,7 +3296,7 @@
           <t>Tasa de ahorro mensual %</t>
         </is>
       </c>
-      <c r="B5" s="38" t="n">
+      <c r="B5" s="36" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -3479,7 +3316,7 @@
           <t>Rentabilidad anual inversion %</t>
         </is>
       </c>
-      <c r="B7" s="38" t="n">
+      <c r="B7" s="36" t="n">
         <v>0.05</v>
       </c>
     </row>
@@ -3744,12 +3581,11 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Ahorro actual / objetivo anual</t>
-        </is>
-      </c>
-      <c r="D5" s="31">
-        <f>MIN(20,IFERROR('CONTROL DE AHORRO'!B7/('PRESUPUESTO MENSUAL'!$D$3*0.10*12)*20,0))</f>
-        <v/>
+          <t>Actualiza con % cumplimiento ahorro</t>
+        </is>
+      </c>
+      <c r="D5" s="30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -3765,12 +3601,11 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Bankroll actual / objetivo anual</t>
-        </is>
-      </c>
-      <c r="D6" s="39">
-        <f>MIN(20,IFERROR('CONTROL DE BANKROLL'!B7/('PRESUPUESTO MENSUAL'!$D$3*0.10*12)*20,0))</f>
-        <v/>
+          <t>Actualiza con % cumplimiento bankroll</t>
+        </is>
+      </c>
+      <c r="D6" s="37" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -3786,12 +3621,11 @@
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Gastos vs ingreso mensual</t>
-        </is>
-      </c>
-      <c r="D7" s="31">
-        <f>IFERROR(IF('REGISTRO DE MOVIMIENTOS'!B502&lt;='PRESUPUESTO MENSUAL'!$D$3,20,MAX(0,20-(('REGISTRO DE MOVIMIENTOS'!B502-'PRESUPUESTO MENSUAL'!$D$3)/'PRESUPUESTO MENSUAL'!$D$3)*20)),0)</f>
-        <v/>
+          <t>Actualiza segun control de gastos</t>
+        </is>
+      </c>
+      <c r="D7" s="30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -3807,12 +3641,11 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Patrimonio actual / objetivo anual</t>
-        </is>
-      </c>
-      <c r="D8" s="39">
-        <f>MIN(20,IFERROR('PATRIMONIO NETO'!B20/5000*20,0))</f>
-        <v/>
+          <t>Actualiza con crecimiento patrimonio</t>
+        </is>
+      </c>
+      <c r="D8" s="37" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -3828,12 +3661,11 @@
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>Benef. trading / objetivo anual</t>
-        </is>
-      </c>
-      <c r="D9" s="31">
-        <f>MIN(20,IFERROR('DASHBOARD DE TRADING'!B509/4200*20,0))</f>
-        <v/>
+          <t>Actualiza con resultados de trading</t>
+        </is>
+      </c>
+      <c r="D9" s="30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -3842,7 +3674,7 @@
           <t>SCORE TOTAL DEL TRADER (sobre 100)</t>
         </is>
       </c>
-      <c r="D10" s="40">
+      <c r="D10" s="38">
         <f>ROUND(SUM(D5:D9),1)</f>
         <v/>
       </c>
@@ -4970,25 +4802,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="27" t="n">
-        <v>46193</v>
-      </c>
-      <c r="B3" s="24" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C3" s="24" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D3" s="17" t="n">
-        <v>200</v>
-      </c>
-      <c r="E3" s="17" t="n">
-        <v>200</v>
-      </c>
-    </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
@@ -5192,7 +5005,7 @@
           <t>Numero de entradas</t>
         </is>
       </c>
-      <c r="B510" s="28">
+      <c r="B510" s="27">
         <f>COUNTA(B3:B500)</f>
         <v/>
       </c>
@@ -5388,7 +5201,7 @@
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
@@ -5403,7 +5216,7 @@
         </is>
       </c>
       <c r="B6" s="19" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
@@ -5418,7 +5231,7 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
@@ -5462,7 +5275,7 @@
           <t>TOTAL ACTIVOS</t>
         </is>
       </c>
-      <c r="B10" s="29">
+      <c r="B10" s="28">
         <f>SUM(B5:B9)</f>
         <v/>
       </c>
@@ -5530,7 +5343,7 @@
           <t>TOTAL PASIVOS</t>
         </is>
       </c>
-      <c r="B17" s="30">
+      <c r="B17" s="29">
         <f>SUM(B14:B16)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Fix repair dialog: replace empty Table with plain autofilter
Empty Table ref A2:J2 (header-only, no data rows) is invalid for
Excel — it quits the table and autofilter on repair. Replaced with
ws2.auto_filter.ref which works correctly on an empty sheet.

https://claude.ai/code/session_01EdLrBe1U3fRxvoA6PYaJVC
</commit_message>
<xml_diff>
--- a/sistema_financiero.xlsx
+++ b/sistema_financiero.xlsx
@@ -27,6 +27,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'GUIA DE USO'!$A$1:$J$42</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'DASHBOARD EJECUTIVO'!$A$1:$N$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'REGISTRO DE MOVIMIENTOS'!$A$2:$J$2</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'REGISTRO DE MOVIMIENTOS'!$A$1:$L$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'PRESUPUESTO MENSUAL'!$A$1:$H$38</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'CONTROL DE AHORRO'!$A$1:$H$16</definedName>
@@ -1514,25 +1515,6 @@
 </wsDr>
 </file>
 
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Movimientos" displayName="Movimientos" ref="A2:J2" headerRowCount="1">
-  <autoFilter ref="A2:J2"/>
-  <tableColumns count="10">
-    <tableColumn id="1" name="Fecha"/>
-    <tableColumn id="2" name="Mes"/>
-    <tableColumn id="3" name="Anio"/>
-    <tableColumn id="4" name="Tipo"/>
-    <tableColumn id="5" name="Categoria"/>
-    <tableColumn id="6" name="Subcategoria"/>
-    <tableColumn id="7" name="Descripcion"/>
-    <tableColumn id="8" name="Importe"/>
-    <tableColumn id="9" name="Metodo de Pago"/>
-    <tableColumn id="10" name="Comentarios"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -4145,6 +4127,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A2:J2"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
@@ -4161,9 +4144,6 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Fix ESTADO DEL PRESUPUESTO text cells: merge B2:E for visibility
https://claude.ai/code/session_01EdLrBe1U3fRxvoA6PYaJVC
</commit_message>
<xml_diff>
--- a/sistema_financiero.xlsx
+++ b/sistema_financiero.xlsx
@@ -4574,14 +4574,16 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A31:F31"/>
     <mergeCell ref="A6:F6"/>
+    <mergeCell ref="B33:E33"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A20:F20"/>
+    <mergeCell ref="B32:E32"/>
   </mergeCells>
   <conditionalFormatting sqref="C28">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">

</xml_diff>

<commit_message>
Implement Option C: fixed-amount investor distribution system
PRESUPUESTO MENSUAL:
- Replace percentage-based auto-distribution with fixed minimum amounts
- Bankroll: 100EUR fixed (gold editable cell, with comment)
- Ahorro: 100EUR fixed (gold editable cell, with comment)
- Caprichos: 20% of real surplus after fijos+BK+ahorro (not % of income)
- Add 'Ingreso disponible' row showing income minus fixed costs
- Add minimum income threshold alert: warns when income < fijos+BK+ahorro
- Conditional formatting on DISPONIBLE: green if >0, red if <=0

PROYECCIONES FUTURAS:
- Replace 'Tasa ahorro %' parameter with 'Ahorro fijo mensual'
- Replace 'Aportacion bankroll' with 'Bankroll fijo mensual'
- Projections now use fixed amounts x 12 x years (realistic)

https://claude.ai/code/session_01EdLrBe1U3fRxvoA6PYaJVC
</commit_message>
<xml_diff>
--- a/sistema_financiero.xlsx
+++ b/sistema_financiero.xlsx
@@ -29,7 +29,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="1">'DASHBOARD EJECUTIVO'!$A$1:$N$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'REGISTRO DE MOVIMIENTOS'!$A$2:$J$2</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'REGISTRO DE MOVIMIENTOS'!$A$1:$L$7</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'PRESUPUESTO MENSUAL'!$A$1:$H$38</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'PRESUPUESTO MENSUAL'!$A$1:$H$41</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'CONTROL DE AHORRO'!$A$1:$H$16</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'CONTROL DE BANKROLL'!$A$1:$G$14</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'DASHBOARD DE TRADING'!$A$1:$G$515</definedName>
@@ -268,7 +268,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -345,8 +345,8 @@
     <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="15">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="18">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="21">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="14">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -374,9 +374,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="9">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="21">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="14">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -419,6 +416,20 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="00DC3545"/>
         </patternFill>
       </fill>
@@ -434,20 +445,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="0028A745"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00C6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1322,6 +1319,21 @@
         <t>Cambia este valor cada mes. Todo el sistema se actualiza automaticamente.</t>
       </text>
     </comment>
+    <comment ref="B17" authorId="0" shapeId="0">
+      <text>
+        <t>Importe fijo minimo para bankroll. Aumentalo en meses buenos.</t>
+      </text>
+    </comment>
+    <comment ref="B18" authorId="0" shapeId="0">
+      <text>
+        <t>Importe fijo minimo para ahorro. Aumentalo en meses buenos.</t>
+      </text>
+    </comment>
+    <comment ref="B19" authorId="0" shapeId="0">
+      <text>
+        <t>Porcentaje del sobrante real (despues de fijos + bankroll + ahorro).</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -2516,14 +2528,14 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="E3:E10">
-    <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="3">
+    <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>0.75</formula>
     </cfRule>
     <cfRule type="cellIs" priority="2" operator="between" dxfId="5">
       <formula>0.5</formula>
       <formula>0.75</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="lessThan" dxfId="4">
+    <cfRule type="cellIs" priority="3" operator="lessThan" dxfId="1">
       <formula>0.5</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3275,41 +3287,41 @@
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Tasa de ahorro mensual %</t>
-        </is>
-      </c>
-      <c r="B5" s="36" t="n">
-        <v>0.1</v>
+          <t>Ahorro fijo mensual (editar)</t>
+        </is>
+      </c>
+      <c r="B5" s="23" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Beneficio medio mensual trading</t>
+          <t>Bankroll fijo mensual (editar)</t>
         </is>
       </c>
       <c r="B6" s="23" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Rentabilidad anual inversion %</t>
-        </is>
-      </c>
-      <c r="B7" s="36" t="n">
-        <v>0.05</v>
+          <t>Beneficio medio mensual trading</t>
+        </is>
+      </c>
+      <c r="B7" s="23" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Aportacion bankroll mensual</t>
-        </is>
-      </c>
-      <c r="B8" s="23" t="n">
-        <v>200</v>
+          <t>Rentabilidad anual inversion %</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="10">
@@ -3358,11 +3370,11 @@
         </is>
       </c>
       <c r="B12" s="19">
-        <f>$B$4*$B$5*12*1</f>
+        <f>$B$5*12*1</f>
         <v/>
       </c>
       <c r="C12" s="19">
-        <f>$B$8*12*1</f>
+        <f>$B$6*12*1</f>
         <v/>
       </c>
       <c r="D12" s="19">
@@ -3370,11 +3382,11 @@
         <v/>
       </c>
       <c r="E12" s="19">
-        <f>$B$6*12*1</f>
+        <f>$B$7*12*1</f>
         <v/>
       </c>
       <c r="F12" s="20">
-        <f>IFERROR($B$6/1575,0)</f>
+        <f>IFERROR($B$7/1575,0)</f>
         <v/>
       </c>
     </row>
@@ -3385,11 +3397,11 @@
         </is>
       </c>
       <c r="B13" s="17">
-        <f>$B$4*$B$5*12*2</f>
+        <f>$B$5*12*2</f>
         <v/>
       </c>
       <c r="C13" s="17">
-        <f>$B$8*12*2</f>
+        <f>$B$6*12*2</f>
         <v/>
       </c>
       <c r="D13" s="17">
@@ -3397,11 +3409,11 @@
         <v/>
       </c>
       <c r="E13" s="17">
-        <f>$B$6*12*2</f>
+        <f>$B$7*12*2</f>
         <v/>
       </c>
       <c r="F13" s="18">
-        <f>IFERROR($B$6/1575,0)</f>
+        <f>IFERROR($B$7/1575,0)</f>
         <v/>
       </c>
     </row>
@@ -3412,11 +3424,11 @@
         </is>
       </c>
       <c r="B14" s="19">
-        <f>$B$4*$B$5*12*3</f>
+        <f>$B$5*12*3</f>
         <v/>
       </c>
       <c r="C14" s="19">
-        <f>$B$8*12*3</f>
+        <f>$B$6*12*3</f>
         <v/>
       </c>
       <c r="D14" s="19">
@@ -3424,11 +3436,11 @@
         <v/>
       </c>
       <c r="E14" s="19">
-        <f>$B$6*12*3</f>
+        <f>$B$7*12*3</f>
         <v/>
       </c>
       <c r="F14" s="20">
-        <f>IFERROR($B$6/1575,0)</f>
+        <f>IFERROR($B$7/1575,0)</f>
         <v/>
       </c>
     </row>
@@ -3439,11 +3451,11 @@
         </is>
       </c>
       <c r="B15" s="17">
-        <f>$B$4*$B$5*12*4</f>
+        <f>$B$5*12*4</f>
         <v/>
       </c>
       <c r="C15" s="17">
-        <f>$B$8*12*4</f>
+        <f>$B$6*12*4</f>
         <v/>
       </c>
       <c r="D15" s="17">
@@ -3451,11 +3463,11 @@
         <v/>
       </c>
       <c r="E15" s="17">
-        <f>$B$6*12*4</f>
+        <f>$B$7*12*4</f>
         <v/>
       </c>
       <c r="F15" s="18">
-        <f>IFERROR($B$6/1575,0)</f>
+        <f>IFERROR($B$7/1575,0)</f>
         <v/>
       </c>
     </row>
@@ -3466,11 +3478,11 @@
         </is>
       </c>
       <c r="B16" s="19">
-        <f>$B$4*$B$5*12*5</f>
+        <f>$B$5*12*5</f>
         <v/>
       </c>
       <c r="C16" s="19">
-        <f>$B$8*12*5</f>
+        <f>$B$6*12*5</f>
         <v/>
       </c>
       <c r="D16" s="19">
@@ -3478,11 +3490,11 @@
         <v/>
       </c>
       <c r="E16" s="19">
-        <f>$B$6*12*5</f>
+        <f>$B$7*12*5</f>
         <v/>
       </c>
       <c r="F16" s="20">
-        <f>IFERROR($B$6/1575,0)</f>
+        <f>IFERROR($B$7/1575,0)</f>
         <v/>
       </c>
     </row>
@@ -3586,7 +3598,7 @@
           <t>Actualiza con % cumplimiento bankroll</t>
         </is>
       </c>
-      <c r="D6" s="37" t="n">
+      <c r="D6" s="36" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3626,7 +3638,7 @@
           <t>Actualiza con crecimiento patrimonio</t>
         </is>
       </c>
-      <c r="D8" s="37" t="n">
+      <c r="D8" s="36" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3656,7 +3668,7 @@
           <t>SCORE TOTAL DEL TRADER (sobre 100)</t>
         </is>
       </c>
-      <c r="D10" s="38">
+      <c r="D10" s="37">
         <f>ROUND(SUM(D5:D9),1)</f>
         <v/>
       </c>
@@ -4154,7 +4166,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -4337,7 +4349,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>DISTRIBUCION AUTOMATICA (% INGRESO)</t>
+          <t>DISTRIBUCION AUTOMATICA - SISTEMA INVERSOR (IMPORTES FIJOS)</t>
         </is>
       </c>
     </row>
@@ -4349,7 +4361,7 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>% Aplicado</t>
+          <t>Importe fijo/mes</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
@@ -4371,229 +4383,277 @@
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>Bankroll</t>
-        </is>
-      </c>
-      <c r="B16" s="26" t="n">
-        <v>0.1</v>
+          <t>Ingreso disponible (tras fijos)</t>
+        </is>
       </c>
       <c r="C16" s="17">
-        <f>$D$3*B16</f>
-        <v/>
-      </c>
-      <c r="D16" s="17">
-        <f>$D$3*B16*12</f>
+        <f>$D$3-C12</f>
         <v/>
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>10% para capital de trading</t>
+          <t>Base real = Ingreso - Gastos fijos</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Ahorro</t>
-        </is>
-      </c>
-      <c r="B17" s="15" t="n">
-        <v>0.1</v>
+          <t>Bankroll (inversion trading)</t>
+        </is>
+      </c>
+      <c r="B17" s="23" t="n">
+        <v>100</v>
       </c>
       <c r="C17" s="19">
-        <f>$D$3*B17</f>
+        <f>B17</f>
         <v/>
       </c>
       <c r="D17" s="19">
-        <f>$D$3*B17*12</f>
+        <f>B17*12</f>
         <v/>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>10% para fondo de ahorro</t>
+          <t>Fijo minimo garantizado cada mes</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Caprichos</t>
-        </is>
-      </c>
-      <c r="B18" s="26" t="n">
-        <v>0.05</v>
+          <t>Ahorro (fondo personal)</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="n">
+        <v>100</v>
       </c>
       <c r="C18" s="17">
-        <f>$D$3*B18</f>
+        <f>B18</f>
         <v/>
       </c>
       <c r="D18" s="17">
-        <f>$D$3*B18*12</f>
+        <f>B18*12</f>
         <v/>
       </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
-          <t>5% para gastos personales</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+          <t>Fijo minimo garantizado cada mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Caprichos y ocio (% del sobrante)</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C19" s="19">
+        <f>MAX(0,($D$3-C12-B17-B18)*B19)</f>
+        <v/>
+      </c>
+      <c r="D19" s="19">
+        <f>C19*12</f>
+        <v/>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>20% del sobrante real del mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>RESUMEN Y DISPONIBLE</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>Importe</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>Ingreso neto mensual</t>
         </is>
       </c>
-      <c r="C22" s="17">
+      <c r="C23" s="17">
         <f>$D$3</f>
         <v/>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>(-) Total gastos fijos</t>
         </is>
       </c>
-      <c r="C23" s="19">
+      <c r="C24" s="19">
         <f>-C12</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
-        <is>
-          <t>(-) Bankroll (10%)</t>
-        </is>
-      </c>
-      <c r="C24" s="17">
-        <f>-C16</f>
-        <v/>
-      </c>
-    </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>(-) Ahorro (10%)</t>
-        </is>
-      </c>
-      <c r="C25" s="19">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>(-) Bankroll (fijo)</t>
+        </is>
+      </c>
+      <c r="C25" s="17">
         <f>-C17</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>(-) Caprichos (5%)</t>
-        </is>
-      </c>
-      <c r="C26" s="17">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>(-) Ahorro (fijo)</t>
+        </is>
+      </c>
+      <c r="C26" s="19">
         <f>-C18</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>DISPONIBLE RESTANTE</t>
-        </is>
-      </c>
-      <c r="C27" s="21">
-        <f>SUM(C22:C26)</f>
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>(-) Caprichos (% sobrante)</t>
+        </is>
+      </c>
+      <c r="C27" s="17">
+        <f>-C19</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>% Gastado (fijos/ingreso)</t>
-        </is>
-      </c>
-      <c r="C28" s="22">
-        <f>C12/$D$3</f>
+          <t>DISPONIBLE RESTANTE (reserva flexible)</t>
+        </is>
+      </c>
+      <c r="C28" s="21">
+        <f>SUM(C23:C27)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Desviacion vs presupuesto</t>
-        </is>
-      </c>
-      <c r="C29" s="21">
-        <f>$D$3-C12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="1" t="inlineStr">
+          <t>% Gastado fijos / ingreso</t>
+        </is>
+      </c>
+      <c r="C29" s="22">
+        <f>C12/$D$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Total comprometido (fijos+BK+ahorro+cap)</t>
+        </is>
+      </c>
+      <c r="C30" s="21">
+        <f>C12+C17+C18+C19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
         <is>
           <t>ESTADO DEL PRESUPUESTO</t>
         </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="9" t="inlineStr">
-        <is>
-          <t>Progreso gastos fijos:</t>
-        </is>
-      </c>
-      <c r="B32" s="10">
-        <f>TEXT(C28,"0.0%")&amp;" del ingreso en gastos fijos"</f>
-        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
+          <t>Umbral minimo de ingreso:</t>
+        </is>
+      </c>
+      <c r="B33" s="10">
+        <f>TEXT(C12+B17+B18,"#,##0.00")&amp;" EUR (fijos + BK + ahorro)"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>Alerta de ingreso:</t>
+        </is>
+      </c>
+      <c r="B34" s="10">
+        <f>IF($D$3&gt;=(C12+B17+B18),"OK - Ingresos suficientes para cubrir todos los compromisos","ATENCION: Ingreso por debajo del umbral minimo - reduce BK o ahorro este mes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
           <t>Disponible restante:</t>
         </is>
       </c>
-      <c r="B33" s="10">
-        <f>TEXT(C27,"#,##0.00")&amp;" EUR disponibles este mes"</f>
+      <c r="B35" s="10">
+        <f>TEXT(C28,"#,##0.00")&amp;" EUR de reserva flexible este mes"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>Progreso gastos fijos:</t>
+        </is>
+      </c>
+      <c r="B36" s="10">
+        <f>TEXT(C29,"0.0%")&amp;" del ingreso en gastos fijos"</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="11">
+    <mergeCell ref="B35:E35"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A32:F32"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="B33:E33"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="B36:E36"/>
   </mergeCells>
   <conditionalFormatting sqref="C28">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="lessThanOrEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C29">
+    <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
+    <cfRule type="cellIs" priority="4" operator="between" dxfId="3">
       <formula>0.9</formula>
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="lessThanOrEqual" dxfId="2">
+    <cfRule type="cellIs" priority="5" operator="lessThanOrEqual" dxfId="4">
       <formula>0.9</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4998,10 +5058,10 @@
     <mergeCell ref="A502:E502"/>
   </mergeCells>
   <conditionalFormatting sqref="C3:C1000">
-    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="3">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="4">
+    <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5111,7 +5171,7 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <conditionalFormatting sqref="D3:D1000">
-    <cfRule type="expression" priority="1" dxfId="3">
+    <cfRule type="expression" priority="1" dxfId="0">
       <formula>D3="Cobrado"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="5">

</xml_diff>

<commit_message>
Fix dashboard refs + improve Registro usability
Dashboard Ejecutivo:
- Replace hardcoded 10% formulas with actual cell references to
  PRESUPUESTO MENSUAL (C rows for total_fixed, bankroll, ahorro,
  caprichos, disponible) — now shows 100EUR not 200EUR
- Update labels: Bankroll/Ahorro (fijo) instead of (10%)

Registro de Movimientos:
- Mes/Anio columns now auto-calculate from Fecha (rows 3-300)
  User only needs to enter date — month and year fill automatically
- Expand categories from 15 to 25 more specific options including:
  Peluqueria/Estetica, Farmacia/Salud, Gasolina, Parking,
  Cafeteria/Bar, Ropa/Calzado, Viajes/Vacaciones, etc.
- Type validation changed to allow_blank=True for easier entry

https://claude.ai/code/session_01EdLrBe1U3fRxvoA6PYaJVC
</commit_message>
<xml_diff>
--- a/sistema_financiero.xlsx
+++ b/sistema_financiero.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">'GUIA DE USO'!$A$1:$J$42</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'DASHBOARD EJECUTIVO'!$A$1:$N$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'REGISTRO DE MOVIMIENTOS'!$A$2:$J$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'REGISTRO DE MOVIMIENTOS'!$A$1:$L$7</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'REGISTRO DE MOVIMIENTOS'!$A$1:$L$305</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'PRESUPUESTO MENSUAL'!$A$1:$H$41</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'CONTROL DE AHORRO'!$A$1:$H$16</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'CONTROL DE BANKROLL'!$A$1:$G$14</definedName>
@@ -336,14 +336,14 @@
     <xf numFmtId="165" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="21">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="15">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="18">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="15">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="21">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="21">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -2239,7 +2239,7 @@
           <t>Capital actual fondo emergencia:</t>
         </is>
       </c>
-      <c r="B9" s="23" t="n">
+      <c r="B9" s="25" t="n">
         <v>500</v>
       </c>
     </row>
@@ -2679,7 +2679,7 @@
         <f>B505/'PRESUPUESTO MENSUAL'!$D$3</f>
         <v/>
       </c>
-      <c r="D505" s="25" t="inlineStr">
+      <c r="D505" s="23" t="inlineStr">
         <is>
           <t>5% limite</t>
         </is>
@@ -2727,7 +2727,7 @@
         <f>B507/'PRESUPUESTO MENSUAL'!$D$3</f>
         <v/>
       </c>
-      <c r="D507" s="25" t="inlineStr">
+      <c r="D507" s="23" t="inlineStr">
         <is>
           <t>5% limite</t>
         </is>
@@ -3280,7 +3280,7 @@
           <t>Ingreso medio mensual neto</t>
         </is>
       </c>
-      <c r="B4" s="23" t="n">
+      <c r="B4" s="25" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3290,7 +3290,7 @@
           <t>Ahorro fijo mensual (editar)</t>
         </is>
       </c>
-      <c r="B5" s="23" t="n">
+      <c r="B5" s="25" t="n">
         <v>100</v>
       </c>
     </row>
@@ -3300,7 +3300,7 @@
           <t>Bankroll fijo mensual (editar)</t>
         </is>
       </c>
-      <c r="B6" s="23" t="n">
+      <c r="B6" s="25" t="n">
         <v>100</v>
       </c>
     </row>
@@ -3310,7 +3310,7 @@
           <t>Beneficio medio mensual trading</t>
         </is>
       </c>
-      <c r="B7" s="23" t="n">
+      <c r="B7" s="25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3588,7 +3588,7 @@
           <t>Cumplimiento Bankroll</t>
         </is>
       </c>
-      <c r="B6" s="25" t="inlineStr">
+      <c r="B6" s="23" t="inlineStr">
         <is>
           <t>20 pts</t>
         </is>
@@ -3628,7 +3628,7 @@
           <t>Crecimiento Patrimonio</t>
         </is>
       </c>
-      <c r="B8" s="25" t="inlineStr">
+      <c r="B8" s="23" t="inlineStr">
         <is>
           <t>20 pts</t>
         </is>
@@ -3944,7 +3944,7 @@
         </is>
       </c>
       <c r="C16" s="19">
-        <f>1575</f>
+        <f>'PRESUPUESTO MENSUAL'!$C$12</f>
         <v/>
       </c>
       <c r="E16" s="20">
@@ -3955,11 +3955,11 @@
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>Bankroll (10%)</t>
+          <t>Bankroll (fijo)</t>
         </is>
       </c>
       <c r="C17" s="17">
-        <f>'PRESUPUESTO MENSUAL'!$D$3*0.1</f>
+        <f>'PRESUPUESTO MENSUAL'!$C$17</f>
         <v/>
       </c>
       <c r="E17" s="18">
@@ -3970,11 +3970,11 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Ahorro (10%)</t>
+          <t>Ahorro (fijo)</t>
         </is>
       </c>
       <c r="C18" s="19">
-        <f>'PRESUPUESTO MENSUAL'!$D$3*0.1</f>
+        <f>'PRESUPUESTO MENSUAL'!$C$18</f>
         <v/>
       </c>
       <c r="E18" s="20">
@@ -3985,11 +3985,11 @@
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>Caprichos (5%)</t>
+          <t>Caprichos</t>
         </is>
       </c>
       <c r="C19" s="17">
-        <f>'PRESUPUESTO MENSUAL'!$D$3*0.05</f>
+        <f>'PRESUPUESTO MENSUAL'!$C$19</f>
         <v/>
       </c>
       <c r="E19" s="18">
@@ -4004,7 +4004,7 @@
         </is>
       </c>
       <c r="C20" s="21">
-        <f>'PRESUPUESTO MENSUAL'!$D$3-1575-'PRESUPUESTO MENSUAL'!$D$3*0.25</f>
+        <f>'PRESUPUESTO MENSUAL'!$C$28</f>
         <v/>
       </c>
       <c r="E20" s="22">
@@ -4064,7 +4064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4094,12 +4094,12 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Mes</t>
+          <t>Mes (auto)</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Anio</t>
+          <t>Anio (auto)</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
@@ -4136,6 +4136,2986 @@
         <is>
           <t>Comentarios</t>
         </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="23">
+        <f>IF(A3="","",TEXT(A3,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C3" s="23">
+        <f>IF(A3="","",YEAR(A3))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="24">
+        <f>IF(A4="","",TEXT(A4,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C4" s="24">
+        <f>IF(A4="","",YEAR(A4))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="23">
+        <f>IF(A5="","",TEXT(A5,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C5" s="23">
+        <f>IF(A5="","",YEAR(A5))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="24">
+        <f>IF(A6="","",TEXT(A6,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C6" s="24">
+        <f>IF(A6="","",YEAR(A6))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="23">
+        <f>IF(A7="","",TEXT(A7,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C7" s="23">
+        <f>IF(A7="","",YEAR(A7))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="24">
+        <f>IF(A8="","",TEXT(A8,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C8" s="24">
+        <f>IF(A8="","",YEAR(A8))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="23">
+        <f>IF(A9="","",TEXT(A9,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C9" s="23">
+        <f>IF(A9="","",YEAR(A9))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="24">
+        <f>IF(A10="","",TEXT(A10,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C10" s="24">
+        <f>IF(A10="","",YEAR(A10))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="23">
+        <f>IF(A11="","",TEXT(A11,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C11" s="23">
+        <f>IF(A11="","",YEAR(A11))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="24">
+        <f>IF(A12="","",TEXT(A12,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C12" s="24">
+        <f>IF(A12="","",YEAR(A12))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="23">
+        <f>IF(A13="","",TEXT(A13,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C13" s="23">
+        <f>IF(A13="","",YEAR(A13))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="24">
+        <f>IF(A14="","",TEXT(A14,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C14" s="24">
+        <f>IF(A14="","",YEAR(A14))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="23">
+        <f>IF(A15="","",TEXT(A15,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C15" s="23">
+        <f>IF(A15="","",YEAR(A15))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="24">
+        <f>IF(A16="","",TEXT(A16,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C16" s="24">
+        <f>IF(A16="","",YEAR(A16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="23">
+        <f>IF(A17="","",TEXT(A17,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C17" s="23">
+        <f>IF(A17="","",YEAR(A17))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="24">
+        <f>IF(A18="","",TEXT(A18,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C18" s="24">
+        <f>IF(A18="","",YEAR(A18))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="23">
+        <f>IF(A19="","",TEXT(A19,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C19" s="23">
+        <f>IF(A19="","",YEAR(A19))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="24">
+        <f>IF(A20="","",TEXT(A20,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C20" s="24">
+        <f>IF(A20="","",YEAR(A20))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="23">
+        <f>IF(A21="","",TEXT(A21,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C21" s="23">
+        <f>IF(A21="","",YEAR(A21))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="24">
+        <f>IF(A22="","",TEXT(A22,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C22" s="24">
+        <f>IF(A22="","",YEAR(A22))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="23">
+        <f>IF(A23="","",TEXT(A23,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C23" s="23">
+        <f>IF(A23="","",YEAR(A23))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="24">
+        <f>IF(A24="","",TEXT(A24,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C24" s="24">
+        <f>IF(A24="","",YEAR(A24))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="23">
+        <f>IF(A25="","",TEXT(A25,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C25" s="23">
+        <f>IF(A25="","",YEAR(A25))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="24">
+        <f>IF(A26="","",TEXT(A26,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C26" s="24">
+        <f>IF(A26="","",YEAR(A26))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="23">
+        <f>IF(A27="","",TEXT(A27,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C27" s="23">
+        <f>IF(A27="","",YEAR(A27))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="24">
+        <f>IF(A28="","",TEXT(A28,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C28" s="24">
+        <f>IF(A28="","",YEAR(A28))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="23">
+        <f>IF(A29="","",TEXT(A29,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C29" s="23">
+        <f>IF(A29="","",YEAR(A29))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="24">
+        <f>IF(A30="","",TEXT(A30,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C30" s="24">
+        <f>IF(A30="","",YEAR(A30))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="23">
+        <f>IF(A31="","",TEXT(A31,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C31" s="23">
+        <f>IF(A31="","",YEAR(A31))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="24">
+        <f>IF(A32="","",TEXT(A32,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C32" s="24">
+        <f>IF(A32="","",YEAR(A32))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="23">
+        <f>IF(A33="","",TEXT(A33,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C33" s="23">
+        <f>IF(A33="","",YEAR(A33))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="24">
+        <f>IF(A34="","",TEXT(A34,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C34" s="24">
+        <f>IF(A34="","",YEAR(A34))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="23">
+        <f>IF(A35="","",TEXT(A35,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C35" s="23">
+        <f>IF(A35="","",YEAR(A35))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="24">
+        <f>IF(A36="","",TEXT(A36,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C36" s="24">
+        <f>IF(A36="","",YEAR(A36))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="23">
+        <f>IF(A37="","",TEXT(A37,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C37" s="23">
+        <f>IF(A37="","",YEAR(A37))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="24">
+        <f>IF(A38="","",TEXT(A38,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C38" s="24">
+        <f>IF(A38="","",YEAR(A38))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="23">
+        <f>IF(A39="","",TEXT(A39,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C39" s="23">
+        <f>IF(A39="","",YEAR(A39))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="24">
+        <f>IF(A40="","",TEXT(A40,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C40" s="24">
+        <f>IF(A40="","",YEAR(A40))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="23">
+        <f>IF(A41="","",TEXT(A41,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C41" s="23">
+        <f>IF(A41="","",YEAR(A41))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="24">
+        <f>IF(A42="","",TEXT(A42,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C42" s="24">
+        <f>IF(A42="","",YEAR(A42))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="23">
+        <f>IF(A43="","",TEXT(A43,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C43" s="23">
+        <f>IF(A43="","",YEAR(A43))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="24">
+        <f>IF(A44="","",TEXT(A44,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C44" s="24">
+        <f>IF(A44="","",YEAR(A44))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="23">
+        <f>IF(A45="","",TEXT(A45,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C45" s="23">
+        <f>IF(A45="","",YEAR(A45))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="24">
+        <f>IF(A46="","",TEXT(A46,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C46" s="24">
+        <f>IF(A46="","",YEAR(A46))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="23">
+        <f>IF(A47="","",TEXT(A47,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C47" s="23">
+        <f>IF(A47="","",YEAR(A47))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="24">
+        <f>IF(A48="","",TEXT(A48,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C48" s="24">
+        <f>IF(A48="","",YEAR(A48))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="23">
+        <f>IF(A49="","",TEXT(A49,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C49" s="23">
+        <f>IF(A49="","",YEAR(A49))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="24">
+        <f>IF(A50="","",TEXT(A50,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C50" s="24">
+        <f>IF(A50="","",YEAR(A50))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="23">
+        <f>IF(A51="","",TEXT(A51,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C51" s="23">
+        <f>IF(A51="","",YEAR(A51))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="24">
+        <f>IF(A52="","",TEXT(A52,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C52" s="24">
+        <f>IF(A52="","",YEAR(A52))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="23">
+        <f>IF(A53="","",TEXT(A53,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C53" s="23">
+        <f>IF(A53="","",YEAR(A53))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="24">
+        <f>IF(A54="","",TEXT(A54,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C54" s="24">
+        <f>IF(A54="","",YEAR(A54))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="23">
+        <f>IF(A55="","",TEXT(A55,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C55" s="23">
+        <f>IF(A55="","",YEAR(A55))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="24">
+        <f>IF(A56="","",TEXT(A56,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C56" s="24">
+        <f>IF(A56="","",YEAR(A56))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="23">
+        <f>IF(A57="","",TEXT(A57,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C57" s="23">
+        <f>IF(A57="","",YEAR(A57))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="24">
+        <f>IF(A58="","",TEXT(A58,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C58" s="24">
+        <f>IF(A58="","",YEAR(A58))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="23">
+        <f>IF(A59="","",TEXT(A59,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C59" s="23">
+        <f>IF(A59="","",YEAR(A59))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="24">
+        <f>IF(A60="","",TEXT(A60,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C60" s="24">
+        <f>IF(A60="","",YEAR(A60))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="23">
+        <f>IF(A61="","",TEXT(A61,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C61" s="23">
+        <f>IF(A61="","",YEAR(A61))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="24">
+        <f>IF(A62="","",TEXT(A62,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C62" s="24">
+        <f>IF(A62="","",YEAR(A62))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="23">
+        <f>IF(A63="","",TEXT(A63,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C63" s="23">
+        <f>IF(A63="","",YEAR(A63))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="24">
+        <f>IF(A64="","",TEXT(A64,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C64" s="24">
+        <f>IF(A64="","",YEAR(A64))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="23">
+        <f>IF(A65="","",TEXT(A65,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C65" s="23">
+        <f>IF(A65="","",YEAR(A65))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="24">
+        <f>IF(A66="","",TEXT(A66,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C66" s="24">
+        <f>IF(A66="","",YEAR(A66))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="23">
+        <f>IF(A67="","",TEXT(A67,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C67" s="23">
+        <f>IF(A67="","",YEAR(A67))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="24">
+        <f>IF(A68="","",TEXT(A68,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C68" s="24">
+        <f>IF(A68="","",YEAR(A68))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="23">
+        <f>IF(A69="","",TEXT(A69,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C69" s="23">
+        <f>IF(A69="","",YEAR(A69))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="24">
+        <f>IF(A70="","",TEXT(A70,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C70" s="24">
+        <f>IF(A70="","",YEAR(A70))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="23">
+        <f>IF(A71="","",TEXT(A71,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C71" s="23">
+        <f>IF(A71="","",YEAR(A71))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="24">
+        <f>IF(A72="","",TEXT(A72,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C72" s="24">
+        <f>IF(A72="","",YEAR(A72))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="23">
+        <f>IF(A73="","",TEXT(A73,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C73" s="23">
+        <f>IF(A73="","",YEAR(A73))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="24">
+        <f>IF(A74="","",TEXT(A74,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C74" s="24">
+        <f>IF(A74="","",YEAR(A74))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="23">
+        <f>IF(A75="","",TEXT(A75,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C75" s="23">
+        <f>IF(A75="","",YEAR(A75))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="24">
+        <f>IF(A76="","",TEXT(A76,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C76" s="24">
+        <f>IF(A76="","",YEAR(A76))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="23">
+        <f>IF(A77="","",TEXT(A77,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C77" s="23">
+        <f>IF(A77="","",YEAR(A77))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="24">
+        <f>IF(A78="","",TEXT(A78,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C78" s="24">
+        <f>IF(A78="","",YEAR(A78))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="23">
+        <f>IF(A79="","",TEXT(A79,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C79" s="23">
+        <f>IF(A79="","",YEAR(A79))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" s="24">
+        <f>IF(A80="","",TEXT(A80,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C80" s="24">
+        <f>IF(A80="","",YEAR(A80))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="23">
+        <f>IF(A81="","",TEXT(A81,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C81" s="23">
+        <f>IF(A81="","",YEAR(A81))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="24">
+        <f>IF(A82="","",TEXT(A82,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C82" s="24">
+        <f>IF(A82="","",YEAR(A82))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" s="23">
+        <f>IF(A83="","",TEXT(A83,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C83" s="23">
+        <f>IF(A83="","",YEAR(A83))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" s="24">
+        <f>IF(A84="","",TEXT(A84,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C84" s="24">
+        <f>IF(A84="","",YEAR(A84))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="23">
+        <f>IF(A85="","",TEXT(A85,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C85" s="23">
+        <f>IF(A85="","",YEAR(A85))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" s="24">
+        <f>IF(A86="","",TEXT(A86,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C86" s="24">
+        <f>IF(A86="","",YEAR(A86))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" s="23">
+        <f>IF(A87="","",TEXT(A87,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C87" s="23">
+        <f>IF(A87="","",YEAR(A87))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="24">
+        <f>IF(A88="","",TEXT(A88,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C88" s="24">
+        <f>IF(A88="","",YEAR(A88))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="23">
+        <f>IF(A89="","",TEXT(A89,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C89" s="23">
+        <f>IF(A89="","",YEAR(A89))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="B90" s="24">
+        <f>IF(A90="","",TEXT(A90,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C90" s="24">
+        <f>IF(A90="","",YEAR(A90))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" s="23">
+        <f>IF(A91="","",TEXT(A91,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C91" s="23">
+        <f>IF(A91="","",YEAR(A91))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="24">
+        <f>IF(A92="","",TEXT(A92,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C92" s="24">
+        <f>IF(A92="","",YEAR(A92))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="B93" s="23">
+        <f>IF(A93="","",TEXT(A93,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C93" s="23">
+        <f>IF(A93="","",YEAR(A93))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="B94" s="24">
+        <f>IF(A94="","",TEXT(A94,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C94" s="24">
+        <f>IF(A94="","",YEAR(A94))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="B95" s="23">
+        <f>IF(A95="","",TEXT(A95,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C95" s="23">
+        <f>IF(A95="","",YEAR(A95))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="B96" s="24">
+        <f>IF(A96="","",TEXT(A96,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C96" s="24">
+        <f>IF(A96="","",YEAR(A96))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="B97" s="23">
+        <f>IF(A97="","",TEXT(A97,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C97" s="23">
+        <f>IF(A97="","",YEAR(A97))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="B98" s="24">
+        <f>IF(A98="","",TEXT(A98,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C98" s="24">
+        <f>IF(A98="","",YEAR(A98))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="B99" s="23">
+        <f>IF(A99="","",TEXT(A99,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C99" s="23">
+        <f>IF(A99="","",YEAR(A99))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="B100" s="24">
+        <f>IF(A100="","",TEXT(A100,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C100" s="24">
+        <f>IF(A100="","",YEAR(A100))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="B101" s="23">
+        <f>IF(A101="","",TEXT(A101,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C101" s="23">
+        <f>IF(A101="","",YEAR(A101))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="B102" s="24">
+        <f>IF(A102="","",TEXT(A102,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C102" s="24">
+        <f>IF(A102="","",YEAR(A102))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="B103" s="23">
+        <f>IF(A103="","",TEXT(A103,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C103" s="23">
+        <f>IF(A103="","",YEAR(A103))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="B104" s="24">
+        <f>IF(A104="","",TEXT(A104,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C104" s="24">
+        <f>IF(A104="","",YEAR(A104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="B105" s="23">
+        <f>IF(A105="","",TEXT(A105,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C105" s="23">
+        <f>IF(A105="","",YEAR(A105))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="B106" s="24">
+        <f>IF(A106="","",TEXT(A106,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C106" s="24">
+        <f>IF(A106="","",YEAR(A106))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="B107" s="23">
+        <f>IF(A107="","",TEXT(A107,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C107" s="23">
+        <f>IF(A107="","",YEAR(A107))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="B108" s="24">
+        <f>IF(A108="","",TEXT(A108,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C108" s="24">
+        <f>IF(A108="","",YEAR(A108))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="B109" s="23">
+        <f>IF(A109="","",TEXT(A109,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C109" s="23">
+        <f>IF(A109="","",YEAR(A109))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="B110" s="24">
+        <f>IF(A110="","",TEXT(A110,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C110" s="24">
+        <f>IF(A110="","",YEAR(A110))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="B111" s="23">
+        <f>IF(A111="","",TEXT(A111,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C111" s="23">
+        <f>IF(A111="","",YEAR(A111))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="B112" s="24">
+        <f>IF(A112="","",TEXT(A112,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C112" s="24">
+        <f>IF(A112="","",YEAR(A112))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" s="23">
+        <f>IF(A113="","",TEXT(A113,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C113" s="23">
+        <f>IF(A113="","",YEAR(A113))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" s="24">
+        <f>IF(A114="","",TEXT(A114,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C114" s="24">
+        <f>IF(A114="","",YEAR(A114))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" s="23">
+        <f>IF(A115="","",TEXT(A115,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C115" s="23">
+        <f>IF(A115="","",YEAR(A115))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116">
+      <c r="B116" s="24">
+        <f>IF(A116="","",TEXT(A116,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C116" s="24">
+        <f>IF(A116="","",YEAR(A116))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="B117" s="23">
+        <f>IF(A117="","",TEXT(A117,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C117" s="23">
+        <f>IF(A117="","",YEAR(A117))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="B118" s="24">
+        <f>IF(A118="","",TEXT(A118,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C118" s="24">
+        <f>IF(A118="","",YEAR(A118))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="B119" s="23">
+        <f>IF(A119="","",TEXT(A119,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C119" s="23">
+        <f>IF(A119="","",YEAR(A119))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="B120" s="24">
+        <f>IF(A120="","",TEXT(A120,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C120" s="24">
+        <f>IF(A120="","",YEAR(A120))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="B121" s="23">
+        <f>IF(A121="","",TEXT(A121,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C121" s="23">
+        <f>IF(A121="","",YEAR(A121))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="122">
+      <c r="B122" s="24">
+        <f>IF(A122="","",TEXT(A122,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C122" s="24">
+        <f>IF(A122="","",YEAR(A122))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="123">
+      <c r="B123" s="23">
+        <f>IF(A123="","",TEXT(A123,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C123" s="23">
+        <f>IF(A123="","",YEAR(A123))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="124">
+      <c r="B124" s="24">
+        <f>IF(A124="","",TEXT(A124,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C124" s="24">
+        <f>IF(A124="","",YEAR(A124))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="125">
+      <c r="B125" s="23">
+        <f>IF(A125="","",TEXT(A125,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C125" s="23">
+        <f>IF(A125="","",YEAR(A125))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="126">
+      <c r="B126" s="24">
+        <f>IF(A126="","",TEXT(A126,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C126" s="24">
+        <f>IF(A126="","",YEAR(A126))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="127">
+      <c r="B127" s="23">
+        <f>IF(A127="","",TEXT(A127,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C127" s="23">
+        <f>IF(A127="","",YEAR(A127))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="128">
+      <c r="B128" s="24">
+        <f>IF(A128="","",TEXT(A128,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C128" s="24">
+        <f>IF(A128="","",YEAR(A128))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="129">
+      <c r="B129" s="23">
+        <f>IF(A129="","",TEXT(A129,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C129" s="23">
+        <f>IF(A129="","",YEAR(A129))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="130">
+      <c r="B130" s="24">
+        <f>IF(A130="","",TEXT(A130,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C130" s="24">
+        <f>IF(A130="","",YEAR(A130))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="B131" s="23">
+        <f>IF(A131="","",TEXT(A131,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C131" s="23">
+        <f>IF(A131="","",YEAR(A131))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="132">
+      <c r="B132" s="24">
+        <f>IF(A132="","",TEXT(A132,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C132" s="24">
+        <f>IF(A132="","",YEAR(A132))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="133">
+      <c r="B133" s="23">
+        <f>IF(A133="","",TEXT(A133,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C133" s="23">
+        <f>IF(A133="","",YEAR(A133))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="134">
+      <c r="B134" s="24">
+        <f>IF(A134="","",TEXT(A134,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C134" s="24">
+        <f>IF(A134="","",YEAR(A134))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="135">
+      <c r="B135" s="23">
+        <f>IF(A135="","",TEXT(A135,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C135" s="23">
+        <f>IF(A135="","",YEAR(A135))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="136">
+      <c r="B136" s="24">
+        <f>IF(A136="","",TEXT(A136,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C136" s="24">
+        <f>IF(A136="","",YEAR(A136))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="137">
+      <c r="B137" s="23">
+        <f>IF(A137="","",TEXT(A137,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C137" s="23">
+        <f>IF(A137="","",YEAR(A137))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="138">
+      <c r="B138" s="24">
+        <f>IF(A138="","",TEXT(A138,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C138" s="24">
+        <f>IF(A138="","",YEAR(A138))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="139">
+      <c r="B139" s="23">
+        <f>IF(A139="","",TEXT(A139,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C139" s="23">
+        <f>IF(A139="","",YEAR(A139))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="140">
+      <c r="B140" s="24">
+        <f>IF(A140="","",TEXT(A140,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C140" s="24">
+        <f>IF(A140="","",YEAR(A140))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="141">
+      <c r="B141" s="23">
+        <f>IF(A141="","",TEXT(A141,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C141" s="23">
+        <f>IF(A141="","",YEAR(A141))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="142">
+      <c r="B142" s="24">
+        <f>IF(A142="","",TEXT(A142,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C142" s="24">
+        <f>IF(A142="","",YEAR(A142))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="143">
+      <c r="B143" s="23">
+        <f>IF(A143="","",TEXT(A143,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C143" s="23">
+        <f>IF(A143="","",YEAR(A143))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="144">
+      <c r="B144" s="24">
+        <f>IF(A144="","",TEXT(A144,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C144" s="24">
+        <f>IF(A144="","",YEAR(A144))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="145">
+      <c r="B145" s="23">
+        <f>IF(A145="","",TEXT(A145,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C145" s="23">
+        <f>IF(A145="","",YEAR(A145))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="146">
+      <c r="B146" s="24">
+        <f>IF(A146="","",TEXT(A146,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C146" s="24">
+        <f>IF(A146="","",YEAR(A146))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="147">
+      <c r="B147" s="23">
+        <f>IF(A147="","",TEXT(A147,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C147" s="23">
+        <f>IF(A147="","",YEAR(A147))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="148">
+      <c r="B148" s="24">
+        <f>IF(A148="","",TEXT(A148,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C148" s="24">
+        <f>IF(A148="","",YEAR(A148))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="149">
+      <c r="B149" s="23">
+        <f>IF(A149="","",TEXT(A149,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C149" s="23">
+        <f>IF(A149="","",YEAR(A149))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="150">
+      <c r="B150" s="24">
+        <f>IF(A150="","",TEXT(A150,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C150" s="24">
+        <f>IF(A150="","",YEAR(A150))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="151">
+      <c r="B151" s="23">
+        <f>IF(A151="","",TEXT(A151,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C151" s="23">
+        <f>IF(A151="","",YEAR(A151))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="152">
+      <c r="B152" s="24">
+        <f>IF(A152="","",TEXT(A152,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C152" s="24">
+        <f>IF(A152="","",YEAR(A152))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="153">
+      <c r="B153" s="23">
+        <f>IF(A153="","",TEXT(A153,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C153" s="23">
+        <f>IF(A153="","",YEAR(A153))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="154">
+      <c r="B154" s="24">
+        <f>IF(A154="","",TEXT(A154,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C154" s="24">
+        <f>IF(A154="","",YEAR(A154))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="155">
+      <c r="B155" s="23">
+        <f>IF(A155="","",TEXT(A155,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C155" s="23">
+        <f>IF(A155="","",YEAR(A155))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="156">
+      <c r="B156" s="24">
+        <f>IF(A156="","",TEXT(A156,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C156" s="24">
+        <f>IF(A156="","",YEAR(A156))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="157">
+      <c r="B157" s="23">
+        <f>IF(A157="","",TEXT(A157,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C157" s="23">
+        <f>IF(A157="","",YEAR(A157))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="158">
+      <c r="B158" s="24">
+        <f>IF(A158="","",TEXT(A158,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C158" s="24">
+        <f>IF(A158="","",YEAR(A158))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="159">
+      <c r="B159" s="23">
+        <f>IF(A159="","",TEXT(A159,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C159" s="23">
+        <f>IF(A159="","",YEAR(A159))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="160">
+      <c r="B160" s="24">
+        <f>IF(A160="","",TEXT(A160,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C160" s="24">
+        <f>IF(A160="","",YEAR(A160))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="161">
+      <c r="B161" s="23">
+        <f>IF(A161="","",TEXT(A161,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C161" s="23">
+        <f>IF(A161="","",YEAR(A161))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="162">
+      <c r="B162" s="24">
+        <f>IF(A162="","",TEXT(A162,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C162" s="24">
+        <f>IF(A162="","",YEAR(A162))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="163">
+      <c r="B163" s="23">
+        <f>IF(A163="","",TEXT(A163,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C163" s="23">
+        <f>IF(A163="","",YEAR(A163))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="164">
+      <c r="B164" s="24">
+        <f>IF(A164="","",TEXT(A164,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C164" s="24">
+        <f>IF(A164="","",YEAR(A164))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="165">
+      <c r="B165" s="23">
+        <f>IF(A165="","",TEXT(A165,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C165" s="23">
+        <f>IF(A165="","",YEAR(A165))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="166">
+      <c r="B166" s="24">
+        <f>IF(A166="","",TEXT(A166,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C166" s="24">
+        <f>IF(A166="","",YEAR(A166))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="167">
+      <c r="B167" s="23">
+        <f>IF(A167="","",TEXT(A167,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C167" s="23">
+        <f>IF(A167="","",YEAR(A167))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="168">
+      <c r="B168" s="24">
+        <f>IF(A168="","",TEXT(A168,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C168" s="24">
+        <f>IF(A168="","",YEAR(A168))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="169">
+      <c r="B169" s="23">
+        <f>IF(A169="","",TEXT(A169,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C169" s="23">
+        <f>IF(A169="","",YEAR(A169))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="170">
+      <c r="B170" s="24">
+        <f>IF(A170="","",TEXT(A170,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C170" s="24">
+        <f>IF(A170="","",YEAR(A170))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="171">
+      <c r="B171" s="23">
+        <f>IF(A171="","",TEXT(A171,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C171" s="23">
+        <f>IF(A171="","",YEAR(A171))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="172">
+      <c r="B172" s="24">
+        <f>IF(A172="","",TEXT(A172,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C172" s="24">
+        <f>IF(A172="","",YEAR(A172))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="173">
+      <c r="B173" s="23">
+        <f>IF(A173="","",TEXT(A173,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C173" s="23">
+        <f>IF(A173="","",YEAR(A173))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="174">
+      <c r="B174" s="24">
+        <f>IF(A174="","",TEXT(A174,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C174" s="24">
+        <f>IF(A174="","",YEAR(A174))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="175">
+      <c r="B175" s="23">
+        <f>IF(A175="","",TEXT(A175,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C175" s="23">
+        <f>IF(A175="","",YEAR(A175))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="176">
+      <c r="B176" s="24">
+        <f>IF(A176="","",TEXT(A176,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C176" s="24">
+        <f>IF(A176="","",YEAR(A176))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="177">
+      <c r="B177" s="23">
+        <f>IF(A177="","",TEXT(A177,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C177" s="23">
+        <f>IF(A177="","",YEAR(A177))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="178">
+      <c r="B178" s="24">
+        <f>IF(A178="","",TEXT(A178,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C178" s="24">
+        <f>IF(A178="","",YEAR(A178))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="179">
+      <c r="B179" s="23">
+        <f>IF(A179="","",TEXT(A179,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C179" s="23">
+        <f>IF(A179="","",YEAR(A179))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="180">
+      <c r="B180" s="24">
+        <f>IF(A180="","",TEXT(A180,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C180" s="24">
+        <f>IF(A180="","",YEAR(A180))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="181">
+      <c r="B181" s="23">
+        <f>IF(A181="","",TEXT(A181,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C181" s="23">
+        <f>IF(A181="","",YEAR(A181))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="182">
+      <c r="B182" s="24">
+        <f>IF(A182="","",TEXT(A182,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C182" s="24">
+        <f>IF(A182="","",YEAR(A182))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="183">
+      <c r="B183" s="23">
+        <f>IF(A183="","",TEXT(A183,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C183" s="23">
+        <f>IF(A183="","",YEAR(A183))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="B184" s="24">
+        <f>IF(A184="","",TEXT(A184,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C184" s="24">
+        <f>IF(A184="","",YEAR(A184))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="B185" s="23">
+        <f>IF(A185="","",TEXT(A185,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C185" s="23">
+        <f>IF(A185="","",YEAR(A185))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="B186" s="24">
+        <f>IF(A186="","",TEXT(A186,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C186" s="24">
+        <f>IF(A186="","",YEAR(A186))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="B187" s="23">
+        <f>IF(A187="","",TEXT(A187,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C187" s="23">
+        <f>IF(A187="","",YEAR(A187))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="B188" s="24">
+        <f>IF(A188="","",TEXT(A188,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C188" s="24">
+        <f>IF(A188="","",YEAR(A188))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="B189" s="23">
+        <f>IF(A189="","",TEXT(A189,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C189" s="23">
+        <f>IF(A189="","",YEAR(A189))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="B190" s="24">
+        <f>IF(A190="","",TEXT(A190,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C190" s="24">
+        <f>IF(A190="","",YEAR(A190))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="B191" s="23">
+        <f>IF(A191="","",TEXT(A191,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C191" s="23">
+        <f>IF(A191="","",YEAR(A191))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="B192" s="24">
+        <f>IF(A192="","",TEXT(A192,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C192" s="24">
+        <f>IF(A192="","",YEAR(A192))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="B193" s="23">
+        <f>IF(A193="","",TEXT(A193,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C193" s="23">
+        <f>IF(A193="","",YEAR(A193))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="194">
+      <c r="B194" s="24">
+        <f>IF(A194="","",TEXT(A194,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C194" s="24">
+        <f>IF(A194="","",YEAR(A194))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="B195" s="23">
+        <f>IF(A195="","",TEXT(A195,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C195" s="23">
+        <f>IF(A195="","",YEAR(A195))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="B196" s="24">
+        <f>IF(A196="","",TEXT(A196,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C196" s="24">
+        <f>IF(A196="","",YEAR(A196))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="B197" s="23">
+        <f>IF(A197="","",TEXT(A197,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C197" s="23">
+        <f>IF(A197="","",YEAR(A197))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="B198" s="24">
+        <f>IF(A198="","",TEXT(A198,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C198" s="24">
+        <f>IF(A198="","",YEAR(A198))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="199">
+      <c r="B199" s="23">
+        <f>IF(A199="","",TEXT(A199,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C199" s="23">
+        <f>IF(A199="","",YEAR(A199))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="200">
+      <c r="B200" s="24">
+        <f>IF(A200="","",TEXT(A200,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C200" s="24">
+        <f>IF(A200="","",YEAR(A200))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="201">
+      <c r="B201" s="23">
+        <f>IF(A201="","",TEXT(A201,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C201" s="23">
+        <f>IF(A201="","",YEAR(A201))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="202">
+      <c r="B202" s="24">
+        <f>IF(A202="","",TEXT(A202,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C202" s="24">
+        <f>IF(A202="","",YEAR(A202))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="203">
+      <c r="B203" s="23">
+        <f>IF(A203="","",TEXT(A203,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C203" s="23">
+        <f>IF(A203="","",YEAR(A203))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="204">
+      <c r="B204" s="24">
+        <f>IF(A204="","",TEXT(A204,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C204" s="24">
+        <f>IF(A204="","",YEAR(A204))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="205">
+      <c r="B205" s="23">
+        <f>IF(A205="","",TEXT(A205,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C205" s="23">
+        <f>IF(A205="","",YEAR(A205))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="206">
+      <c r="B206" s="24">
+        <f>IF(A206="","",TEXT(A206,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C206" s="24">
+        <f>IF(A206="","",YEAR(A206))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="207">
+      <c r="B207" s="23">
+        <f>IF(A207="","",TEXT(A207,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C207" s="23">
+        <f>IF(A207="","",YEAR(A207))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="208">
+      <c r="B208" s="24">
+        <f>IF(A208="","",TEXT(A208,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C208" s="24">
+        <f>IF(A208="","",YEAR(A208))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="209">
+      <c r="B209" s="23">
+        <f>IF(A209="","",TEXT(A209,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C209" s="23">
+        <f>IF(A209="","",YEAR(A209))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="210">
+      <c r="B210" s="24">
+        <f>IF(A210="","",TEXT(A210,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C210" s="24">
+        <f>IF(A210="","",YEAR(A210))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="211">
+      <c r="B211" s="23">
+        <f>IF(A211="","",TEXT(A211,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C211" s="23">
+        <f>IF(A211="","",YEAR(A211))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="212">
+      <c r="B212" s="24">
+        <f>IF(A212="","",TEXT(A212,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C212" s="24">
+        <f>IF(A212="","",YEAR(A212))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="213">
+      <c r="B213" s="23">
+        <f>IF(A213="","",TEXT(A213,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C213" s="23">
+        <f>IF(A213="","",YEAR(A213))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="214">
+      <c r="B214" s="24">
+        <f>IF(A214="","",TEXT(A214,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C214" s="24">
+        <f>IF(A214="","",YEAR(A214))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="215">
+      <c r="B215" s="23">
+        <f>IF(A215="","",TEXT(A215,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C215" s="23">
+        <f>IF(A215="","",YEAR(A215))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="216">
+      <c r="B216" s="24">
+        <f>IF(A216="","",TEXT(A216,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C216" s="24">
+        <f>IF(A216="","",YEAR(A216))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="217">
+      <c r="B217" s="23">
+        <f>IF(A217="","",TEXT(A217,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C217" s="23">
+        <f>IF(A217="","",YEAR(A217))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="218">
+      <c r="B218" s="24">
+        <f>IF(A218="","",TEXT(A218,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C218" s="24">
+        <f>IF(A218="","",YEAR(A218))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="219">
+      <c r="B219" s="23">
+        <f>IF(A219="","",TEXT(A219,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C219" s="23">
+        <f>IF(A219="","",YEAR(A219))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="220">
+      <c r="B220" s="24">
+        <f>IF(A220="","",TEXT(A220,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C220" s="24">
+        <f>IF(A220="","",YEAR(A220))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="221">
+      <c r="B221" s="23">
+        <f>IF(A221="","",TEXT(A221,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C221" s="23">
+        <f>IF(A221="","",YEAR(A221))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="222">
+      <c r="B222" s="24">
+        <f>IF(A222="","",TEXT(A222,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C222" s="24">
+        <f>IF(A222="","",YEAR(A222))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="223">
+      <c r="B223" s="23">
+        <f>IF(A223="","",TEXT(A223,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C223" s="23">
+        <f>IF(A223="","",YEAR(A223))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="224">
+      <c r="B224" s="24">
+        <f>IF(A224="","",TEXT(A224,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C224" s="24">
+        <f>IF(A224="","",YEAR(A224))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="225">
+      <c r="B225" s="23">
+        <f>IF(A225="","",TEXT(A225,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C225" s="23">
+        <f>IF(A225="","",YEAR(A225))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="226">
+      <c r="B226" s="24">
+        <f>IF(A226="","",TEXT(A226,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C226" s="24">
+        <f>IF(A226="","",YEAR(A226))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="227">
+      <c r="B227" s="23">
+        <f>IF(A227="","",TEXT(A227,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C227" s="23">
+        <f>IF(A227="","",YEAR(A227))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="228">
+      <c r="B228" s="24">
+        <f>IF(A228="","",TEXT(A228,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C228" s="24">
+        <f>IF(A228="","",YEAR(A228))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="229">
+      <c r="B229" s="23">
+        <f>IF(A229="","",TEXT(A229,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C229" s="23">
+        <f>IF(A229="","",YEAR(A229))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="230">
+      <c r="B230" s="24">
+        <f>IF(A230="","",TEXT(A230,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C230" s="24">
+        <f>IF(A230="","",YEAR(A230))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="231">
+      <c r="B231" s="23">
+        <f>IF(A231="","",TEXT(A231,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C231" s="23">
+        <f>IF(A231="","",YEAR(A231))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="232">
+      <c r="B232" s="24">
+        <f>IF(A232="","",TEXT(A232,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C232" s="24">
+        <f>IF(A232="","",YEAR(A232))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="233">
+      <c r="B233" s="23">
+        <f>IF(A233="","",TEXT(A233,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C233" s="23">
+        <f>IF(A233="","",YEAR(A233))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="234">
+      <c r="B234" s="24">
+        <f>IF(A234="","",TEXT(A234,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C234" s="24">
+        <f>IF(A234="","",YEAR(A234))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="235">
+      <c r="B235" s="23">
+        <f>IF(A235="","",TEXT(A235,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C235" s="23">
+        <f>IF(A235="","",YEAR(A235))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="236">
+      <c r="B236" s="24">
+        <f>IF(A236="","",TEXT(A236,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C236" s="24">
+        <f>IF(A236="","",YEAR(A236))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="237">
+      <c r="B237" s="23">
+        <f>IF(A237="","",TEXT(A237,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C237" s="23">
+        <f>IF(A237="","",YEAR(A237))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="238">
+      <c r="B238" s="24">
+        <f>IF(A238="","",TEXT(A238,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C238" s="24">
+        <f>IF(A238="","",YEAR(A238))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="239">
+      <c r="B239" s="23">
+        <f>IF(A239="","",TEXT(A239,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C239" s="23">
+        <f>IF(A239="","",YEAR(A239))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="240">
+      <c r="B240" s="24">
+        <f>IF(A240="","",TEXT(A240,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C240" s="24">
+        <f>IF(A240="","",YEAR(A240))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="241">
+      <c r="B241" s="23">
+        <f>IF(A241="","",TEXT(A241,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C241" s="23">
+        <f>IF(A241="","",YEAR(A241))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="242">
+      <c r="B242" s="24">
+        <f>IF(A242="","",TEXT(A242,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C242" s="24">
+        <f>IF(A242="","",YEAR(A242))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="243">
+      <c r="B243" s="23">
+        <f>IF(A243="","",TEXT(A243,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C243" s="23">
+        <f>IF(A243="","",YEAR(A243))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="244">
+      <c r="B244" s="24">
+        <f>IF(A244="","",TEXT(A244,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C244" s="24">
+        <f>IF(A244="","",YEAR(A244))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="245">
+      <c r="B245" s="23">
+        <f>IF(A245="","",TEXT(A245,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C245" s="23">
+        <f>IF(A245="","",YEAR(A245))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="246">
+      <c r="B246" s="24">
+        <f>IF(A246="","",TEXT(A246,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C246" s="24">
+        <f>IF(A246="","",YEAR(A246))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="247">
+      <c r="B247" s="23">
+        <f>IF(A247="","",TEXT(A247,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C247" s="23">
+        <f>IF(A247="","",YEAR(A247))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="248">
+      <c r="B248" s="24">
+        <f>IF(A248="","",TEXT(A248,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C248" s="24">
+        <f>IF(A248="","",YEAR(A248))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="249">
+      <c r="B249" s="23">
+        <f>IF(A249="","",TEXT(A249,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C249" s="23">
+        <f>IF(A249="","",YEAR(A249))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="250">
+      <c r="B250" s="24">
+        <f>IF(A250="","",TEXT(A250,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C250" s="24">
+        <f>IF(A250="","",YEAR(A250))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="251">
+      <c r="B251" s="23">
+        <f>IF(A251="","",TEXT(A251,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C251" s="23">
+        <f>IF(A251="","",YEAR(A251))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="252">
+      <c r="B252" s="24">
+        <f>IF(A252="","",TEXT(A252,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C252" s="24">
+        <f>IF(A252="","",YEAR(A252))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="253">
+      <c r="B253" s="23">
+        <f>IF(A253="","",TEXT(A253,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C253" s="23">
+        <f>IF(A253="","",YEAR(A253))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="254">
+      <c r="B254" s="24">
+        <f>IF(A254="","",TEXT(A254,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C254" s="24">
+        <f>IF(A254="","",YEAR(A254))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="255">
+      <c r="B255" s="23">
+        <f>IF(A255="","",TEXT(A255,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C255" s="23">
+        <f>IF(A255="","",YEAR(A255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="256">
+      <c r="B256" s="24">
+        <f>IF(A256="","",TEXT(A256,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C256" s="24">
+        <f>IF(A256="","",YEAR(A256))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="257">
+      <c r="B257" s="23">
+        <f>IF(A257="","",TEXT(A257,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C257" s="23">
+        <f>IF(A257="","",YEAR(A257))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="258">
+      <c r="B258" s="24">
+        <f>IF(A258="","",TEXT(A258,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C258" s="24">
+        <f>IF(A258="","",YEAR(A258))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="259">
+      <c r="B259" s="23">
+        <f>IF(A259="","",TEXT(A259,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C259" s="23">
+        <f>IF(A259="","",YEAR(A259))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="260">
+      <c r="B260" s="24">
+        <f>IF(A260="","",TEXT(A260,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C260" s="24">
+        <f>IF(A260="","",YEAR(A260))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="261">
+      <c r="B261" s="23">
+        <f>IF(A261="","",TEXT(A261,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C261" s="23">
+        <f>IF(A261="","",YEAR(A261))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="262">
+      <c r="B262" s="24">
+        <f>IF(A262="","",TEXT(A262,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C262" s="24">
+        <f>IF(A262="","",YEAR(A262))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="263">
+      <c r="B263" s="23">
+        <f>IF(A263="","",TEXT(A263,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C263" s="23">
+        <f>IF(A263="","",YEAR(A263))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="264">
+      <c r="B264" s="24">
+        <f>IF(A264="","",TEXT(A264,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C264" s="24">
+        <f>IF(A264="","",YEAR(A264))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="265">
+      <c r="B265" s="23">
+        <f>IF(A265="","",TEXT(A265,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C265" s="23">
+        <f>IF(A265="","",YEAR(A265))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="266">
+      <c r="B266" s="24">
+        <f>IF(A266="","",TEXT(A266,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C266" s="24">
+        <f>IF(A266="","",YEAR(A266))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="267">
+      <c r="B267" s="23">
+        <f>IF(A267="","",TEXT(A267,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C267" s="23">
+        <f>IF(A267="","",YEAR(A267))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="268">
+      <c r="B268" s="24">
+        <f>IF(A268="","",TEXT(A268,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C268" s="24">
+        <f>IF(A268="","",YEAR(A268))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="269">
+      <c r="B269" s="23">
+        <f>IF(A269="","",TEXT(A269,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C269" s="23">
+        <f>IF(A269="","",YEAR(A269))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="270">
+      <c r="B270" s="24">
+        <f>IF(A270="","",TEXT(A270,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C270" s="24">
+        <f>IF(A270="","",YEAR(A270))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="271">
+      <c r="B271" s="23">
+        <f>IF(A271="","",TEXT(A271,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C271" s="23">
+        <f>IF(A271="","",YEAR(A271))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="272">
+      <c r="B272" s="24">
+        <f>IF(A272="","",TEXT(A272,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C272" s="24">
+        <f>IF(A272="","",YEAR(A272))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="273">
+      <c r="B273" s="23">
+        <f>IF(A273="","",TEXT(A273,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C273" s="23">
+        <f>IF(A273="","",YEAR(A273))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="274">
+      <c r="B274" s="24">
+        <f>IF(A274="","",TEXT(A274,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C274" s="24">
+        <f>IF(A274="","",YEAR(A274))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="275">
+      <c r="B275" s="23">
+        <f>IF(A275="","",TEXT(A275,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C275" s="23">
+        <f>IF(A275="","",YEAR(A275))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="276">
+      <c r="B276" s="24">
+        <f>IF(A276="","",TEXT(A276,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C276" s="24">
+        <f>IF(A276="","",YEAR(A276))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="277">
+      <c r="B277" s="23">
+        <f>IF(A277="","",TEXT(A277,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C277" s="23">
+        <f>IF(A277="","",YEAR(A277))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="278">
+      <c r="B278" s="24">
+        <f>IF(A278="","",TEXT(A278,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C278" s="24">
+        <f>IF(A278="","",YEAR(A278))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="279">
+      <c r="B279" s="23">
+        <f>IF(A279="","",TEXT(A279,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C279" s="23">
+        <f>IF(A279="","",YEAR(A279))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="280">
+      <c r="B280" s="24">
+        <f>IF(A280="","",TEXT(A280,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C280" s="24">
+        <f>IF(A280="","",YEAR(A280))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="281">
+      <c r="B281" s="23">
+        <f>IF(A281="","",TEXT(A281,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C281" s="23">
+        <f>IF(A281="","",YEAR(A281))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="282">
+      <c r="B282" s="24">
+        <f>IF(A282="","",TEXT(A282,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C282" s="24">
+        <f>IF(A282="","",YEAR(A282))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="283">
+      <c r="B283" s="23">
+        <f>IF(A283="","",TEXT(A283,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C283" s="23">
+        <f>IF(A283="","",YEAR(A283))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="284">
+      <c r="B284" s="24">
+        <f>IF(A284="","",TEXT(A284,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C284" s="24">
+        <f>IF(A284="","",YEAR(A284))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="285">
+      <c r="B285" s="23">
+        <f>IF(A285="","",TEXT(A285,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C285" s="23">
+        <f>IF(A285="","",YEAR(A285))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="286">
+      <c r="B286" s="24">
+        <f>IF(A286="","",TEXT(A286,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C286" s="24">
+        <f>IF(A286="","",YEAR(A286))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="287">
+      <c r="B287" s="23">
+        <f>IF(A287="","",TEXT(A287,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C287" s="23">
+        <f>IF(A287="","",YEAR(A287))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="288">
+      <c r="B288" s="24">
+        <f>IF(A288="","",TEXT(A288,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C288" s="24">
+        <f>IF(A288="","",YEAR(A288))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="289">
+      <c r="B289" s="23">
+        <f>IF(A289="","",TEXT(A289,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C289" s="23">
+        <f>IF(A289="","",YEAR(A289))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="290">
+      <c r="B290" s="24">
+        <f>IF(A290="","",TEXT(A290,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C290" s="24">
+        <f>IF(A290="","",YEAR(A290))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="291">
+      <c r="B291" s="23">
+        <f>IF(A291="","",TEXT(A291,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C291" s="23">
+        <f>IF(A291="","",YEAR(A291))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="292">
+      <c r="B292" s="24">
+        <f>IF(A292="","",TEXT(A292,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C292" s="24">
+        <f>IF(A292="","",YEAR(A292))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="293">
+      <c r="B293" s="23">
+        <f>IF(A293="","",TEXT(A293,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C293" s="23">
+        <f>IF(A293="","",YEAR(A293))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="294">
+      <c r="B294" s="24">
+        <f>IF(A294="","",TEXT(A294,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C294" s="24">
+        <f>IF(A294="","",YEAR(A294))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="295">
+      <c r="B295" s="23">
+        <f>IF(A295="","",TEXT(A295,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C295" s="23">
+        <f>IF(A295="","",YEAR(A295))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="296">
+      <c r="B296" s="24">
+        <f>IF(A296="","",TEXT(A296,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C296" s="24">
+        <f>IF(A296="","",YEAR(A296))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="297">
+      <c r="B297" s="23">
+        <f>IF(A297="","",TEXT(A297,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C297" s="23">
+        <f>IF(A297="","",YEAR(A297))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="298">
+      <c r="B298" s="24">
+        <f>IF(A298="","",TEXT(A298,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C298" s="24">
+        <f>IF(A298="","",YEAR(A298))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="299">
+      <c r="B299" s="23">
+        <f>IF(A299="","",TEXT(A299,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C299" s="23">
+        <f>IF(A299="","",YEAR(A299))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="300">
+      <c r="B300" s="24">
+        <f>IF(A300="","",TEXT(A300,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C300" s="24">
+        <f>IF(A300="","",YEAR(A300))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -4144,11 +7124,11 @@
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation sqref="D3:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="D3:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Ingreso,Gasto"</formula1>
     </dataValidation>
     <dataValidation sqref="E3:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Nomina,Vivienda,Transporte,Salud/Deporte,Formacion,Alimentacion,Restaurantes,Trading,Ahorro,Inversion,Ocio,Suscripciones,Amazon,Compras,Otros"</formula1>
+      <formula1>"Nomina,Trading/Payout,Otro ingreso,Vivienda/Alquiler,Coche/Transporte,Gasolina,Parking,Supermercado,Restaurante,Cafeteria/Bar,Peluqueria/Estetica,Farmacia/Salud,Deporte/Gimnasio,Ropa/Calzado,Electronica/Amazon,Hogar,Ocio/Entretenimiento,Viajes/Vacaciones,Formacion/Suscripciones,TraderLab,Software/Apps,Ahorro,Bankroll,Transferencia,Otros"</formula1>
     </dataValidation>
     <dataValidation sqref="I3:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Efectivo,Tarjeta,Transferencia,Domiciliacion,Bizum"</formula1>
@@ -4189,7 +7169,7 @@
           <t>Ingreso neto mensual - MODIFICA AQUI CADA MES:</t>
         </is>
       </c>
-      <c r="D3" s="23" t="n">
+      <c r="D3" s="25" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4276,7 +7256,7 @@
         <f>C9/$D$3</f>
         <v/>
       </c>
-      <c r="E9" s="25" t="inlineStr">
+      <c r="E9" s="23" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
@@ -4324,7 +7304,7 @@
         <f>C11/$D$3</f>
         <v/>
       </c>
-      <c r="E11" s="25" t="inlineStr">
+      <c r="E11" s="23" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
@@ -4402,7 +7382,7 @@
           <t>Bankroll (inversion trading)</t>
         </is>
       </c>
-      <c r="B17" s="23" t="n">
+      <c r="B17" s="25" t="n">
         <v>100</v>
       </c>
       <c r="C17" s="19">
@@ -4425,7 +7405,7 @@
           <t>Ahorro (fondo personal)</t>
         </is>
       </c>
-      <c r="B18" s="23" t="n">
+      <c r="B18" s="25" t="n">
         <v>100</v>
       </c>
       <c r="C18" s="17">

</xml_diff>

<commit_message>
Fix empty category dropdown using named range
Replace 322-char inline string (exceeds Excel 255-char limit) with a
ListaCategorias DefinedName pointing to hidden _LISTAS sheet so the
category dropdown in REGISTRO DE MOVIMIENTOS shows all 25 categories.

https://claude.ai/code/session_01EdLrBe1U3fRxvoA6PYaJVC
</commit_message>
<xml_diff>
--- a/sistema_financiero.xlsx
+++ b/sistema_financiero.xlsx
@@ -23,8 +23,10 @@
     <sheet name="LIBERTAD FINANCIERA" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="PROYECCIONES FUTURAS" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="SCORE DEL TRADER" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="_LISTAS" sheetId="17" state="hidden" r:id="rId17"/>
   </sheets>
   <definedNames>
+    <definedName name="ListaCategorias">_LISTAS!$A$1:$A$25</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'GUIA DE USO'!$A$1:$J$42</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'DASHBOARD EJECUTIVO'!$A$1:$N$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'REGISTRO DE MOVIMIENTOS'!$A$2:$J$2</definedName>
@@ -42,6 +44,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="13">'LIBERTAD FINANCIERA'!$A$1:$F$20</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="14">'PROYECCIONES FUTURAS'!$A$1:$H$21</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="15">'SCORE DEL TRADER'!$A$1:$F$22</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="16">'_LISTAS'!$A$1:$C$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3728,6 +3731,196 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:A25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Nomina</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Trading/Payout</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Otro ingreso</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Vivienda/Alquiler</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Coche/Transporte</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Gasolina</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Supermercado</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Restaurante</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Cafeteria/Bar</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Peluqueria/Estetica</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Farmacia/Salud</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Deporte/Gimnasio</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Ropa/Calzado</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Electronica/Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Hogar</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Ocio/Entretenimiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Viajes/Vacaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Formacion/Suscripciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TraderLab</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Software/Apps</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Ahorro</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Bankroll</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Transferencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -7128,7 +7321,7 @@
       <formula1>"Ingreso,Gasto"</formula1>
     </dataValidation>
     <dataValidation sqref="E3:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Nomina,Trading/Payout,Otro ingreso,Vivienda/Alquiler,Coche/Transporte,Gasolina,Parking,Supermercado,Restaurante,Cafeteria/Bar,Peluqueria/Estetica,Farmacia/Salud,Deporte/Gimnasio,Ropa/Calzado,Electronica/Amazon,Hogar,Ocio/Entretenimiento,Viajes/Vacaciones,Formacion/Suscripciones,TraderLab,Software/Apps,Ahorro,Bankroll,Transferencia,Otros"</formula1>
+      <formula1>ListaCategorias</formula1>
     </dataValidation>
     <dataValidation sqref="I3:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Efectivo,Tarjeta,Transferencia,Domiciliacion,Bizum"</formula1>

</xml_diff>

<commit_message>
Conectar todas las hojas al REGISTRO DE MOVIMIENTOS
- Añade helper reg_sum() para generar SUMPRODUCT filtrados por mes/año/tipo/categoría
- PRESUPUESTO MENSUAL: nueva sección SEGUIMIENTO REAL DEL MES ACTUAL (14 categorías vs presupuesto)
- CONTROL DE AHORRO: muestra total ahorro del mes y 2026 desde REGISTRO (cat=Ahorro)
- CONTROL DE BANKROLL: muestra total bankroll del mes y 2026 desde REGISTRO (cat=Bankroll)
- GASTOS HORMIGA: nueva sección automática (12 categorías, mes actual + acumulado 2026)
- OBJETIVOS: actual ahorro/bankroll conectado a REGISTRO; patrimonio a PATRIMONIO NETO; trading a DASHBOARD
- LIBERTAD FINANCIERA: beneficio medio trading calculado automáticamente desde DASHBOARD
- DASHBOARD EJECUTIVO: KPIs Gastos/Flujo/Trading filtrados por mes actual; nuevo bloque 12 categorías
Todo actualizado en tiempo real al introducir datos en REGISTRO DE MOVIMIENTOS.

https://claude.ai/code/session_01EdLrBe1U3fRxvoA6PYaJVC
</commit_message>
<xml_diff>
--- a/sistema_financiero.xlsx
+++ b/sistema_financiero.xlsx
@@ -28,18 +28,18 @@
   <definedNames>
     <definedName name="ListaCategorias">_LISTAS!$A$1:$A$25</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'GUIA DE USO'!$A$1:$J$42</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'DASHBOARD EJECUTIVO'!$A$1:$N$27</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'DASHBOARD EJECUTIVO'!$A$1:$N$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'REGISTRO DE MOVIMIENTOS'!$A$2:$J$2</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'REGISTRO DE MOVIMIENTOS'!$A$1:$L$305</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'PRESUPUESTO MENSUAL'!$A$1:$H$41</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'CONTROL DE AHORRO'!$A$1:$H$16</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">'CONTROL DE BANKROLL'!$A$1:$G$14</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'PRESUPUESTO MENSUAL'!$A$1:$H$61</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'CONTROL DE AHORRO'!$A$1:$H$19</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'CONTROL DE BANKROLL'!$A$1:$G$17</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'DASHBOARD DE TRADING'!$A$1:$G$515</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'CONTROL DE PAYOUTS'!$A$1:$G$14</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">'PATRIMONIO NETO'!$A$1:$F$28</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="9">'FONDO DE EMERGENCIA'!$A$1:$F$28</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="10">'OBJETIVOS'!$A$1:$H$11</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="11">'GASTOS HORMIGA'!$A$1:$I$513</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="11">'GASTOS HORMIGA'!$A$1:$I$531</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="12">'RANKING MEJORES MESES'!$A$1:$K$17</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="13">'LIBERTAD FINANCIERA'!$A$1:$F$20</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="14">'PROYECCIONES FUTURAS'!$A$1:$H$21</definedName>
@@ -2435,8 +2435,9 @@
       <c r="B3" s="19" t="n">
         <v>2400</v>
       </c>
-      <c r="C3" s="19" t="n">
-        <v>0</v>
+      <c r="C3" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
       </c>
       <c r="D3" s="19">
         <f>C3-B3</f>
@@ -2460,8 +2461,9 @@
       <c r="B4" s="17" t="n">
         <v>2400</v>
       </c>
-      <c r="C4" s="17" t="n">
-        <v>0</v>
+      <c r="C4" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
       </c>
       <c r="D4" s="17">
         <f>C4-B4</f>
@@ -2485,8 +2487,9 @@
       <c r="B5" s="19" t="n">
         <v>5000</v>
       </c>
-      <c r="C5" s="19" t="n">
-        <v>0</v>
+      <c r="C5" s="19">
+        <f>'PATRIMONIO NETO'!B20</f>
+        <v/>
       </c>
       <c r="D5" s="19">
         <f>C5-B5</f>
@@ -2510,8 +2513,9 @@
       <c r="B6" s="17" t="n">
         <v>4200</v>
       </c>
-      <c r="C6" s="17" t="n">
-        <v>0</v>
+      <c r="C6" s="17">
+        <f>SUM('DASHBOARD DE TRADING'!C3:C500)</f>
+        <v/>
       </c>
       <c r="D6" s="17">
         <f>C6-B6</f>
@@ -2554,7 +2558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G508"/>
+  <dimension ref="A1:G526"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2764,8 +2768,338 @@
         <v/>
       </c>
     </row>
+    <row r="512">
+      <c r="A512" s="3" t="inlineStr">
+        <is>
+          <t>GASTOS DEL MES ACTUAL POR CATEGORIA  (automatico desde REGISTRO DE MOVIMIENTOS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" s="7" t="inlineStr">
+        <is>
+          <t>Categoria</t>
+        </is>
+      </c>
+      <c r="B513" s="7" t="inlineStr">
+        <is>
+          <t>Mes Actual (EUR)</t>
+        </is>
+      </c>
+      <c r="C513" s="7" t="inlineStr">
+        <is>
+          <t>% Ingreso</t>
+        </is>
+      </c>
+      <c r="D513" s="7" t="inlineStr">
+        <is>
+          <t>Acumulado 2026 (EUR)</t>
+        </is>
+      </c>
+      <c r="E513" s="7" t="inlineStr">
+        <is>
+          <t>Limite 5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="9" t="inlineStr">
+        <is>
+          <t>Supermercado</t>
+        </is>
+      </c>
+      <c r="B514" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C514" s="18">
+        <f>B514/'PRESUPUESTO MENSUAL'!$D$3</f>
+        <v/>
+      </c>
+      <c r="D514" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E514" s="24">
+        <f>IF(B514&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="8" t="inlineStr">
+        <is>
+          <t>Restaurante</t>
+        </is>
+      </c>
+      <c r="B515" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C515" s="20">
+        <f>B515/'PRESUPUESTO MENSUAL'!$D$3</f>
+        <v/>
+      </c>
+      <c r="D515" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E515" s="23">
+        <f>IF(B515&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="9" t="inlineStr">
+        <is>
+          <t>Cafeteria/Bar</t>
+        </is>
+      </c>
+      <c r="B516" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C516" s="18">
+        <f>B516/'PRESUPUESTO MENSUAL'!$D$3</f>
+        <v/>
+      </c>
+      <c r="D516" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E516" s="24">
+        <f>IF(B516&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" s="8" t="inlineStr">
+        <is>
+          <t>Ocio/Entretenimiento</t>
+        </is>
+      </c>
+      <c r="B517" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C517" s="20">
+        <f>B517/'PRESUPUESTO MENSUAL'!$D$3</f>
+        <v/>
+      </c>
+      <c r="D517" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E517" s="23">
+        <f>IF(B517&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="9" t="inlineStr">
+        <is>
+          <t>Ropa/Calzado</t>
+        </is>
+      </c>
+      <c r="B518" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C518" s="18">
+        <f>B518/'PRESUPUESTO MENSUAL'!$D$3</f>
+        <v/>
+      </c>
+      <c r="D518" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E518" s="24">
+        <f>IF(B518&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" s="8" t="inlineStr">
+        <is>
+          <t>Electronica/Amazon</t>
+        </is>
+      </c>
+      <c r="B519" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Electronica/Amazon")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C519" s="20">
+        <f>B519/'PRESUPUESTO MENSUAL'!$D$3</f>
+        <v/>
+      </c>
+      <c r="D519" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Electronica/Amazon")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E519" s="23">
+        <f>IF(B519&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" s="9" t="inlineStr">
+        <is>
+          <t>Farmacia/Salud</t>
+        </is>
+      </c>
+      <c r="B520" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C520" s="18">
+        <f>B520/'PRESUPUESTO MENSUAL'!$D$3</f>
+        <v/>
+      </c>
+      <c r="D520" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E520" s="24">
+        <f>IF(B520&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" s="8" t="inlineStr">
+        <is>
+          <t>Peluqueria/Estetica</t>
+        </is>
+      </c>
+      <c r="B521" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Peluqueria/Estetica")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C521" s="20">
+        <f>B521/'PRESUPUESTO MENSUAL'!$D$3</f>
+        <v/>
+      </c>
+      <c r="D521" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Peluqueria/Estetica")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E521" s="23">
+        <f>IF(B521&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="9" t="inlineStr">
+        <is>
+          <t>Hogar</t>
+        </is>
+      </c>
+      <c r="B522" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Hogar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C522" s="18">
+        <f>B522/'PRESUPUESTO MENSUAL'!$D$3</f>
+        <v/>
+      </c>
+      <c r="D522" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Hogar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E522" s="24">
+        <f>IF(B522&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" s="8" t="inlineStr">
+        <is>
+          <t>Formacion/Suscripciones</t>
+        </is>
+      </c>
+      <c r="B523" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C523" s="20">
+        <f>B523/'PRESUPUESTO MENSUAL'!$D$3</f>
+        <v/>
+      </c>
+      <c r="D523" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E523" s="23">
+        <f>IF(B523&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="9" t="inlineStr">
+        <is>
+          <t>Software/Apps</t>
+        </is>
+      </c>
+      <c r="B524" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Software/Apps")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C524" s="18">
+        <f>B524/'PRESUPUESTO MENSUAL'!$D$3</f>
+        <v/>
+      </c>
+      <c r="D524" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Software/Apps")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E524" s="24">
+        <f>IF(B524&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" s="8" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
+      <c r="B525" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C525" s="20">
+        <f>B525/'PRESUPUESTO MENSUAL'!$D$3</f>
+        <v/>
+      </c>
+      <c r="D525" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E525" s="23">
+        <f>IF(B525&gt;'PRESUPUESTO MENSUAL'!$D$3*0.05,"EXCEDIDO","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL GASTOS VARIABLES DEL MES</t>
+        </is>
+      </c>
+      <c r="B526" s="21">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C526" s="22">
+        <f>B526/'PRESUPUESTO MENSUAL'!$D$3</f>
+        <v/>
+      </c>
+      <c r="D526" s="21">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A512:E512"/>
     <mergeCell ref="A502:G502"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
@@ -3133,8 +3467,9 @@
           <t>Beneficio medio mensual trading (editar)</t>
         </is>
       </c>
-      <c r="B4" s="17" t="n">
-        <v>0</v>
+      <c r="B4" s="17">
+        <f>IFERROR(SUM('DASHBOARD DE TRADING'!C3:C500)/MAX(1,COUNTA('DASHBOARD DE TRADING'!A3:A500)),0)</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -3928,7 +4263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3981,12 +4316,12 @@
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>Gastos Totales (Movimientos)</t>
+          <t>Gastos Reales (mes actual)</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
-          <t>Flujo de Caja</t>
+          <t>Flujo de Caja (mes actual)</t>
         </is>
       </c>
       <c r="G6" s="13" t="inlineStr">
@@ -4011,11 +4346,11 @@
         <v/>
       </c>
       <c r="C7" s="14">
-        <f>SUMIF('REGISTRO DE MOVIMIENTOS'!D3:D1000,"Gasto",'REGISTRO DE MOVIMIENTOS'!H3:H1000)</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="E7" s="14">
-        <f>'PRESUPUESTO MENSUAL'!$D$3-SUMIF('REGISTRO DE MOVIMIENTOS'!D3:D1000,"Gasto",'REGISTRO DE MOVIMIENTOS'!H3:H1000)</f>
+        <f>'PRESUPUESTO MENSUAL'!$D$3-(SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500)))</f>
         <v/>
       </c>
       <c r="G7" s="14">
@@ -4035,7 +4370,7 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>Benef. Trading Mes</t>
+          <t>Benef. Trading (mes actual)</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
@@ -4066,7 +4401,7 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="14">
-        <f>SUM('DASHBOARD DE TRADING'!C3:C1000)</f>
+        <f>SUMPRODUCT((ISNUMBER('DASHBOARD DE TRADING'!A3:A500))*(MONTH(IF(ISNUMBER('DASHBOARD DE TRADING'!A3:A500),'DASHBOARD DE TRADING'!A3:A500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('DASHBOARD DE TRADING'!A3:A500),'DASHBOARD DE TRADING'!A3:A500,TODAY()))=YEAR(TODAY()))*('DASHBOARD DE TRADING'!C3:C500))</f>
         <v/>
       </c>
       <c r="C10" s="14">
@@ -4205,20 +4540,155 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>GASTOS POR CATEGORIA DEL MES ACTUAL (desde REGISTRO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Vivienda/Alquiler</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>Coche/Transporte</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>Gasolina</t>
+        </is>
+      </c>
+      <c r="G23" s="13" t="inlineStr">
+        <is>
+          <t>Supermercado</t>
+        </is>
+      </c>
+      <c r="I23" s="13" t="inlineStr">
+        <is>
+          <t>Restaurante</t>
+        </is>
+      </c>
+      <c r="K23" s="13" t="inlineStr">
+        <is>
+          <t>Cafeteria/Bar</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="14">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Vivienda/Alquiler")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C24" s="14">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Coche/Transporte")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E24" s="14">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Gasolina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G24" s="14">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I24" s="14">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K24" s="14">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="12" customHeight="1"/>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>Ocio/Entretenimiento</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>Ropa/Calzado</t>
+        </is>
+      </c>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
+          <t>Farmacia/Salud</t>
+        </is>
+      </c>
+      <c r="G26" s="13" t="inlineStr">
+        <is>
+          <t>Formacion/Suscripciones</t>
+        </is>
+      </c>
+      <c r="I26" s="13" t="inlineStr">
+        <is>
+          <t>Ahorro</t>
+        </is>
+      </c>
+      <c r="K26" s="13" t="inlineStr">
+        <is>
+          <t>Bankroll</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="14">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C27" s="14">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E27" s="14">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G27" s="14">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I27" s="14">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K27" s="14">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="12" customHeight="1"/>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>NAVEGACION: Usa las pestanas de abajo para acceder a cada seccion del sistema</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="30">
+  <mergeCells count="55">
+    <mergeCell ref="K27:L28"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="I6:J6"/>
+    <mergeCell ref="G24:H25"/>
+    <mergeCell ref="I24:J25"/>
     <mergeCell ref="K9:L9"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="E27:F28"/>
+    <mergeCell ref="G23:H23"/>
     <mergeCell ref="A3:L3"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="I26:J26"/>
     <mergeCell ref="A6:B6"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="C27:D28"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="K7:L8"/>
     <mergeCell ref="C7:D8"/>
@@ -4230,10 +4700,25 @@
     <mergeCell ref="A22:L22"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="C9:D9"/>
+    <mergeCell ref="A27:B28"/>
     <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G27:H28"/>
+    <mergeCell ref="A26:B26"/>
     <mergeCell ref="E6:F6"/>
+    <mergeCell ref="C24:D25"/>
+    <mergeCell ref="E24:F25"/>
+    <mergeCell ref="K24:L25"/>
     <mergeCell ref="K6:L6"/>
     <mergeCell ref="A13:L13"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="I27:J28"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="K23:L23"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="A24:B25"/>
+    <mergeCell ref="A30:L30"/>
     <mergeCell ref="G7:H8"/>
     <mergeCell ref="I7:J8"/>
     <mergeCell ref="C10:D11"/>
@@ -7339,7 +7824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -7796,9 +8281,399 @@
         <v/>
       </c>
     </row>
+    <row r="38" ht="25" customHeight="1">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>SEGUIMIENTO REAL DEL MES ACTUAL  (actualizado automaticamente desde REGISTRO DE MOVIMIENTOS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>Categoria / Concepto</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Presupuestado</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Gastado Real (mes)</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Diferencia</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>Vivienda/Alquiler</t>
+        </is>
+      </c>
+      <c r="B40" s="17">
+        <f>C8</f>
+        <v/>
+      </c>
+      <c r="C40" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Vivienda/Alquiler")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D40" s="17">
+        <f>B40-C40</f>
+        <v/>
+      </c>
+      <c r="E40" s="24">
+        <f>IF(B40=0,"Sin limite",IF(C40&lt;=B40,"OK","EXCEDIDO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>Coche/Transporte</t>
+        </is>
+      </c>
+      <c r="B41" s="19">
+        <f>C9</f>
+        <v/>
+      </c>
+      <c r="C41" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Coche/Transporte")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D41" s="19">
+        <f>B41-C41</f>
+        <v/>
+      </c>
+      <c r="E41" s="23">
+        <f>IF(B41=0,"Sin limite",IF(C41&lt;=B41,"OK","EXCEDIDO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>Gasolina</t>
+        </is>
+      </c>
+      <c r="B42" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Gasolina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D42" s="17">
+        <f>B42-C42</f>
+        <v/>
+      </c>
+      <c r="E42" s="24">
+        <f>IF(B42=0,"Sin limite",IF(C42&lt;=B42,"OK","EXCEDIDO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>Supermercado</t>
+        </is>
+      </c>
+      <c r="B43" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D43" s="19">
+        <f>B43-C43</f>
+        <v/>
+      </c>
+      <c r="E43" s="23">
+        <f>IF(B43=0,"Sin limite",IF(C43&lt;=B43,"OK","EXCEDIDO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>Restaurante</t>
+        </is>
+      </c>
+      <c r="B44" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D44" s="17">
+        <f>B44-C44</f>
+        <v/>
+      </c>
+      <c r="E44" s="24">
+        <f>IF(B44=0,"Sin limite",IF(C44&lt;=B44,"OK","EXCEDIDO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>Cafeteria/Bar</t>
+        </is>
+      </c>
+      <c r="B45" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D45" s="19">
+        <f>B45-C45</f>
+        <v/>
+      </c>
+      <c r="E45" s="23">
+        <f>IF(B45=0,"Sin limite",IF(C45&lt;=B45,"OK","EXCEDIDO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>Ocio/Entretenimiento</t>
+        </is>
+      </c>
+      <c r="B46" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D46" s="17">
+        <f>B46-C46</f>
+        <v/>
+      </c>
+      <c r="E46" s="24">
+        <f>IF(B46=0,"Sin limite",IF(C46&lt;=B46,"OK","EXCEDIDO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>Ropa/Calzado</t>
+        </is>
+      </c>
+      <c r="B47" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D47" s="19">
+        <f>B47-C47</f>
+        <v/>
+      </c>
+      <c r="E47" s="23">
+        <f>IF(B47=0,"Sin limite",IF(C47&lt;=B47,"OK","EXCEDIDO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>Farmacia/Salud</t>
+        </is>
+      </c>
+      <c r="B48" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D48" s="17">
+        <f>B48-C48</f>
+        <v/>
+      </c>
+      <c r="E48" s="24">
+        <f>IF(B48=0,"Sin limite",IF(C48&lt;=B48,"OK","EXCEDIDO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>Deporte/Gimnasio</t>
+        </is>
+      </c>
+      <c r="B49" s="19">
+        <f>C10</f>
+        <v/>
+      </c>
+      <c r="C49" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Deporte/Gimnasio")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D49" s="19">
+        <f>B49-C49</f>
+        <v/>
+      </c>
+      <c r="E49" s="23">
+        <f>IF(B49=0,"Sin limite",IF(C49&lt;=B49,"OK","EXCEDIDO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>Formacion/Suscripciones</t>
+        </is>
+      </c>
+      <c r="B50" s="17">
+        <f>C11</f>
+        <v/>
+      </c>
+      <c r="C50" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D50" s="17">
+        <f>B50-C50</f>
+        <v/>
+      </c>
+      <c r="E50" s="24">
+        <f>IF(B50=0,"Sin limite",IF(C50&lt;=B50,"OK","EXCEDIDO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>Ahorro</t>
+        </is>
+      </c>
+      <c r="B51" s="19">
+        <f>B18</f>
+        <v/>
+      </c>
+      <c r="C51" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D51" s="19">
+        <f>B51-C51</f>
+        <v/>
+      </c>
+      <c r="E51" s="23">
+        <f>IF(B51=0,"Sin limite",IF(C51&lt;=B51,"OK","EXCEDIDO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>Bankroll</t>
+        </is>
+      </c>
+      <c r="B52" s="17">
+        <f>B17</f>
+        <v/>
+      </c>
+      <c r="C52" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D52" s="17">
+        <f>B52-C52</f>
+        <v/>
+      </c>
+      <c r="E52" s="24">
+        <f>IF(B52=0,"Sin limite",IF(C52&lt;=B52,"OK","EXCEDIDO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
+      <c r="B53" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D53" s="19">
+        <f>B53-C53</f>
+        <v/>
+      </c>
+      <c r="E53" s="23">
+        <f>IF(B53=0,"Sin limite",IF(C53&lt;=B53,"OK","EXCEDIDO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL GASTOS REALES DEL MES</t>
+        </is>
+      </c>
+      <c r="C54" s="21">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D54" s="21">
+        <f>$D$3-C54</f>
+        <v/>
+      </c>
+      <c r="E54" s="4">
+        <f>IF(C54&lt;=$D$3,"Dentro del ingreso","SUPERA EL INGRESO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL INGRESOS REGISTRADOS DEL MES</t>
+        </is>
+      </c>
+      <c r="C55" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>% del presupuesto ejecutado (gastos / ingreso)</t>
+        </is>
+      </c>
+      <c r="C56" s="18">
+        <f>IFERROR(C54/$D$3,0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="B35:E35"/>
+    <mergeCell ref="A38:E38"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A32:F32"/>
@@ -7843,7 +8718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -7955,10 +8830,50 @@
         <v/>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>DESDE REGISTRO DE MOVIMIENTOS (automatico)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Ahorro registrado este mes</t>
+        </is>
+      </c>
+      <c r="B13" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Suma entradas Categoria=Ahorro del mes en curso</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Ahorro registrado en 2026</t>
+        </is>
+      </c>
+      <c r="B14" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Acumulado anual segun REGISTRO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A12:F12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
@@ -7973,7 +8888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -8068,10 +8983,50 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>DESDE REGISTRO DE MOVIMIENTOS (automatico)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Bankroll registrado este mes</t>
+        </is>
+      </c>
+      <c r="B11" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Suma entradas Categoria=Bankroll del mes en curso</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Bankroll registrado en 2026</t>
+        </is>
+      </c>
+      <c r="B12" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Acumulado anual segun REGISTRO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A10:E10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>

</xml_diff>

<commit_message>
Auto-Tipo en REGISTRO, semaforo verde/amarillo/rojo, limites editables
- REGISTRO DE MOVIMIENTOS: columna Tipo (auto) con formula basada en Categoria.
  Nomina/Trading/Otro ingreso = Ingreso; todo lo demas = Gasto.
  El usuario ya no tiene que rellenar Tipo manualmente.
- PRESUPUESTO MENSUAL seguimiento: semaforo completo en filas A41:E54.
  Verde claro (<80% del limite), amarillo (80-100%), rojo (excedido).
- Limites mensuales editables (celdas doradas) para categorias variables:
  Gasolina 80€, Supermercado 200€, Restaurante 100€, Cafeteria 40€,
  Ocio 80€, Ropa 60€, Farmacia 40€, Otros 50€. El usuario los cambia libremente.
- Corregida sintaxis OR() en formula auto-Tipo.

https://claude.ai/code/session_01EdLrBe1U3fRxvoA6PYaJVC
</commit_message>
<xml_diff>
--- a/sistema_financiero.xlsx
+++ b/sistema_financiero.xlsx
@@ -31,7 +31,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="1">'DASHBOARD EJECUTIVO'!$A$1:$N$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'REGISTRO DE MOVIMIENTOS'!$A$2:$J$2</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'REGISTRO DE MOVIMIENTOS'!$A$1:$L$305</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'PRESUPUESTO MENSUAL'!$A$1:$H$61</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'PRESUPUESTO MENSUAL'!$A$1:$H$62</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'CONTROL DE AHORRO'!$A$1:$H$19</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'CONTROL DE BANKROLL'!$A$1:$G$17</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'DASHBOARD DE TRADING'!$A$1:$G$515</definedName>
@@ -419,14 +419,21 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00C6EFCE"/>
+          <fgColor rgb="00FFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFC7CE"/>
+          <fgColor rgb="00FFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -448,13 +455,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="0028A745"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2535,14 +2535,14 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="E3:E10">
-    <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
+    <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="2">
       <formula>0.75</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="between" dxfId="5">
+    <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
       <formula>0.5</formula>
       <formula>0.75</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="lessThan" dxfId="1">
+    <cfRule type="cellIs" priority="3" operator="lessThan" dxfId="0">
       <formula>0.5</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4782,7 +4782,7 @@
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>Tipo</t>
+          <t>Tipo (auto)</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
@@ -4825,6 +4825,10 @@
         <f>IF(A3="","",YEAR(A3))</f>
         <v/>
       </c>
+      <c r="D3" s="23">
+        <f>IF(A3="","",IF(OR(E3="Nomina",E3="Trading/Payout",E3="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="B4" s="24">
@@ -4835,6 +4839,10 @@
         <f>IF(A4="","",YEAR(A4))</f>
         <v/>
       </c>
+      <c r="D4" s="24">
+        <f>IF(A4="","",IF(OR(E4="Nomina",E4="Trading/Payout",E4="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="B5" s="23">
@@ -4845,6 +4853,10 @@
         <f>IF(A5="","",YEAR(A5))</f>
         <v/>
       </c>
+      <c r="D5" s="23">
+        <f>IF(A5="","",IF(OR(E5="Nomina",E5="Trading/Payout",E5="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="B6" s="24">
@@ -4855,6 +4867,10 @@
         <f>IF(A6="","",YEAR(A6))</f>
         <v/>
       </c>
+      <c r="D6" s="24">
+        <f>IF(A6="","",IF(OR(E6="Nomina",E6="Trading/Payout",E6="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="23">
@@ -4865,6 +4881,10 @@
         <f>IF(A7="","",YEAR(A7))</f>
         <v/>
       </c>
+      <c r="D7" s="23">
+        <f>IF(A7="","",IF(OR(E7="Nomina",E7="Trading/Payout",E7="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="B8" s="24">
@@ -4875,6 +4895,10 @@
         <f>IF(A8="","",YEAR(A8))</f>
         <v/>
       </c>
+      <c r="D8" s="24">
+        <f>IF(A8="","",IF(OR(E8="Nomina",E8="Trading/Payout",E8="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="B9" s="23">
@@ -4885,6 +4909,10 @@
         <f>IF(A9="","",YEAR(A9))</f>
         <v/>
       </c>
+      <c r="D9" s="23">
+        <f>IF(A9="","",IF(OR(E9="Nomina",E9="Trading/Payout",E9="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="24">
@@ -4895,6 +4923,10 @@
         <f>IF(A10="","",YEAR(A10))</f>
         <v/>
       </c>
+      <c r="D10" s="24">
+        <f>IF(A10="","",IF(OR(E10="Nomina",E10="Trading/Payout",E10="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="B11" s="23">
@@ -4905,6 +4937,10 @@
         <f>IF(A11="","",YEAR(A11))</f>
         <v/>
       </c>
+      <c r="D11" s="23">
+        <f>IF(A11="","",IF(OR(E11="Nomina",E11="Trading/Payout",E11="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="B12" s="24">
@@ -4915,6 +4951,10 @@
         <f>IF(A12="","",YEAR(A12))</f>
         <v/>
       </c>
+      <c r="D12" s="24">
+        <f>IF(A12="","",IF(OR(E12="Nomina",E12="Trading/Payout",E12="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="23">
@@ -4925,6 +4965,10 @@
         <f>IF(A13="","",YEAR(A13))</f>
         <v/>
       </c>
+      <c r="D13" s="23">
+        <f>IF(A13="","",IF(OR(E13="Nomina",E13="Trading/Payout",E13="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="24">
@@ -4935,6 +4979,10 @@
         <f>IF(A14="","",YEAR(A14))</f>
         <v/>
       </c>
+      <c r="D14" s="24">
+        <f>IF(A14="","",IF(OR(E14="Nomina",E14="Trading/Payout",E14="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="B15" s="23">
@@ -4945,6 +4993,10 @@
         <f>IF(A15="","",YEAR(A15))</f>
         <v/>
       </c>
+      <c r="D15" s="23">
+        <f>IF(A15="","",IF(OR(E15="Nomina",E15="Trading/Payout",E15="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="B16" s="24">
@@ -4955,6 +5007,10 @@
         <f>IF(A16="","",YEAR(A16))</f>
         <v/>
       </c>
+      <c r="D16" s="24">
+        <f>IF(A16="","",IF(OR(E16="Nomina",E16="Trading/Payout",E16="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="B17" s="23">
@@ -4965,6 +5021,10 @@
         <f>IF(A17="","",YEAR(A17))</f>
         <v/>
       </c>
+      <c r="D17" s="23">
+        <f>IF(A17="","",IF(OR(E17="Nomina",E17="Trading/Payout",E17="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="24">
@@ -4975,6 +5035,10 @@
         <f>IF(A18="","",YEAR(A18))</f>
         <v/>
       </c>
+      <c r="D18" s="24">
+        <f>IF(A18="","",IF(OR(E18="Nomina",E18="Trading/Payout",E18="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="B19" s="23">
@@ -4985,6 +5049,10 @@
         <f>IF(A19="","",YEAR(A19))</f>
         <v/>
       </c>
+      <c r="D19" s="23">
+        <f>IF(A19="","",IF(OR(E19="Nomina",E19="Trading/Payout",E19="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="B20" s="24">
@@ -4995,6 +5063,10 @@
         <f>IF(A20="","",YEAR(A20))</f>
         <v/>
       </c>
+      <c r="D20" s="24">
+        <f>IF(A20="","",IF(OR(E20="Nomina",E20="Trading/Payout",E20="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="23">
@@ -5005,6 +5077,10 @@
         <f>IF(A21="","",YEAR(A21))</f>
         <v/>
       </c>
+      <c r="D21" s="23">
+        <f>IF(A21="","",IF(OR(E21="Nomina",E21="Trading/Payout",E21="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="B22" s="24">
@@ -5015,6 +5091,10 @@
         <f>IF(A22="","",YEAR(A22))</f>
         <v/>
       </c>
+      <c r="D22" s="24">
+        <f>IF(A22="","",IF(OR(E22="Nomina",E22="Trading/Payout",E22="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="23">
@@ -5025,6 +5105,10 @@
         <f>IF(A23="","",YEAR(A23))</f>
         <v/>
       </c>
+      <c r="D23" s="23">
+        <f>IF(A23="","",IF(OR(E23="Nomina",E23="Trading/Payout",E23="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="B24" s="24">
@@ -5035,6 +5119,10 @@
         <f>IF(A24="","",YEAR(A24))</f>
         <v/>
       </c>
+      <c r="D24" s="24">
+        <f>IF(A24="","",IF(OR(E24="Nomina",E24="Trading/Payout",E24="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="23">
@@ -5045,6 +5133,10 @@
         <f>IF(A25="","",YEAR(A25))</f>
         <v/>
       </c>
+      <c r="D25" s="23">
+        <f>IF(A25="","",IF(OR(E25="Nomina",E25="Trading/Payout",E25="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="24">
@@ -5055,6 +5147,10 @@
         <f>IF(A26="","",YEAR(A26))</f>
         <v/>
       </c>
+      <c r="D26" s="24">
+        <f>IF(A26="","",IF(OR(E26="Nomina",E26="Trading/Payout",E26="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="23">
@@ -5065,6 +5161,10 @@
         <f>IF(A27="","",YEAR(A27))</f>
         <v/>
       </c>
+      <c r="D27" s="23">
+        <f>IF(A27="","",IF(OR(E27="Nomina",E27="Trading/Payout",E27="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="B28" s="24">
@@ -5075,6 +5175,10 @@
         <f>IF(A28="","",YEAR(A28))</f>
         <v/>
       </c>
+      <c r="D28" s="24">
+        <f>IF(A28="","",IF(OR(E28="Nomina",E28="Trading/Payout",E28="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="B29" s="23">
@@ -5085,6 +5189,10 @@
         <f>IF(A29="","",YEAR(A29))</f>
         <v/>
       </c>
+      <c r="D29" s="23">
+        <f>IF(A29="","",IF(OR(E29="Nomina",E29="Trading/Payout",E29="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="B30" s="24">
@@ -5095,6 +5203,10 @@
         <f>IF(A30="","",YEAR(A30))</f>
         <v/>
       </c>
+      <c r="D30" s="24">
+        <f>IF(A30="","",IF(OR(E30="Nomina",E30="Trading/Payout",E30="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="B31" s="23">
@@ -5105,6 +5217,10 @@
         <f>IF(A31="","",YEAR(A31))</f>
         <v/>
       </c>
+      <c r="D31" s="23">
+        <f>IF(A31="","",IF(OR(E31="Nomina",E31="Trading/Payout",E31="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="B32" s="24">
@@ -5115,6 +5231,10 @@
         <f>IF(A32="","",YEAR(A32))</f>
         <v/>
       </c>
+      <c r="D32" s="24">
+        <f>IF(A32="","",IF(OR(E32="Nomina",E32="Trading/Payout",E32="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="B33" s="23">
@@ -5125,6 +5245,10 @@
         <f>IF(A33="","",YEAR(A33))</f>
         <v/>
       </c>
+      <c r="D33" s="23">
+        <f>IF(A33="","",IF(OR(E33="Nomina",E33="Trading/Payout",E33="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="B34" s="24">
@@ -5135,6 +5259,10 @@
         <f>IF(A34="","",YEAR(A34))</f>
         <v/>
       </c>
+      <c r="D34" s="24">
+        <f>IF(A34="","",IF(OR(E34="Nomina",E34="Trading/Payout",E34="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="B35" s="23">
@@ -5145,6 +5273,10 @@
         <f>IF(A35="","",YEAR(A35))</f>
         <v/>
       </c>
+      <c r="D35" s="23">
+        <f>IF(A35="","",IF(OR(E35="Nomina",E35="Trading/Payout",E35="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="B36" s="24">
@@ -5155,6 +5287,10 @@
         <f>IF(A36="","",YEAR(A36))</f>
         <v/>
       </c>
+      <c r="D36" s="24">
+        <f>IF(A36="","",IF(OR(E36="Nomina",E36="Trading/Payout",E36="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="B37" s="23">
@@ -5165,6 +5301,10 @@
         <f>IF(A37="","",YEAR(A37))</f>
         <v/>
       </c>
+      <c r="D37" s="23">
+        <f>IF(A37="","",IF(OR(E37="Nomina",E37="Trading/Payout",E37="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="B38" s="24">
@@ -5175,6 +5315,10 @@
         <f>IF(A38="","",YEAR(A38))</f>
         <v/>
       </c>
+      <c r="D38" s="24">
+        <f>IF(A38="","",IF(OR(E38="Nomina",E38="Trading/Payout",E38="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="B39" s="23">
@@ -5185,6 +5329,10 @@
         <f>IF(A39="","",YEAR(A39))</f>
         <v/>
       </c>
+      <c r="D39" s="23">
+        <f>IF(A39="","",IF(OR(E39="Nomina",E39="Trading/Payout",E39="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="B40" s="24">
@@ -5195,6 +5343,10 @@
         <f>IF(A40="","",YEAR(A40))</f>
         <v/>
       </c>
+      <c r="D40" s="24">
+        <f>IF(A40="","",IF(OR(E40="Nomina",E40="Trading/Payout",E40="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="B41" s="23">
@@ -5205,6 +5357,10 @@
         <f>IF(A41="","",YEAR(A41))</f>
         <v/>
       </c>
+      <c r="D41" s="23">
+        <f>IF(A41="","",IF(OR(E41="Nomina",E41="Trading/Payout",E41="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="B42" s="24">
@@ -5215,6 +5371,10 @@
         <f>IF(A42="","",YEAR(A42))</f>
         <v/>
       </c>
+      <c r="D42" s="24">
+        <f>IF(A42="","",IF(OR(E42="Nomina",E42="Trading/Payout",E42="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="B43" s="23">
@@ -5225,6 +5385,10 @@
         <f>IF(A43="","",YEAR(A43))</f>
         <v/>
       </c>
+      <c r="D43" s="23">
+        <f>IF(A43="","",IF(OR(E43="Nomina",E43="Trading/Payout",E43="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="B44" s="24">
@@ -5235,6 +5399,10 @@
         <f>IF(A44="","",YEAR(A44))</f>
         <v/>
       </c>
+      <c r="D44" s="24">
+        <f>IF(A44="","",IF(OR(E44="Nomina",E44="Trading/Payout",E44="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="B45" s="23">
@@ -5245,6 +5413,10 @@
         <f>IF(A45="","",YEAR(A45))</f>
         <v/>
       </c>
+      <c r="D45" s="23">
+        <f>IF(A45="","",IF(OR(E45="Nomina",E45="Trading/Payout",E45="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="B46" s="24">
@@ -5255,6 +5427,10 @@
         <f>IF(A46="","",YEAR(A46))</f>
         <v/>
       </c>
+      <c r="D46" s="24">
+        <f>IF(A46="","",IF(OR(E46="Nomina",E46="Trading/Payout",E46="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="B47" s="23">
@@ -5265,6 +5441,10 @@
         <f>IF(A47="","",YEAR(A47))</f>
         <v/>
       </c>
+      <c r="D47" s="23">
+        <f>IF(A47="","",IF(OR(E47="Nomina",E47="Trading/Payout",E47="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="B48" s="24">
@@ -5275,6 +5455,10 @@
         <f>IF(A48="","",YEAR(A48))</f>
         <v/>
       </c>
+      <c r="D48" s="24">
+        <f>IF(A48="","",IF(OR(E48="Nomina",E48="Trading/Payout",E48="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="B49" s="23">
@@ -5285,6 +5469,10 @@
         <f>IF(A49="","",YEAR(A49))</f>
         <v/>
       </c>
+      <c r="D49" s="23">
+        <f>IF(A49="","",IF(OR(E49="Nomina",E49="Trading/Payout",E49="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="B50" s="24">
@@ -5295,6 +5483,10 @@
         <f>IF(A50="","",YEAR(A50))</f>
         <v/>
       </c>
+      <c r="D50" s="24">
+        <f>IF(A50="","",IF(OR(E50="Nomina",E50="Trading/Payout",E50="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="B51" s="23">
@@ -5305,6 +5497,10 @@
         <f>IF(A51="","",YEAR(A51))</f>
         <v/>
       </c>
+      <c r="D51" s="23">
+        <f>IF(A51="","",IF(OR(E51="Nomina",E51="Trading/Payout",E51="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="B52" s="24">
@@ -5315,6 +5511,10 @@
         <f>IF(A52="","",YEAR(A52))</f>
         <v/>
       </c>
+      <c r="D52" s="24">
+        <f>IF(A52="","",IF(OR(E52="Nomina",E52="Trading/Payout",E52="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="B53" s="23">
@@ -5325,6 +5525,10 @@
         <f>IF(A53="","",YEAR(A53))</f>
         <v/>
       </c>
+      <c r="D53" s="23">
+        <f>IF(A53="","",IF(OR(E53="Nomina",E53="Trading/Payout",E53="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="B54" s="24">
@@ -5335,6 +5539,10 @@
         <f>IF(A54="","",YEAR(A54))</f>
         <v/>
       </c>
+      <c r="D54" s="24">
+        <f>IF(A54="","",IF(OR(E54="Nomina",E54="Trading/Payout",E54="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="B55" s="23">
@@ -5345,6 +5553,10 @@
         <f>IF(A55="","",YEAR(A55))</f>
         <v/>
       </c>
+      <c r="D55" s="23">
+        <f>IF(A55="","",IF(OR(E55="Nomina",E55="Trading/Payout",E55="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="B56" s="24">
@@ -5355,6 +5567,10 @@
         <f>IF(A56="","",YEAR(A56))</f>
         <v/>
       </c>
+      <c r="D56" s="24">
+        <f>IF(A56="","",IF(OR(E56="Nomina",E56="Trading/Payout",E56="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="B57" s="23">
@@ -5365,6 +5581,10 @@
         <f>IF(A57="","",YEAR(A57))</f>
         <v/>
       </c>
+      <c r="D57" s="23">
+        <f>IF(A57="","",IF(OR(E57="Nomina",E57="Trading/Payout",E57="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="B58" s="24">
@@ -5375,6 +5595,10 @@
         <f>IF(A58="","",YEAR(A58))</f>
         <v/>
       </c>
+      <c r="D58" s="24">
+        <f>IF(A58="","",IF(OR(E58="Nomina",E58="Trading/Payout",E58="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="B59" s="23">
@@ -5385,6 +5609,10 @@
         <f>IF(A59="","",YEAR(A59))</f>
         <v/>
       </c>
+      <c r="D59" s="23">
+        <f>IF(A59="","",IF(OR(E59="Nomina",E59="Trading/Payout",E59="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="B60" s="24">
@@ -5395,6 +5623,10 @@
         <f>IF(A60="","",YEAR(A60))</f>
         <v/>
       </c>
+      <c r="D60" s="24">
+        <f>IF(A60="","",IF(OR(E60="Nomina",E60="Trading/Payout",E60="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="B61" s="23">
@@ -5405,6 +5637,10 @@
         <f>IF(A61="","",YEAR(A61))</f>
         <v/>
       </c>
+      <c r="D61" s="23">
+        <f>IF(A61="","",IF(OR(E61="Nomina",E61="Trading/Payout",E61="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="B62" s="24">
@@ -5415,6 +5651,10 @@
         <f>IF(A62="","",YEAR(A62))</f>
         <v/>
       </c>
+      <c r="D62" s="24">
+        <f>IF(A62="","",IF(OR(E62="Nomina",E62="Trading/Payout",E62="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="B63" s="23">
@@ -5425,6 +5665,10 @@
         <f>IF(A63="","",YEAR(A63))</f>
         <v/>
       </c>
+      <c r="D63" s="23">
+        <f>IF(A63="","",IF(OR(E63="Nomina",E63="Trading/Payout",E63="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="B64" s="24">
@@ -5435,6 +5679,10 @@
         <f>IF(A64="","",YEAR(A64))</f>
         <v/>
       </c>
+      <c r="D64" s="24">
+        <f>IF(A64="","",IF(OR(E64="Nomina",E64="Trading/Payout",E64="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="B65" s="23">
@@ -5445,6 +5693,10 @@
         <f>IF(A65="","",YEAR(A65))</f>
         <v/>
       </c>
+      <c r="D65" s="23">
+        <f>IF(A65="","",IF(OR(E65="Nomina",E65="Trading/Payout",E65="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="B66" s="24">
@@ -5455,6 +5707,10 @@
         <f>IF(A66="","",YEAR(A66))</f>
         <v/>
       </c>
+      <c r="D66" s="24">
+        <f>IF(A66="","",IF(OR(E66="Nomina",E66="Trading/Payout",E66="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="B67" s="23">
@@ -5465,6 +5721,10 @@
         <f>IF(A67="","",YEAR(A67))</f>
         <v/>
       </c>
+      <c r="D67" s="23">
+        <f>IF(A67="","",IF(OR(E67="Nomina",E67="Trading/Payout",E67="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="B68" s="24">
@@ -5475,6 +5735,10 @@
         <f>IF(A68="","",YEAR(A68))</f>
         <v/>
       </c>
+      <c r="D68" s="24">
+        <f>IF(A68="","",IF(OR(E68="Nomina",E68="Trading/Payout",E68="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="B69" s="23">
@@ -5485,6 +5749,10 @@
         <f>IF(A69="","",YEAR(A69))</f>
         <v/>
       </c>
+      <c r="D69" s="23">
+        <f>IF(A69="","",IF(OR(E69="Nomina",E69="Trading/Payout",E69="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="B70" s="24">
@@ -5495,6 +5763,10 @@
         <f>IF(A70="","",YEAR(A70))</f>
         <v/>
       </c>
+      <c r="D70" s="24">
+        <f>IF(A70="","",IF(OR(E70="Nomina",E70="Trading/Payout",E70="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="B71" s="23">
@@ -5505,6 +5777,10 @@
         <f>IF(A71="","",YEAR(A71))</f>
         <v/>
       </c>
+      <c r="D71" s="23">
+        <f>IF(A71="","",IF(OR(E71="Nomina",E71="Trading/Payout",E71="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="B72" s="24">
@@ -5515,6 +5791,10 @@
         <f>IF(A72="","",YEAR(A72))</f>
         <v/>
       </c>
+      <c r="D72" s="24">
+        <f>IF(A72="","",IF(OR(E72="Nomina",E72="Trading/Payout",E72="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="B73" s="23">
@@ -5525,6 +5805,10 @@
         <f>IF(A73="","",YEAR(A73))</f>
         <v/>
       </c>
+      <c r="D73" s="23">
+        <f>IF(A73="","",IF(OR(E73="Nomina",E73="Trading/Payout",E73="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="B74" s="24">
@@ -5535,6 +5819,10 @@
         <f>IF(A74="","",YEAR(A74))</f>
         <v/>
       </c>
+      <c r="D74" s="24">
+        <f>IF(A74="","",IF(OR(E74="Nomina",E74="Trading/Payout",E74="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="B75" s="23">
@@ -5545,6 +5833,10 @@
         <f>IF(A75="","",YEAR(A75))</f>
         <v/>
       </c>
+      <c r="D75" s="23">
+        <f>IF(A75="","",IF(OR(E75="Nomina",E75="Trading/Payout",E75="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="B76" s="24">
@@ -5555,6 +5847,10 @@
         <f>IF(A76="","",YEAR(A76))</f>
         <v/>
       </c>
+      <c r="D76" s="24">
+        <f>IF(A76="","",IF(OR(E76="Nomina",E76="Trading/Payout",E76="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="B77" s="23">
@@ -5565,6 +5861,10 @@
         <f>IF(A77="","",YEAR(A77))</f>
         <v/>
       </c>
+      <c r="D77" s="23">
+        <f>IF(A77="","",IF(OR(E77="Nomina",E77="Trading/Payout",E77="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="B78" s="24">
@@ -5575,6 +5875,10 @@
         <f>IF(A78="","",YEAR(A78))</f>
         <v/>
       </c>
+      <c r="D78" s="24">
+        <f>IF(A78="","",IF(OR(E78="Nomina",E78="Trading/Payout",E78="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="B79" s="23">
@@ -5585,6 +5889,10 @@
         <f>IF(A79="","",YEAR(A79))</f>
         <v/>
       </c>
+      <c r="D79" s="23">
+        <f>IF(A79="","",IF(OR(E79="Nomina",E79="Trading/Payout",E79="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="B80" s="24">
@@ -5595,6 +5903,10 @@
         <f>IF(A80="","",YEAR(A80))</f>
         <v/>
       </c>
+      <c r="D80" s="24">
+        <f>IF(A80="","",IF(OR(E80="Nomina",E80="Trading/Payout",E80="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="B81" s="23">
@@ -5605,6 +5917,10 @@
         <f>IF(A81="","",YEAR(A81))</f>
         <v/>
       </c>
+      <c r="D81" s="23">
+        <f>IF(A81="","",IF(OR(E81="Nomina",E81="Trading/Payout",E81="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="B82" s="24">
@@ -5615,6 +5931,10 @@
         <f>IF(A82="","",YEAR(A82))</f>
         <v/>
       </c>
+      <c r="D82" s="24">
+        <f>IF(A82="","",IF(OR(E82="Nomina",E82="Trading/Payout",E82="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="B83" s="23">
@@ -5625,6 +5945,10 @@
         <f>IF(A83="","",YEAR(A83))</f>
         <v/>
       </c>
+      <c r="D83" s="23">
+        <f>IF(A83="","",IF(OR(E83="Nomina",E83="Trading/Payout",E83="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="B84" s="24">
@@ -5635,6 +5959,10 @@
         <f>IF(A84="","",YEAR(A84))</f>
         <v/>
       </c>
+      <c r="D84" s="24">
+        <f>IF(A84="","",IF(OR(E84="Nomina",E84="Trading/Payout",E84="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="B85" s="23">
@@ -5645,6 +5973,10 @@
         <f>IF(A85="","",YEAR(A85))</f>
         <v/>
       </c>
+      <c r="D85" s="23">
+        <f>IF(A85="","",IF(OR(E85="Nomina",E85="Trading/Payout",E85="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="B86" s="24">
@@ -5655,6 +5987,10 @@
         <f>IF(A86="","",YEAR(A86))</f>
         <v/>
       </c>
+      <c r="D86" s="24">
+        <f>IF(A86="","",IF(OR(E86="Nomina",E86="Trading/Payout",E86="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="B87" s="23">
@@ -5665,6 +6001,10 @@
         <f>IF(A87="","",YEAR(A87))</f>
         <v/>
       </c>
+      <c r="D87" s="23">
+        <f>IF(A87="","",IF(OR(E87="Nomina",E87="Trading/Payout",E87="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="B88" s="24">
@@ -5675,6 +6015,10 @@
         <f>IF(A88="","",YEAR(A88))</f>
         <v/>
       </c>
+      <c r="D88" s="24">
+        <f>IF(A88="","",IF(OR(E88="Nomina",E88="Trading/Payout",E88="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="B89" s="23">
@@ -5685,6 +6029,10 @@
         <f>IF(A89="","",YEAR(A89))</f>
         <v/>
       </c>
+      <c r="D89" s="23">
+        <f>IF(A89="","",IF(OR(E89="Nomina",E89="Trading/Payout",E89="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="B90" s="24">
@@ -5695,6 +6043,10 @@
         <f>IF(A90="","",YEAR(A90))</f>
         <v/>
       </c>
+      <c r="D90" s="24">
+        <f>IF(A90="","",IF(OR(E90="Nomina",E90="Trading/Payout",E90="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="B91" s="23">
@@ -5705,6 +6057,10 @@
         <f>IF(A91="","",YEAR(A91))</f>
         <v/>
       </c>
+      <c r="D91" s="23">
+        <f>IF(A91="","",IF(OR(E91="Nomina",E91="Trading/Payout",E91="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="B92" s="24">
@@ -5715,6 +6071,10 @@
         <f>IF(A92="","",YEAR(A92))</f>
         <v/>
       </c>
+      <c r="D92" s="24">
+        <f>IF(A92="","",IF(OR(E92="Nomina",E92="Trading/Payout",E92="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="B93" s="23">
@@ -5725,6 +6085,10 @@
         <f>IF(A93="","",YEAR(A93))</f>
         <v/>
       </c>
+      <c r="D93" s="23">
+        <f>IF(A93="","",IF(OR(E93="Nomina",E93="Trading/Payout",E93="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="B94" s="24">
@@ -5735,6 +6099,10 @@
         <f>IF(A94="","",YEAR(A94))</f>
         <v/>
       </c>
+      <c r="D94" s="24">
+        <f>IF(A94="","",IF(OR(E94="Nomina",E94="Trading/Payout",E94="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="B95" s="23">
@@ -5745,6 +6113,10 @@
         <f>IF(A95="","",YEAR(A95))</f>
         <v/>
       </c>
+      <c r="D95" s="23">
+        <f>IF(A95="","",IF(OR(E95="Nomina",E95="Trading/Payout",E95="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="B96" s="24">
@@ -5755,6 +6127,10 @@
         <f>IF(A96="","",YEAR(A96))</f>
         <v/>
       </c>
+      <c r="D96" s="24">
+        <f>IF(A96="","",IF(OR(E96="Nomina",E96="Trading/Payout",E96="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="B97" s="23">
@@ -5765,6 +6141,10 @@
         <f>IF(A97="","",YEAR(A97))</f>
         <v/>
       </c>
+      <c r="D97" s="23">
+        <f>IF(A97="","",IF(OR(E97="Nomina",E97="Trading/Payout",E97="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="B98" s="24">
@@ -5775,6 +6155,10 @@
         <f>IF(A98="","",YEAR(A98))</f>
         <v/>
       </c>
+      <c r="D98" s="24">
+        <f>IF(A98="","",IF(OR(E98="Nomina",E98="Trading/Payout",E98="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="B99" s="23">
@@ -5785,6 +6169,10 @@
         <f>IF(A99="","",YEAR(A99))</f>
         <v/>
       </c>
+      <c r="D99" s="23">
+        <f>IF(A99="","",IF(OR(E99="Nomina",E99="Trading/Payout",E99="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="B100" s="24">
@@ -5795,6 +6183,10 @@
         <f>IF(A100="","",YEAR(A100))</f>
         <v/>
       </c>
+      <c r="D100" s="24">
+        <f>IF(A100="","",IF(OR(E100="Nomina",E100="Trading/Payout",E100="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="B101" s="23">
@@ -5805,6 +6197,10 @@
         <f>IF(A101="","",YEAR(A101))</f>
         <v/>
       </c>
+      <c r="D101" s="23">
+        <f>IF(A101="","",IF(OR(E101="Nomina",E101="Trading/Payout",E101="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="B102" s="24">
@@ -5815,6 +6211,10 @@
         <f>IF(A102="","",YEAR(A102))</f>
         <v/>
       </c>
+      <c r="D102" s="24">
+        <f>IF(A102="","",IF(OR(E102="Nomina",E102="Trading/Payout",E102="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="103">
       <c r="B103" s="23">
@@ -5825,6 +6225,10 @@
         <f>IF(A103="","",YEAR(A103))</f>
         <v/>
       </c>
+      <c r="D103" s="23">
+        <f>IF(A103="","",IF(OR(E103="Nomina",E103="Trading/Payout",E103="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="104">
       <c r="B104" s="24">
@@ -5835,6 +6239,10 @@
         <f>IF(A104="","",YEAR(A104))</f>
         <v/>
       </c>
+      <c r="D104" s="24">
+        <f>IF(A104="","",IF(OR(E104="Nomina",E104="Trading/Payout",E104="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="105">
       <c r="B105" s="23">
@@ -5845,6 +6253,10 @@
         <f>IF(A105="","",YEAR(A105))</f>
         <v/>
       </c>
+      <c r="D105" s="23">
+        <f>IF(A105="","",IF(OR(E105="Nomina",E105="Trading/Payout",E105="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="106">
       <c r="B106" s="24">
@@ -5855,6 +6267,10 @@
         <f>IF(A106="","",YEAR(A106))</f>
         <v/>
       </c>
+      <c r="D106" s="24">
+        <f>IF(A106="","",IF(OR(E106="Nomina",E106="Trading/Payout",E106="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="107">
       <c r="B107" s="23">
@@ -5865,6 +6281,10 @@
         <f>IF(A107="","",YEAR(A107))</f>
         <v/>
       </c>
+      <c r="D107" s="23">
+        <f>IF(A107="","",IF(OR(E107="Nomina",E107="Trading/Payout",E107="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="108">
       <c r="B108" s="24">
@@ -5875,6 +6295,10 @@
         <f>IF(A108="","",YEAR(A108))</f>
         <v/>
       </c>
+      <c r="D108" s="24">
+        <f>IF(A108="","",IF(OR(E108="Nomina",E108="Trading/Payout",E108="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="109">
       <c r="B109" s="23">
@@ -5885,6 +6309,10 @@
         <f>IF(A109="","",YEAR(A109))</f>
         <v/>
       </c>
+      <c r="D109" s="23">
+        <f>IF(A109="","",IF(OR(E109="Nomina",E109="Trading/Payout",E109="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="110">
       <c r="B110" s="24">
@@ -5895,6 +6323,10 @@
         <f>IF(A110="","",YEAR(A110))</f>
         <v/>
       </c>
+      <c r="D110" s="24">
+        <f>IF(A110="","",IF(OR(E110="Nomina",E110="Trading/Payout",E110="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="111">
       <c r="B111" s="23">
@@ -5905,6 +6337,10 @@
         <f>IF(A111="","",YEAR(A111))</f>
         <v/>
       </c>
+      <c r="D111" s="23">
+        <f>IF(A111="","",IF(OR(E111="Nomina",E111="Trading/Payout",E111="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="112">
       <c r="B112" s="24">
@@ -5915,6 +6351,10 @@
         <f>IF(A112="","",YEAR(A112))</f>
         <v/>
       </c>
+      <c r="D112" s="24">
+        <f>IF(A112="","",IF(OR(E112="Nomina",E112="Trading/Payout",E112="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="113">
       <c r="B113" s="23">
@@ -5925,6 +6365,10 @@
         <f>IF(A113="","",YEAR(A113))</f>
         <v/>
       </c>
+      <c r="D113" s="23">
+        <f>IF(A113="","",IF(OR(E113="Nomina",E113="Trading/Payout",E113="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="114">
       <c r="B114" s="24">
@@ -5935,6 +6379,10 @@
         <f>IF(A114="","",YEAR(A114))</f>
         <v/>
       </c>
+      <c r="D114" s="24">
+        <f>IF(A114="","",IF(OR(E114="Nomina",E114="Trading/Payout",E114="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="115">
       <c r="B115" s="23">
@@ -5945,6 +6393,10 @@
         <f>IF(A115="","",YEAR(A115))</f>
         <v/>
       </c>
+      <c r="D115" s="23">
+        <f>IF(A115="","",IF(OR(E115="Nomina",E115="Trading/Payout",E115="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="116">
       <c r="B116" s="24">
@@ -5955,6 +6407,10 @@
         <f>IF(A116="","",YEAR(A116))</f>
         <v/>
       </c>
+      <c r="D116" s="24">
+        <f>IF(A116="","",IF(OR(E116="Nomina",E116="Trading/Payout",E116="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="117">
       <c r="B117" s="23">
@@ -5965,6 +6421,10 @@
         <f>IF(A117="","",YEAR(A117))</f>
         <v/>
       </c>
+      <c r="D117" s="23">
+        <f>IF(A117="","",IF(OR(E117="Nomina",E117="Trading/Payout",E117="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="118">
       <c r="B118" s="24">
@@ -5975,6 +6435,10 @@
         <f>IF(A118="","",YEAR(A118))</f>
         <v/>
       </c>
+      <c r="D118" s="24">
+        <f>IF(A118="","",IF(OR(E118="Nomina",E118="Trading/Payout",E118="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="119">
       <c r="B119" s="23">
@@ -5985,6 +6449,10 @@
         <f>IF(A119="","",YEAR(A119))</f>
         <v/>
       </c>
+      <c r="D119" s="23">
+        <f>IF(A119="","",IF(OR(E119="Nomina",E119="Trading/Payout",E119="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="120">
       <c r="B120" s="24">
@@ -5995,6 +6463,10 @@
         <f>IF(A120="","",YEAR(A120))</f>
         <v/>
       </c>
+      <c r="D120" s="24">
+        <f>IF(A120="","",IF(OR(E120="Nomina",E120="Trading/Payout",E120="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="121">
       <c r="B121" s="23">
@@ -6005,6 +6477,10 @@
         <f>IF(A121="","",YEAR(A121))</f>
         <v/>
       </c>
+      <c r="D121" s="23">
+        <f>IF(A121="","",IF(OR(E121="Nomina",E121="Trading/Payout",E121="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="122">
       <c r="B122" s="24">
@@ -6015,6 +6491,10 @@
         <f>IF(A122="","",YEAR(A122))</f>
         <v/>
       </c>
+      <c r="D122" s="24">
+        <f>IF(A122="","",IF(OR(E122="Nomina",E122="Trading/Payout",E122="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="123">
       <c r="B123" s="23">
@@ -6025,6 +6505,10 @@
         <f>IF(A123="","",YEAR(A123))</f>
         <v/>
       </c>
+      <c r="D123" s="23">
+        <f>IF(A123="","",IF(OR(E123="Nomina",E123="Trading/Payout",E123="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="124">
       <c r="B124" s="24">
@@ -6035,6 +6519,10 @@
         <f>IF(A124="","",YEAR(A124))</f>
         <v/>
       </c>
+      <c r="D124" s="24">
+        <f>IF(A124="","",IF(OR(E124="Nomina",E124="Trading/Payout",E124="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="125">
       <c r="B125" s="23">
@@ -6045,6 +6533,10 @@
         <f>IF(A125="","",YEAR(A125))</f>
         <v/>
       </c>
+      <c r="D125" s="23">
+        <f>IF(A125="","",IF(OR(E125="Nomina",E125="Trading/Payout",E125="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="126">
       <c r="B126" s="24">
@@ -6055,6 +6547,10 @@
         <f>IF(A126="","",YEAR(A126))</f>
         <v/>
       </c>
+      <c r="D126" s="24">
+        <f>IF(A126="","",IF(OR(E126="Nomina",E126="Trading/Payout",E126="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="127">
       <c r="B127" s="23">
@@ -6065,6 +6561,10 @@
         <f>IF(A127="","",YEAR(A127))</f>
         <v/>
       </c>
+      <c r="D127" s="23">
+        <f>IF(A127="","",IF(OR(E127="Nomina",E127="Trading/Payout",E127="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="128">
       <c r="B128" s="24">
@@ -6075,6 +6575,10 @@
         <f>IF(A128="","",YEAR(A128))</f>
         <v/>
       </c>
+      <c r="D128" s="24">
+        <f>IF(A128="","",IF(OR(E128="Nomina",E128="Trading/Payout",E128="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="129">
       <c r="B129" s="23">
@@ -6085,6 +6589,10 @@
         <f>IF(A129="","",YEAR(A129))</f>
         <v/>
       </c>
+      <c r="D129" s="23">
+        <f>IF(A129="","",IF(OR(E129="Nomina",E129="Trading/Payout",E129="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="130">
       <c r="B130" s="24">
@@ -6095,6 +6603,10 @@
         <f>IF(A130="","",YEAR(A130))</f>
         <v/>
       </c>
+      <c r="D130" s="24">
+        <f>IF(A130="","",IF(OR(E130="Nomina",E130="Trading/Payout",E130="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="131">
       <c r="B131" s="23">
@@ -6105,6 +6617,10 @@
         <f>IF(A131="","",YEAR(A131))</f>
         <v/>
       </c>
+      <c r="D131" s="23">
+        <f>IF(A131="","",IF(OR(E131="Nomina",E131="Trading/Payout",E131="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="132">
       <c r="B132" s="24">
@@ -6115,6 +6631,10 @@
         <f>IF(A132="","",YEAR(A132))</f>
         <v/>
       </c>
+      <c r="D132" s="24">
+        <f>IF(A132="","",IF(OR(E132="Nomina",E132="Trading/Payout",E132="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="133">
       <c r="B133" s="23">
@@ -6125,6 +6645,10 @@
         <f>IF(A133="","",YEAR(A133))</f>
         <v/>
       </c>
+      <c r="D133" s="23">
+        <f>IF(A133="","",IF(OR(E133="Nomina",E133="Trading/Payout",E133="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="134">
       <c r="B134" s="24">
@@ -6135,6 +6659,10 @@
         <f>IF(A134="","",YEAR(A134))</f>
         <v/>
       </c>
+      <c r="D134" s="24">
+        <f>IF(A134="","",IF(OR(E134="Nomina",E134="Trading/Payout",E134="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="135">
       <c r="B135" s="23">
@@ -6145,6 +6673,10 @@
         <f>IF(A135="","",YEAR(A135))</f>
         <v/>
       </c>
+      <c r="D135" s="23">
+        <f>IF(A135="","",IF(OR(E135="Nomina",E135="Trading/Payout",E135="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="136">
       <c r="B136" s="24">
@@ -6155,6 +6687,10 @@
         <f>IF(A136="","",YEAR(A136))</f>
         <v/>
       </c>
+      <c r="D136" s="24">
+        <f>IF(A136="","",IF(OR(E136="Nomina",E136="Trading/Payout",E136="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="137">
       <c r="B137" s="23">
@@ -6165,6 +6701,10 @@
         <f>IF(A137="","",YEAR(A137))</f>
         <v/>
       </c>
+      <c r="D137" s="23">
+        <f>IF(A137="","",IF(OR(E137="Nomina",E137="Trading/Payout",E137="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="138">
       <c r="B138" s="24">
@@ -6175,6 +6715,10 @@
         <f>IF(A138="","",YEAR(A138))</f>
         <v/>
       </c>
+      <c r="D138" s="24">
+        <f>IF(A138="","",IF(OR(E138="Nomina",E138="Trading/Payout",E138="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="139">
       <c r="B139" s="23">
@@ -6185,6 +6729,10 @@
         <f>IF(A139="","",YEAR(A139))</f>
         <v/>
       </c>
+      <c r="D139" s="23">
+        <f>IF(A139="","",IF(OR(E139="Nomina",E139="Trading/Payout",E139="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="140">
       <c r="B140" s="24">
@@ -6195,6 +6743,10 @@
         <f>IF(A140="","",YEAR(A140))</f>
         <v/>
       </c>
+      <c r="D140" s="24">
+        <f>IF(A140="","",IF(OR(E140="Nomina",E140="Trading/Payout",E140="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="141">
       <c r="B141" s="23">
@@ -6205,6 +6757,10 @@
         <f>IF(A141="","",YEAR(A141))</f>
         <v/>
       </c>
+      <c r="D141" s="23">
+        <f>IF(A141="","",IF(OR(E141="Nomina",E141="Trading/Payout",E141="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="142">
       <c r="B142" s="24">
@@ -6215,6 +6771,10 @@
         <f>IF(A142="","",YEAR(A142))</f>
         <v/>
       </c>
+      <c r="D142" s="24">
+        <f>IF(A142="","",IF(OR(E142="Nomina",E142="Trading/Payout",E142="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="143">
       <c r="B143" s="23">
@@ -6225,6 +6785,10 @@
         <f>IF(A143="","",YEAR(A143))</f>
         <v/>
       </c>
+      <c r="D143" s="23">
+        <f>IF(A143="","",IF(OR(E143="Nomina",E143="Trading/Payout",E143="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="144">
       <c r="B144" s="24">
@@ -6235,6 +6799,10 @@
         <f>IF(A144="","",YEAR(A144))</f>
         <v/>
       </c>
+      <c r="D144" s="24">
+        <f>IF(A144="","",IF(OR(E144="Nomina",E144="Trading/Payout",E144="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="145">
       <c r="B145" s="23">
@@ -6245,6 +6813,10 @@
         <f>IF(A145="","",YEAR(A145))</f>
         <v/>
       </c>
+      <c r="D145" s="23">
+        <f>IF(A145="","",IF(OR(E145="Nomina",E145="Trading/Payout",E145="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="146">
       <c r="B146" s="24">
@@ -6255,6 +6827,10 @@
         <f>IF(A146="","",YEAR(A146))</f>
         <v/>
       </c>
+      <c r="D146" s="24">
+        <f>IF(A146="","",IF(OR(E146="Nomina",E146="Trading/Payout",E146="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="147">
       <c r="B147" s="23">
@@ -6265,6 +6841,10 @@
         <f>IF(A147="","",YEAR(A147))</f>
         <v/>
       </c>
+      <c r="D147" s="23">
+        <f>IF(A147="","",IF(OR(E147="Nomina",E147="Trading/Payout",E147="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="148">
       <c r="B148" s="24">
@@ -6275,6 +6855,10 @@
         <f>IF(A148="","",YEAR(A148))</f>
         <v/>
       </c>
+      <c r="D148" s="24">
+        <f>IF(A148="","",IF(OR(E148="Nomina",E148="Trading/Payout",E148="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="149">
       <c r="B149" s="23">
@@ -6285,6 +6869,10 @@
         <f>IF(A149="","",YEAR(A149))</f>
         <v/>
       </c>
+      <c r="D149" s="23">
+        <f>IF(A149="","",IF(OR(E149="Nomina",E149="Trading/Payout",E149="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="150">
       <c r="B150" s="24">
@@ -6295,6 +6883,10 @@
         <f>IF(A150="","",YEAR(A150))</f>
         <v/>
       </c>
+      <c r="D150" s="24">
+        <f>IF(A150="","",IF(OR(E150="Nomina",E150="Trading/Payout",E150="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="151">
       <c r="B151" s="23">
@@ -6305,6 +6897,10 @@
         <f>IF(A151="","",YEAR(A151))</f>
         <v/>
       </c>
+      <c r="D151" s="23">
+        <f>IF(A151="","",IF(OR(E151="Nomina",E151="Trading/Payout",E151="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="152">
       <c r="B152" s="24">
@@ -6315,6 +6911,10 @@
         <f>IF(A152="","",YEAR(A152))</f>
         <v/>
       </c>
+      <c r="D152" s="24">
+        <f>IF(A152="","",IF(OR(E152="Nomina",E152="Trading/Payout",E152="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="153">
       <c r="B153" s="23">
@@ -6325,6 +6925,10 @@
         <f>IF(A153="","",YEAR(A153))</f>
         <v/>
       </c>
+      <c r="D153" s="23">
+        <f>IF(A153="","",IF(OR(E153="Nomina",E153="Trading/Payout",E153="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="154">
       <c r="B154" s="24">
@@ -6335,6 +6939,10 @@
         <f>IF(A154="","",YEAR(A154))</f>
         <v/>
       </c>
+      <c r="D154" s="24">
+        <f>IF(A154="","",IF(OR(E154="Nomina",E154="Trading/Payout",E154="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="155">
       <c r="B155" s="23">
@@ -6345,6 +6953,10 @@
         <f>IF(A155="","",YEAR(A155))</f>
         <v/>
       </c>
+      <c r="D155" s="23">
+        <f>IF(A155="","",IF(OR(E155="Nomina",E155="Trading/Payout",E155="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="156">
       <c r="B156" s="24">
@@ -6355,6 +6967,10 @@
         <f>IF(A156="","",YEAR(A156))</f>
         <v/>
       </c>
+      <c r="D156" s="24">
+        <f>IF(A156="","",IF(OR(E156="Nomina",E156="Trading/Payout",E156="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="157">
       <c r="B157" s="23">
@@ -6365,6 +6981,10 @@
         <f>IF(A157="","",YEAR(A157))</f>
         <v/>
       </c>
+      <c r="D157" s="23">
+        <f>IF(A157="","",IF(OR(E157="Nomina",E157="Trading/Payout",E157="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="158">
       <c r="B158" s="24">
@@ -6375,6 +6995,10 @@
         <f>IF(A158="","",YEAR(A158))</f>
         <v/>
       </c>
+      <c r="D158" s="24">
+        <f>IF(A158="","",IF(OR(E158="Nomina",E158="Trading/Payout",E158="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="159">
       <c r="B159" s="23">
@@ -6385,6 +7009,10 @@
         <f>IF(A159="","",YEAR(A159))</f>
         <v/>
       </c>
+      <c r="D159" s="23">
+        <f>IF(A159="","",IF(OR(E159="Nomina",E159="Trading/Payout",E159="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="160">
       <c r="B160" s="24">
@@ -6395,6 +7023,10 @@
         <f>IF(A160="","",YEAR(A160))</f>
         <v/>
       </c>
+      <c r="D160" s="24">
+        <f>IF(A160="","",IF(OR(E160="Nomina",E160="Trading/Payout",E160="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="161">
       <c r="B161" s="23">
@@ -6405,6 +7037,10 @@
         <f>IF(A161="","",YEAR(A161))</f>
         <v/>
       </c>
+      <c r="D161" s="23">
+        <f>IF(A161="","",IF(OR(E161="Nomina",E161="Trading/Payout",E161="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="162">
       <c r="B162" s="24">
@@ -6415,6 +7051,10 @@
         <f>IF(A162="","",YEAR(A162))</f>
         <v/>
       </c>
+      <c r="D162" s="24">
+        <f>IF(A162="","",IF(OR(E162="Nomina",E162="Trading/Payout",E162="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="163">
       <c r="B163" s="23">
@@ -6425,6 +7065,10 @@
         <f>IF(A163="","",YEAR(A163))</f>
         <v/>
       </c>
+      <c r="D163" s="23">
+        <f>IF(A163="","",IF(OR(E163="Nomina",E163="Trading/Payout",E163="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="164">
       <c r="B164" s="24">
@@ -6435,6 +7079,10 @@
         <f>IF(A164="","",YEAR(A164))</f>
         <v/>
       </c>
+      <c r="D164" s="24">
+        <f>IF(A164="","",IF(OR(E164="Nomina",E164="Trading/Payout",E164="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="165">
       <c r="B165" s="23">
@@ -6445,6 +7093,10 @@
         <f>IF(A165="","",YEAR(A165))</f>
         <v/>
       </c>
+      <c r="D165" s="23">
+        <f>IF(A165="","",IF(OR(E165="Nomina",E165="Trading/Payout",E165="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="166">
       <c r="B166" s="24">
@@ -6455,6 +7107,10 @@
         <f>IF(A166="","",YEAR(A166))</f>
         <v/>
       </c>
+      <c r="D166" s="24">
+        <f>IF(A166="","",IF(OR(E166="Nomina",E166="Trading/Payout",E166="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="167">
       <c r="B167" s="23">
@@ -6465,6 +7121,10 @@
         <f>IF(A167="","",YEAR(A167))</f>
         <v/>
       </c>
+      <c r="D167" s="23">
+        <f>IF(A167="","",IF(OR(E167="Nomina",E167="Trading/Payout",E167="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="168">
       <c r="B168" s="24">
@@ -6475,6 +7135,10 @@
         <f>IF(A168="","",YEAR(A168))</f>
         <v/>
       </c>
+      <c r="D168" s="24">
+        <f>IF(A168="","",IF(OR(E168="Nomina",E168="Trading/Payout",E168="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="169">
       <c r="B169" s="23">
@@ -6485,6 +7149,10 @@
         <f>IF(A169="","",YEAR(A169))</f>
         <v/>
       </c>
+      <c r="D169" s="23">
+        <f>IF(A169="","",IF(OR(E169="Nomina",E169="Trading/Payout",E169="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="170">
       <c r="B170" s="24">
@@ -6495,6 +7163,10 @@
         <f>IF(A170="","",YEAR(A170))</f>
         <v/>
       </c>
+      <c r="D170" s="24">
+        <f>IF(A170="","",IF(OR(E170="Nomina",E170="Trading/Payout",E170="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="171">
       <c r="B171" s="23">
@@ -6505,6 +7177,10 @@
         <f>IF(A171="","",YEAR(A171))</f>
         <v/>
       </c>
+      <c r="D171" s="23">
+        <f>IF(A171="","",IF(OR(E171="Nomina",E171="Trading/Payout",E171="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="172">
       <c r="B172" s="24">
@@ -6515,6 +7191,10 @@
         <f>IF(A172="","",YEAR(A172))</f>
         <v/>
       </c>
+      <c r="D172" s="24">
+        <f>IF(A172="","",IF(OR(E172="Nomina",E172="Trading/Payout",E172="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="173">
       <c r="B173" s="23">
@@ -6525,6 +7205,10 @@
         <f>IF(A173="","",YEAR(A173))</f>
         <v/>
       </c>
+      <c r="D173" s="23">
+        <f>IF(A173="","",IF(OR(E173="Nomina",E173="Trading/Payout",E173="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="174">
       <c r="B174" s="24">
@@ -6535,6 +7219,10 @@
         <f>IF(A174="","",YEAR(A174))</f>
         <v/>
       </c>
+      <c r="D174" s="24">
+        <f>IF(A174="","",IF(OR(E174="Nomina",E174="Trading/Payout",E174="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="175">
       <c r="B175" s="23">
@@ -6545,6 +7233,10 @@
         <f>IF(A175="","",YEAR(A175))</f>
         <v/>
       </c>
+      <c r="D175" s="23">
+        <f>IF(A175="","",IF(OR(E175="Nomina",E175="Trading/Payout",E175="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="176">
       <c r="B176" s="24">
@@ -6555,6 +7247,10 @@
         <f>IF(A176="","",YEAR(A176))</f>
         <v/>
       </c>
+      <c r="D176" s="24">
+        <f>IF(A176="","",IF(OR(E176="Nomina",E176="Trading/Payout",E176="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="177">
       <c r="B177" s="23">
@@ -6565,6 +7261,10 @@
         <f>IF(A177="","",YEAR(A177))</f>
         <v/>
       </c>
+      <c r="D177" s="23">
+        <f>IF(A177="","",IF(OR(E177="Nomina",E177="Trading/Payout",E177="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="178">
       <c r="B178" s="24">
@@ -6575,6 +7275,10 @@
         <f>IF(A178="","",YEAR(A178))</f>
         <v/>
       </c>
+      <c r="D178" s="24">
+        <f>IF(A178="","",IF(OR(E178="Nomina",E178="Trading/Payout",E178="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="179">
       <c r="B179" s="23">
@@ -6585,6 +7289,10 @@
         <f>IF(A179="","",YEAR(A179))</f>
         <v/>
       </c>
+      <c r="D179" s="23">
+        <f>IF(A179="","",IF(OR(E179="Nomina",E179="Trading/Payout",E179="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="180">
       <c r="B180" s="24">
@@ -6595,6 +7303,10 @@
         <f>IF(A180="","",YEAR(A180))</f>
         <v/>
       </c>
+      <c r="D180" s="24">
+        <f>IF(A180="","",IF(OR(E180="Nomina",E180="Trading/Payout",E180="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="181">
       <c r="B181" s="23">
@@ -6605,6 +7317,10 @@
         <f>IF(A181="","",YEAR(A181))</f>
         <v/>
       </c>
+      <c r="D181" s="23">
+        <f>IF(A181="","",IF(OR(E181="Nomina",E181="Trading/Payout",E181="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="182">
       <c r="B182" s="24">
@@ -6615,6 +7331,10 @@
         <f>IF(A182="","",YEAR(A182))</f>
         <v/>
       </c>
+      <c r="D182" s="24">
+        <f>IF(A182="","",IF(OR(E182="Nomina",E182="Trading/Payout",E182="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="183">
       <c r="B183" s="23">
@@ -6625,6 +7345,10 @@
         <f>IF(A183="","",YEAR(A183))</f>
         <v/>
       </c>
+      <c r="D183" s="23">
+        <f>IF(A183="","",IF(OR(E183="Nomina",E183="Trading/Payout",E183="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="184">
       <c r="B184" s="24">
@@ -6635,6 +7359,10 @@
         <f>IF(A184="","",YEAR(A184))</f>
         <v/>
       </c>
+      <c r="D184" s="24">
+        <f>IF(A184="","",IF(OR(E184="Nomina",E184="Trading/Payout",E184="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="185">
       <c r="B185" s="23">
@@ -6645,6 +7373,10 @@
         <f>IF(A185="","",YEAR(A185))</f>
         <v/>
       </c>
+      <c r="D185" s="23">
+        <f>IF(A185="","",IF(OR(E185="Nomina",E185="Trading/Payout",E185="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="186">
       <c r="B186" s="24">
@@ -6655,6 +7387,10 @@
         <f>IF(A186="","",YEAR(A186))</f>
         <v/>
       </c>
+      <c r="D186" s="24">
+        <f>IF(A186="","",IF(OR(E186="Nomina",E186="Trading/Payout",E186="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="187">
       <c r="B187" s="23">
@@ -6665,6 +7401,10 @@
         <f>IF(A187="","",YEAR(A187))</f>
         <v/>
       </c>
+      <c r="D187" s="23">
+        <f>IF(A187="","",IF(OR(E187="Nomina",E187="Trading/Payout",E187="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="188">
       <c r="B188" s="24">
@@ -6675,6 +7415,10 @@
         <f>IF(A188="","",YEAR(A188))</f>
         <v/>
       </c>
+      <c r="D188" s="24">
+        <f>IF(A188="","",IF(OR(E188="Nomina",E188="Trading/Payout",E188="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="189">
       <c r="B189" s="23">
@@ -6685,6 +7429,10 @@
         <f>IF(A189="","",YEAR(A189))</f>
         <v/>
       </c>
+      <c r="D189" s="23">
+        <f>IF(A189="","",IF(OR(E189="Nomina",E189="Trading/Payout",E189="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="190">
       <c r="B190" s="24">
@@ -6695,6 +7443,10 @@
         <f>IF(A190="","",YEAR(A190))</f>
         <v/>
       </c>
+      <c r="D190" s="24">
+        <f>IF(A190="","",IF(OR(E190="Nomina",E190="Trading/Payout",E190="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="191">
       <c r="B191" s="23">
@@ -6705,6 +7457,10 @@
         <f>IF(A191="","",YEAR(A191))</f>
         <v/>
       </c>
+      <c r="D191" s="23">
+        <f>IF(A191="","",IF(OR(E191="Nomina",E191="Trading/Payout",E191="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="192">
       <c r="B192" s="24">
@@ -6715,6 +7471,10 @@
         <f>IF(A192="","",YEAR(A192))</f>
         <v/>
       </c>
+      <c r="D192" s="24">
+        <f>IF(A192="","",IF(OR(E192="Nomina",E192="Trading/Payout",E192="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="193">
       <c r="B193" s="23">
@@ -6725,6 +7485,10 @@
         <f>IF(A193="","",YEAR(A193))</f>
         <v/>
       </c>
+      <c r="D193" s="23">
+        <f>IF(A193="","",IF(OR(E193="Nomina",E193="Trading/Payout",E193="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="194">
       <c r="B194" s="24">
@@ -6735,6 +7499,10 @@
         <f>IF(A194="","",YEAR(A194))</f>
         <v/>
       </c>
+      <c r="D194" s="24">
+        <f>IF(A194="","",IF(OR(E194="Nomina",E194="Trading/Payout",E194="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="195">
       <c r="B195" s="23">
@@ -6745,6 +7513,10 @@
         <f>IF(A195="","",YEAR(A195))</f>
         <v/>
       </c>
+      <c r="D195" s="23">
+        <f>IF(A195="","",IF(OR(E195="Nomina",E195="Trading/Payout",E195="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="196">
       <c r="B196" s="24">
@@ -6755,6 +7527,10 @@
         <f>IF(A196="","",YEAR(A196))</f>
         <v/>
       </c>
+      <c r="D196" s="24">
+        <f>IF(A196="","",IF(OR(E196="Nomina",E196="Trading/Payout",E196="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="197">
       <c r="B197" s="23">
@@ -6765,6 +7541,10 @@
         <f>IF(A197="","",YEAR(A197))</f>
         <v/>
       </c>
+      <c r="D197" s="23">
+        <f>IF(A197="","",IF(OR(E197="Nomina",E197="Trading/Payout",E197="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="198">
       <c r="B198" s="24">
@@ -6775,6 +7555,10 @@
         <f>IF(A198="","",YEAR(A198))</f>
         <v/>
       </c>
+      <c r="D198" s="24">
+        <f>IF(A198="","",IF(OR(E198="Nomina",E198="Trading/Payout",E198="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="199">
       <c r="B199" s="23">
@@ -6785,6 +7569,10 @@
         <f>IF(A199="","",YEAR(A199))</f>
         <v/>
       </c>
+      <c r="D199" s="23">
+        <f>IF(A199="","",IF(OR(E199="Nomina",E199="Trading/Payout",E199="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="200">
       <c r="B200" s="24">
@@ -6795,6 +7583,10 @@
         <f>IF(A200="","",YEAR(A200))</f>
         <v/>
       </c>
+      <c r="D200" s="24">
+        <f>IF(A200="","",IF(OR(E200="Nomina",E200="Trading/Payout",E200="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="201">
       <c r="B201" s="23">
@@ -6805,6 +7597,10 @@
         <f>IF(A201="","",YEAR(A201))</f>
         <v/>
       </c>
+      <c r="D201" s="23">
+        <f>IF(A201="","",IF(OR(E201="Nomina",E201="Trading/Payout",E201="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="202">
       <c r="B202" s="24">
@@ -6815,6 +7611,10 @@
         <f>IF(A202="","",YEAR(A202))</f>
         <v/>
       </c>
+      <c r="D202" s="24">
+        <f>IF(A202="","",IF(OR(E202="Nomina",E202="Trading/Payout",E202="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="203">
       <c r="B203" s="23">
@@ -6825,6 +7625,10 @@
         <f>IF(A203="","",YEAR(A203))</f>
         <v/>
       </c>
+      <c r="D203" s="23">
+        <f>IF(A203="","",IF(OR(E203="Nomina",E203="Trading/Payout",E203="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="204">
       <c r="B204" s="24">
@@ -6835,6 +7639,10 @@
         <f>IF(A204="","",YEAR(A204))</f>
         <v/>
       </c>
+      <c r="D204" s="24">
+        <f>IF(A204="","",IF(OR(E204="Nomina",E204="Trading/Payout",E204="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="205">
       <c r="B205" s="23">
@@ -6845,6 +7653,10 @@
         <f>IF(A205="","",YEAR(A205))</f>
         <v/>
       </c>
+      <c r="D205" s="23">
+        <f>IF(A205="","",IF(OR(E205="Nomina",E205="Trading/Payout",E205="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="206">
       <c r="B206" s="24">
@@ -6855,6 +7667,10 @@
         <f>IF(A206="","",YEAR(A206))</f>
         <v/>
       </c>
+      <c r="D206" s="24">
+        <f>IF(A206="","",IF(OR(E206="Nomina",E206="Trading/Payout",E206="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="207">
       <c r="B207" s="23">
@@ -6865,6 +7681,10 @@
         <f>IF(A207="","",YEAR(A207))</f>
         <v/>
       </c>
+      <c r="D207" s="23">
+        <f>IF(A207="","",IF(OR(E207="Nomina",E207="Trading/Payout",E207="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="208">
       <c r="B208" s="24">
@@ -6875,6 +7695,10 @@
         <f>IF(A208="","",YEAR(A208))</f>
         <v/>
       </c>
+      <c r="D208" s="24">
+        <f>IF(A208="","",IF(OR(E208="Nomina",E208="Trading/Payout",E208="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="209">
       <c r="B209" s="23">
@@ -6885,6 +7709,10 @@
         <f>IF(A209="","",YEAR(A209))</f>
         <v/>
       </c>
+      <c r="D209" s="23">
+        <f>IF(A209="","",IF(OR(E209="Nomina",E209="Trading/Payout",E209="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="210">
       <c r="B210" s="24">
@@ -6895,6 +7723,10 @@
         <f>IF(A210="","",YEAR(A210))</f>
         <v/>
       </c>
+      <c r="D210" s="24">
+        <f>IF(A210="","",IF(OR(E210="Nomina",E210="Trading/Payout",E210="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="211">
       <c r="B211" s="23">
@@ -6905,6 +7737,10 @@
         <f>IF(A211="","",YEAR(A211))</f>
         <v/>
       </c>
+      <c r="D211" s="23">
+        <f>IF(A211="","",IF(OR(E211="Nomina",E211="Trading/Payout",E211="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="212">
       <c r="B212" s="24">
@@ -6915,6 +7751,10 @@
         <f>IF(A212="","",YEAR(A212))</f>
         <v/>
       </c>
+      <c r="D212" s="24">
+        <f>IF(A212="","",IF(OR(E212="Nomina",E212="Trading/Payout",E212="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="213">
       <c r="B213" s="23">
@@ -6925,6 +7765,10 @@
         <f>IF(A213="","",YEAR(A213))</f>
         <v/>
       </c>
+      <c r="D213" s="23">
+        <f>IF(A213="","",IF(OR(E213="Nomina",E213="Trading/Payout",E213="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="214">
       <c r="B214" s="24">
@@ -6935,6 +7779,10 @@
         <f>IF(A214="","",YEAR(A214))</f>
         <v/>
       </c>
+      <c r="D214" s="24">
+        <f>IF(A214="","",IF(OR(E214="Nomina",E214="Trading/Payout",E214="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="215">
       <c r="B215" s="23">
@@ -6945,6 +7793,10 @@
         <f>IF(A215="","",YEAR(A215))</f>
         <v/>
       </c>
+      <c r="D215" s="23">
+        <f>IF(A215="","",IF(OR(E215="Nomina",E215="Trading/Payout",E215="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="216">
       <c r="B216" s="24">
@@ -6955,6 +7807,10 @@
         <f>IF(A216="","",YEAR(A216))</f>
         <v/>
       </c>
+      <c r="D216" s="24">
+        <f>IF(A216="","",IF(OR(E216="Nomina",E216="Trading/Payout",E216="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="217">
       <c r="B217" s="23">
@@ -6965,6 +7821,10 @@
         <f>IF(A217="","",YEAR(A217))</f>
         <v/>
       </c>
+      <c r="D217" s="23">
+        <f>IF(A217="","",IF(OR(E217="Nomina",E217="Trading/Payout",E217="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="218">
       <c r="B218" s="24">
@@ -6975,6 +7835,10 @@
         <f>IF(A218="","",YEAR(A218))</f>
         <v/>
       </c>
+      <c r="D218" s="24">
+        <f>IF(A218="","",IF(OR(E218="Nomina",E218="Trading/Payout",E218="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="219">
       <c r="B219" s="23">
@@ -6985,6 +7849,10 @@
         <f>IF(A219="","",YEAR(A219))</f>
         <v/>
       </c>
+      <c r="D219" s="23">
+        <f>IF(A219="","",IF(OR(E219="Nomina",E219="Trading/Payout",E219="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="220">
       <c r="B220" s="24">
@@ -6995,6 +7863,10 @@
         <f>IF(A220="","",YEAR(A220))</f>
         <v/>
       </c>
+      <c r="D220" s="24">
+        <f>IF(A220="","",IF(OR(E220="Nomina",E220="Trading/Payout",E220="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="221">
       <c r="B221" s="23">
@@ -7005,6 +7877,10 @@
         <f>IF(A221="","",YEAR(A221))</f>
         <v/>
       </c>
+      <c r="D221" s="23">
+        <f>IF(A221="","",IF(OR(E221="Nomina",E221="Trading/Payout",E221="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="222">
       <c r="B222" s="24">
@@ -7015,6 +7891,10 @@
         <f>IF(A222="","",YEAR(A222))</f>
         <v/>
       </c>
+      <c r="D222" s="24">
+        <f>IF(A222="","",IF(OR(E222="Nomina",E222="Trading/Payout",E222="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="223">
       <c r="B223" s="23">
@@ -7025,6 +7905,10 @@
         <f>IF(A223="","",YEAR(A223))</f>
         <v/>
       </c>
+      <c r="D223" s="23">
+        <f>IF(A223="","",IF(OR(E223="Nomina",E223="Trading/Payout",E223="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="224">
       <c r="B224" s="24">
@@ -7035,6 +7919,10 @@
         <f>IF(A224="","",YEAR(A224))</f>
         <v/>
       </c>
+      <c r="D224" s="24">
+        <f>IF(A224="","",IF(OR(E224="Nomina",E224="Trading/Payout",E224="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="225">
       <c r="B225" s="23">
@@ -7045,6 +7933,10 @@
         <f>IF(A225="","",YEAR(A225))</f>
         <v/>
       </c>
+      <c r="D225" s="23">
+        <f>IF(A225="","",IF(OR(E225="Nomina",E225="Trading/Payout",E225="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="226">
       <c r="B226" s="24">
@@ -7055,6 +7947,10 @@
         <f>IF(A226="","",YEAR(A226))</f>
         <v/>
       </c>
+      <c r="D226" s="24">
+        <f>IF(A226="","",IF(OR(E226="Nomina",E226="Trading/Payout",E226="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="227">
       <c r="B227" s="23">
@@ -7065,6 +7961,10 @@
         <f>IF(A227="","",YEAR(A227))</f>
         <v/>
       </c>
+      <c r="D227" s="23">
+        <f>IF(A227="","",IF(OR(E227="Nomina",E227="Trading/Payout",E227="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="228">
       <c r="B228" s="24">
@@ -7075,6 +7975,10 @@
         <f>IF(A228="","",YEAR(A228))</f>
         <v/>
       </c>
+      <c r="D228" s="24">
+        <f>IF(A228="","",IF(OR(E228="Nomina",E228="Trading/Payout",E228="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="229">
       <c r="B229" s="23">
@@ -7085,6 +7989,10 @@
         <f>IF(A229="","",YEAR(A229))</f>
         <v/>
       </c>
+      <c r="D229" s="23">
+        <f>IF(A229="","",IF(OR(E229="Nomina",E229="Trading/Payout",E229="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="230">
       <c r="B230" s="24">
@@ -7095,6 +8003,10 @@
         <f>IF(A230="","",YEAR(A230))</f>
         <v/>
       </c>
+      <c r="D230" s="24">
+        <f>IF(A230="","",IF(OR(E230="Nomina",E230="Trading/Payout",E230="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="231">
       <c r="B231" s="23">
@@ -7105,6 +8017,10 @@
         <f>IF(A231="","",YEAR(A231))</f>
         <v/>
       </c>
+      <c r="D231" s="23">
+        <f>IF(A231="","",IF(OR(E231="Nomina",E231="Trading/Payout",E231="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="232">
       <c r="B232" s="24">
@@ -7115,6 +8031,10 @@
         <f>IF(A232="","",YEAR(A232))</f>
         <v/>
       </c>
+      <c r="D232" s="24">
+        <f>IF(A232="","",IF(OR(E232="Nomina",E232="Trading/Payout",E232="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="233">
       <c r="B233" s="23">
@@ -7125,6 +8045,10 @@
         <f>IF(A233="","",YEAR(A233))</f>
         <v/>
       </c>
+      <c r="D233" s="23">
+        <f>IF(A233="","",IF(OR(E233="Nomina",E233="Trading/Payout",E233="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="234">
       <c r="B234" s="24">
@@ -7135,6 +8059,10 @@
         <f>IF(A234="","",YEAR(A234))</f>
         <v/>
       </c>
+      <c r="D234" s="24">
+        <f>IF(A234="","",IF(OR(E234="Nomina",E234="Trading/Payout",E234="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="235">
       <c r="B235" s="23">
@@ -7145,6 +8073,10 @@
         <f>IF(A235="","",YEAR(A235))</f>
         <v/>
       </c>
+      <c r="D235" s="23">
+        <f>IF(A235="","",IF(OR(E235="Nomina",E235="Trading/Payout",E235="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="236">
       <c r="B236" s="24">
@@ -7155,6 +8087,10 @@
         <f>IF(A236="","",YEAR(A236))</f>
         <v/>
       </c>
+      <c r="D236" s="24">
+        <f>IF(A236="","",IF(OR(E236="Nomina",E236="Trading/Payout",E236="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="237">
       <c r="B237" s="23">
@@ -7165,6 +8101,10 @@
         <f>IF(A237="","",YEAR(A237))</f>
         <v/>
       </c>
+      <c r="D237" s="23">
+        <f>IF(A237="","",IF(OR(E237="Nomina",E237="Trading/Payout",E237="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="238">
       <c r="B238" s="24">
@@ -7175,6 +8115,10 @@
         <f>IF(A238="","",YEAR(A238))</f>
         <v/>
       </c>
+      <c r="D238" s="24">
+        <f>IF(A238="","",IF(OR(E238="Nomina",E238="Trading/Payout",E238="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="239">
       <c r="B239" s="23">
@@ -7185,6 +8129,10 @@
         <f>IF(A239="","",YEAR(A239))</f>
         <v/>
       </c>
+      <c r="D239" s="23">
+        <f>IF(A239="","",IF(OR(E239="Nomina",E239="Trading/Payout",E239="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="240">
       <c r="B240" s="24">
@@ -7195,6 +8143,10 @@
         <f>IF(A240="","",YEAR(A240))</f>
         <v/>
       </c>
+      <c r="D240" s="24">
+        <f>IF(A240="","",IF(OR(E240="Nomina",E240="Trading/Payout",E240="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="241">
       <c r="B241" s="23">
@@ -7205,6 +8157,10 @@
         <f>IF(A241="","",YEAR(A241))</f>
         <v/>
       </c>
+      <c r="D241" s="23">
+        <f>IF(A241="","",IF(OR(E241="Nomina",E241="Trading/Payout",E241="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="242">
       <c r="B242" s="24">
@@ -7215,6 +8171,10 @@
         <f>IF(A242="","",YEAR(A242))</f>
         <v/>
       </c>
+      <c r="D242" s="24">
+        <f>IF(A242="","",IF(OR(E242="Nomina",E242="Trading/Payout",E242="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="243">
       <c r="B243" s="23">
@@ -7225,6 +8185,10 @@
         <f>IF(A243="","",YEAR(A243))</f>
         <v/>
       </c>
+      <c r="D243" s="23">
+        <f>IF(A243="","",IF(OR(E243="Nomina",E243="Trading/Payout",E243="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="244">
       <c r="B244" s="24">
@@ -7235,6 +8199,10 @@
         <f>IF(A244="","",YEAR(A244))</f>
         <v/>
       </c>
+      <c r="D244" s="24">
+        <f>IF(A244="","",IF(OR(E244="Nomina",E244="Trading/Payout",E244="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="245">
       <c r="B245" s="23">
@@ -7245,6 +8213,10 @@
         <f>IF(A245="","",YEAR(A245))</f>
         <v/>
       </c>
+      <c r="D245" s="23">
+        <f>IF(A245="","",IF(OR(E245="Nomina",E245="Trading/Payout",E245="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="246">
       <c r="B246" s="24">
@@ -7255,6 +8227,10 @@
         <f>IF(A246="","",YEAR(A246))</f>
         <v/>
       </c>
+      <c r="D246" s="24">
+        <f>IF(A246="","",IF(OR(E246="Nomina",E246="Trading/Payout",E246="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="247">
       <c r="B247" s="23">
@@ -7265,6 +8241,10 @@
         <f>IF(A247="","",YEAR(A247))</f>
         <v/>
       </c>
+      <c r="D247" s="23">
+        <f>IF(A247="","",IF(OR(E247="Nomina",E247="Trading/Payout",E247="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="248">
       <c r="B248" s="24">
@@ -7275,6 +8255,10 @@
         <f>IF(A248="","",YEAR(A248))</f>
         <v/>
       </c>
+      <c r="D248" s="24">
+        <f>IF(A248="","",IF(OR(E248="Nomina",E248="Trading/Payout",E248="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="249">
       <c r="B249" s="23">
@@ -7285,6 +8269,10 @@
         <f>IF(A249="","",YEAR(A249))</f>
         <v/>
       </c>
+      <c r="D249" s="23">
+        <f>IF(A249="","",IF(OR(E249="Nomina",E249="Trading/Payout",E249="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="250">
       <c r="B250" s="24">
@@ -7295,6 +8283,10 @@
         <f>IF(A250="","",YEAR(A250))</f>
         <v/>
       </c>
+      <c r="D250" s="24">
+        <f>IF(A250="","",IF(OR(E250="Nomina",E250="Trading/Payout",E250="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="251">
       <c r="B251" s="23">
@@ -7305,6 +8297,10 @@
         <f>IF(A251="","",YEAR(A251))</f>
         <v/>
       </c>
+      <c r="D251" s="23">
+        <f>IF(A251="","",IF(OR(E251="Nomina",E251="Trading/Payout",E251="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="252">
       <c r="B252" s="24">
@@ -7315,6 +8311,10 @@
         <f>IF(A252="","",YEAR(A252))</f>
         <v/>
       </c>
+      <c r="D252" s="24">
+        <f>IF(A252="","",IF(OR(E252="Nomina",E252="Trading/Payout",E252="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="253">
       <c r="B253" s="23">
@@ -7325,6 +8325,10 @@
         <f>IF(A253="","",YEAR(A253))</f>
         <v/>
       </c>
+      <c r="D253" s="23">
+        <f>IF(A253="","",IF(OR(E253="Nomina",E253="Trading/Payout",E253="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="254">
       <c r="B254" s="24">
@@ -7335,6 +8339,10 @@
         <f>IF(A254="","",YEAR(A254))</f>
         <v/>
       </c>
+      <c r="D254" s="24">
+        <f>IF(A254="","",IF(OR(E254="Nomina",E254="Trading/Payout",E254="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="255">
       <c r="B255" s="23">
@@ -7345,6 +8353,10 @@
         <f>IF(A255="","",YEAR(A255))</f>
         <v/>
       </c>
+      <c r="D255" s="23">
+        <f>IF(A255="","",IF(OR(E255="Nomina",E255="Trading/Payout",E255="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="256">
       <c r="B256" s="24">
@@ -7355,6 +8367,10 @@
         <f>IF(A256="","",YEAR(A256))</f>
         <v/>
       </c>
+      <c r="D256" s="24">
+        <f>IF(A256="","",IF(OR(E256="Nomina",E256="Trading/Payout",E256="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="257">
       <c r="B257" s="23">
@@ -7365,6 +8381,10 @@
         <f>IF(A257="","",YEAR(A257))</f>
         <v/>
       </c>
+      <c r="D257" s="23">
+        <f>IF(A257="","",IF(OR(E257="Nomina",E257="Trading/Payout",E257="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="258">
       <c r="B258" s="24">
@@ -7375,6 +8395,10 @@
         <f>IF(A258="","",YEAR(A258))</f>
         <v/>
       </c>
+      <c r="D258" s="24">
+        <f>IF(A258="","",IF(OR(E258="Nomina",E258="Trading/Payout",E258="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="259">
       <c r="B259" s="23">
@@ -7385,6 +8409,10 @@
         <f>IF(A259="","",YEAR(A259))</f>
         <v/>
       </c>
+      <c r="D259" s="23">
+        <f>IF(A259="","",IF(OR(E259="Nomina",E259="Trading/Payout",E259="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="260">
       <c r="B260" s="24">
@@ -7395,6 +8423,10 @@
         <f>IF(A260="","",YEAR(A260))</f>
         <v/>
       </c>
+      <c r="D260" s="24">
+        <f>IF(A260="","",IF(OR(E260="Nomina",E260="Trading/Payout",E260="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="261">
       <c r="B261" s="23">
@@ -7405,6 +8437,10 @@
         <f>IF(A261="","",YEAR(A261))</f>
         <v/>
       </c>
+      <c r="D261" s="23">
+        <f>IF(A261="","",IF(OR(E261="Nomina",E261="Trading/Payout",E261="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="262">
       <c r="B262" s="24">
@@ -7415,6 +8451,10 @@
         <f>IF(A262="","",YEAR(A262))</f>
         <v/>
       </c>
+      <c r="D262" s="24">
+        <f>IF(A262="","",IF(OR(E262="Nomina",E262="Trading/Payout",E262="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="263">
       <c r="B263" s="23">
@@ -7425,6 +8465,10 @@
         <f>IF(A263="","",YEAR(A263))</f>
         <v/>
       </c>
+      <c r="D263" s="23">
+        <f>IF(A263="","",IF(OR(E263="Nomina",E263="Trading/Payout",E263="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="264">
       <c r="B264" s="24">
@@ -7435,6 +8479,10 @@
         <f>IF(A264="","",YEAR(A264))</f>
         <v/>
       </c>
+      <c r="D264" s="24">
+        <f>IF(A264="","",IF(OR(E264="Nomina",E264="Trading/Payout",E264="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="265">
       <c r="B265" s="23">
@@ -7445,6 +8493,10 @@
         <f>IF(A265="","",YEAR(A265))</f>
         <v/>
       </c>
+      <c r="D265" s="23">
+        <f>IF(A265="","",IF(OR(E265="Nomina",E265="Trading/Payout",E265="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="266">
       <c r="B266" s="24">
@@ -7455,6 +8507,10 @@
         <f>IF(A266="","",YEAR(A266))</f>
         <v/>
       </c>
+      <c r="D266" s="24">
+        <f>IF(A266="","",IF(OR(E266="Nomina",E266="Trading/Payout",E266="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="267">
       <c r="B267" s="23">
@@ -7465,6 +8521,10 @@
         <f>IF(A267="","",YEAR(A267))</f>
         <v/>
       </c>
+      <c r="D267" s="23">
+        <f>IF(A267="","",IF(OR(E267="Nomina",E267="Trading/Payout",E267="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="268">
       <c r="B268" s="24">
@@ -7475,6 +8535,10 @@
         <f>IF(A268="","",YEAR(A268))</f>
         <v/>
       </c>
+      <c r="D268" s="24">
+        <f>IF(A268="","",IF(OR(E268="Nomina",E268="Trading/Payout",E268="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="269">
       <c r="B269" s="23">
@@ -7485,6 +8549,10 @@
         <f>IF(A269="","",YEAR(A269))</f>
         <v/>
       </c>
+      <c r="D269" s="23">
+        <f>IF(A269="","",IF(OR(E269="Nomina",E269="Trading/Payout",E269="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="270">
       <c r="B270" s="24">
@@ -7495,6 +8563,10 @@
         <f>IF(A270="","",YEAR(A270))</f>
         <v/>
       </c>
+      <c r="D270" s="24">
+        <f>IF(A270="","",IF(OR(E270="Nomina",E270="Trading/Payout",E270="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="271">
       <c r="B271" s="23">
@@ -7505,6 +8577,10 @@
         <f>IF(A271="","",YEAR(A271))</f>
         <v/>
       </c>
+      <c r="D271" s="23">
+        <f>IF(A271="","",IF(OR(E271="Nomina",E271="Trading/Payout",E271="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="272">
       <c r="B272" s="24">
@@ -7515,6 +8591,10 @@
         <f>IF(A272="","",YEAR(A272))</f>
         <v/>
       </c>
+      <c r="D272" s="24">
+        <f>IF(A272="","",IF(OR(E272="Nomina",E272="Trading/Payout",E272="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="273">
       <c r="B273" s="23">
@@ -7525,6 +8605,10 @@
         <f>IF(A273="","",YEAR(A273))</f>
         <v/>
       </c>
+      <c r="D273" s="23">
+        <f>IF(A273="","",IF(OR(E273="Nomina",E273="Trading/Payout",E273="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="274">
       <c r="B274" s="24">
@@ -7535,6 +8619,10 @@
         <f>IF(A274="","",YEAR(A274))</f>
         <v/>
       </c>
+      <c r="D274" s="24">
+        <f>IF(A274="","",IF(OR(E274="Nomina",E274="Trading/Payout",E274="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="275">
       <c r="B275" s="23">
@@ -7545,6 +8633,10 @@
         <f>IF(A275="","",YEAR(A275))</f>
         <v/>
       </c>
+      <c r="D275" s="23">
+        <f>IF(A275="","",IF(OR(E275="Nomina",E275="Trading/Payout",E275="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="276">
       <c r="B276" s="24">
@@ -7555,6 +8647,10 @@
         <f>IF(A276="","",YEAR(A276))</f>
         <v/>
       </c>
+      <c r="D276" s="24">
+        <f>IF(A276="","",IF(OR(E276="Nomina",E276="Trading/Payout",E276="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="277">
       <c r="B277" s="23">
@@ -7565,6 +8661,10 @@
         <f>IF(A277="","",YEAR(A277))</f>
         <v/>
       </c>
+      <c r="D277" s="23">
+        <f>IF(A277="","",IF(OR(E277="Nomina",E277="Trading/Payout",E277="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="278">
       <c r="B278" s="24">
@@ -7575,6 +8675,10 @@
         <f>IF(A278="","",YEAR(A278))</f>
         <v/>
       </c>
+      <c r="D278" s="24">
+        <f>IF(A278="","",IF(OR(E278="Nomina",E278="Trading/Payout",E278="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="279">
       <c r="B279" s="23">
@@ -7585,6 +8689,10 @@
         <f>IF(A279="","",YEAR(A279))</f>
         <v/>
       </c>
+      <c r="D279" s="23">
+        <f>IF(A279="","",IF(OR(E279="Nomina",E279="Trading/Payout",E279="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="280">
       <c r="B280" s="24">
@@ -7595,6 +8703,10 @@
         <f>IF(A280="","",YEAR(A280))</f>
         <v/>
       </c>
+      <c r="D280" s="24">
+        <f>IF(A280="","",IF(OR(E280="Nomina",E280="Trading/Payout",E280="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="281">
       <c r="B281" s="23">
@@ -7605,6 +8717,10 @@
         <f>IF(A281="","",YEAR(A281))</f>
         <v/>
       </c>
+      <c r="D281" s="23">
+        <f>IF(A281="","",IF(OR(E281="Nomina",E281="Trading/Payout",E281="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="282">
       <c r="B282" s="24">
@@ -7615,6 +8731,10 @@
         <f>IF(A282="","",YEAR(A282))</f>
         <v/>
       </c>
+      <c r="D282" s="24">
+        <f>IF(A282="","",IF(OR(E282="Nomina",E282="Trading/Payout",E282="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="283">
       <c r="B283" s="23">
@@ -7625,6 +8745,10 @@
         <f>IF(A283="","",YEAR(A283))</f>
         <v/>
       </c>
+      <c r="D283" s="23">
+        <f>IF(A283="","",IF(OR(E283="Nomina",E283="Trading/Payout",E283="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="284">
       <c r="B284" s="24">
@@ -7635,6 +8759,10 @@
         <f>IF(A284="","",YEAR(A284))</f>
         <v/>
       </c>
+      <c r="D284" s="24">
+        <f>IF(A284="","",IF(OR(E284="Nomina",E284="Trading/Payout",E284="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="285">
       <c r="B285" s="23">
@@ -7645,6 +8773,10 @@
         <f>IF(A285="","",YEAR(A285))</f>
         <v/>
       </c>
+      <c r="D285" s="23">
+        <f>IF(A285="","",IF(OR(E285="Nomina",E285="Trading/Payout",E285="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="286">
       <c r="B286" s="24">
@@ -7655,6 +8787,10 @@
         <f>IF(A286="","",YEAR(A286))</f>
         <v/>
       </c>
+      <c r="D286" s="24">
+        <f>IF(A286="","",IF(OR(E286="Nomina",E286="Trading/Payout",E286="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="287">
       <c r="B287" s="23">
@@ -7665,6 +8801,10 @@
         <f>IF(A287="","",YEAR(A287))</f>
         <v/>
       </c>
+      <c r="D287" s="23">
+        <f>IF(A287="","",IF(OR(E287="Nomina",E287="Trading/Payout",E287="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="288">
       <c r="B288" s="24">
@@ -7675,6 +8815,10 @@
         <f>IF(A288="","",YEAR(A288))</f>
         <v/>
       </c>
+      <c r="D288" s="24">
+        <f>IF(A288="","",IF(OR(E288="Nomina",E288="Trading/Payout",E288="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="289">
       <c r="B289" s="23">
@@ -7685,6 +8829,10 @@
         <f>IF(A289="","",YEAR(A289))</f>
         <v/>
       </c>
+      <c r="D289" s="23">
+        <f>IF(A289="","",IF(OR(E289="Nomina",E289="Trading/Payout",E289="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="290">
       <c r="B290" s="24">
@@ -7695,6 +8843,10 @@
         <f>IF(A290="","",YEAR(A290))</f>
         <v/>
       </c>
+      <c r="D290" s="24">
+        <f>IF(A290="","",IF(OR(E290="Nomina",E290="Trading/Payout",E290="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="291">
       <c r="B291" s="23">
@@ -7705,6 +8857,10 @@
         <f>IF(A291="","",YEAR(A291))</f>
         <v/>
       </c>
+      <c r="D291" s="23">
+        <f>IF(A291="","",IF(OR(E291="Nomina",E291="Trading/Payout",E291="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="292">
       <c r="B292" s="24">
@@ -7715,6 +8871,10 @@
         <f>IF(A292="","",YEAR(A292))</f>
         <v/>
       </c>
+      <c r="D292" s="24">
+        <f>IF(A292="","",IF(OR(E292="Nomina",E292="Trading/Payout",E292="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="293">
       <c r="B293" s="23">
@@ -7725,6 +8885,10 @@
         <f>IF(A293="","",YEAR(A293))</f>
         <v/>
       </c>
+      <c r="D293" s="23">
+        <f>IF(A293="","",IF(OR(E293="Nomina",E293="Trading/Payout",E293="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="294">
       <c r="B294" s="24">
@@ -7735,6 +8899,10 @@
         <f>IF(A294="","",YEAR(A294))</f>
         <v/>
       </c>
+      <c r="D294" s="24">
+        <f>IF(A294="","",IF(OR(E294="Nomina",E294="Trading/Payout",E294="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="295">
       <c r="B295" s="23">
@@ -7745,6 +8913,10 @@
         <f>IF(A295="","",YEAR(A295))</f>
         <v/>
       </c>
+      <c r="D295" s="23">
+        <f>IF(A295="","",IF(OR(E295="Nomina",E295="Trading/Payout",E295="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="296">
       <c r="B296" s="24">
@@ -7755,6 +8927,10 @@
         <f>IF(A296="","",YEAR(A296))</f>
         <v/>
       </c>
+      <c r="D296" s="24">
+        <f>IF(A296="","",IF(OR(E296="Nomina",E296="Trading/Payout",E296="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="297">
       <c r="B297" s="23">
@@ -7765,6 +8941,10 @@
         <f>IF(A297="","",YEAR(A297))</f>
         <v/>
       </c>
+      <c r="D297" s="23">
+        <f>IF(A297="","",IF(OR(E297="Nomina",E297="Trading/Payout",E297="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="298">
       <c r="B298" s="24">
@@ -7775,6 +8955,10 @@
         <f>IF(A298="","",YEAR(A298))</f>
         <v/>
       </c>
+      <c r="D298" s="24">
+        <f>IF(A298="","",IF(OR(E298="Nomina",E298="Trading/Payout",E298="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="299">
       <c r="B299" s="23">
@@ -7785,6 +8969,10 @@
         <f>IF(A299="","",YEAR(A299))</f>
         <v/>
       </c>
+      <c r="D299" s="23">
+        <f>IF(A299="","",IF(OR(E299="Nomina",E299="Trading/Payout",E299="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
     </row>
     <row r="300">
       <c r="B300" s="24">
@@ -7793,6 +8981,10 @@
       </c>
       <c r="C300" s="24">
         <f>IF(A300="","",YEAR(A300))</f>
+        <v/>
+      </c>
+      <c r="D300" s="24">
+        <f>IF(A300="","",IF(OR(E300="Nomina",E300="Trading/Payout",E300="Otro ingreso"),"Ingreso","Gasto"))</f>
         <v/>
       </c>
     </row>
@@ -7801,10 +8993,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
-  <dataValidations count="3">
-    <dataValidation sqref="D3:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Ingreso,Gasto"</formula1>
-    </dataValidation>
+  <dataValidations count="2">
     <dataValidation sqref="E3:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>ListaCategorias</formula1>
     </dataValidation>
@@ -7824,7 +9013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -8288,390 +9477,398 @@
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="7" t="inlineStr">
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>&gt;&gt;&gt; Las celdas DORADAS son editables: cambia el limite mensual de cada categoria &lt;&lt;&lt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
         <is>
           <t>Categoria / Concepto</t>
         </is>
       </c>
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>Presupuestado</t>
-        </is>
-      </c>
-      <c r="C39" s="7" t="inlineStr">
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Limite Mensual (edita doradas)</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
         <is>
           <t>Gastado Real (mes)</t>
         </is>
       </c>
-      <c r="D39" s="7" t="inlineStr">
+      <c r="D40" s="7" t="inlineStr">
         <is>
           <t>Diferencia</t>
         </is>
       </c>
-      <c r="E39" s="7" t="inlineStr">
+      <c r="E40" s="7" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="9" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr">
         <is>
           <t>Vivienda/Alquiler</t>
         </is>
       </c>
-      <c r="B40" s="17">
+      <c r="B41" s="17">
         <f>C8</f>
         <v/>
       </c>
-      <c r="C40" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Vivienda/Alquiler")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
-        <v/>
-      </c>
-      <c r="D40" s="17">
-        <f>B40-C40</f>
-        <v/>
-      </c>
-      <c r="E40" s="24">
-        <f>IF(B40=0,"Sin limite",IF(C40&lt;=B40,"OK","EXCEDIDO"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="C41" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Vivienda/Alquiler")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D41" s="17">
+        <f>B41-C41</f>
+        <v/>
+      </c>
+      <c r="E41" s="24">
+        <f>IF(B41=0,"Sin limite",IF(C41&lt;=B41*0.8,"OK",IF(C41&lt;=B41,"AVISO","EXCEDIDO")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>Coche/Transporte</t>
         </is>
       </c>
-      <c r="B41" s="19">
+      <c r="B42" s="19">
         <f>C9</f>
         <v/>
       </c>
-      <c r="C41" s="19">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Coche/Transporte")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
-        <v/>
-      </c>
-      <c r="D41" s="19">
-        <f>B41-C41</f>
-        <v/>
-      </c>
-      <c r="E41" s="23">
-        <f>IF(B41=0,"Sin limite",IF(C41&lt;=B41,"OK","EXCEDIDO"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="9" t="inlineStr">
+      <c r="C42" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Coche/Transporte")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D42" s="19">
+        <f>B42-C42</f>
+        <v/>
+      </c>
+      <c r="E42" s="23">
+        <f>IF(B42=0,"Sin limite",IF(C42&lt;=B42*0.8,"OK",IF(C42&lt;=B42,"AVISO","EXCEDIDO")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
         <is>
           <t>Gasolina</t>
         </is>
       </c>
-      <c r="B42" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="C42" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Gasolina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
-        <v/>
-      </c>
-      <c r="D42" s="17">
-        <f>B42-C42</f>
-        <v/>
-      </c>
-      <c r="E42" s="24">
-        <f>IF(B42=0,"Sin limite",IF(C42&lt;=B42,"OK","EXCEDIDO"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="B43" s="25" t="n">
+        <v>80</v>
+      </c>
+      <c r="C43" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Gasolina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D43" s="17">
+        <f>B43-C43</f>
+        <v/>
+      </c>
+      <c r="E43" s="24">
+        <f>IF(B43=0,"Sin limite",IF(C43&lt;=B43*0.8,"OK",IF(C43&lt;=B43,"AVISO","EXCEDIDO")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>Supermercado</t>
         </is>
       </c>
-      <c r="B43" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C43" s="19">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
-        <v/>
-      </c>
-      <c r="D43" s="19">
-        <f>B43-C43</f>
-        <v/>
-      </c>
-      <c r="E43" s="23">
-        <f>IF(B43=0,"Sin limite",IF(C43&lt;=B43,"OK","EXCEDIDO"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="9" t="inlineStr">
+      <c r="B44" s="25" t="n">
+        <v>200</v>
+      </c>
+      <c r="C44" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D44" s="19">
+        <f>B44-C44</f>
+        <v/>
+      </c>
+      <c r="E44" s="23">
+        <f>IF(B44=0,"Sin limite",IF(C44&lt;=B44*0.8,"OK",IF(C44&lt;=B44,"AVISO","EXCEDIDO")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
         <is>
           <t>Restaurante</t>
         </is>
       </c>
-      <c r="B44" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="C44" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
-        <v/>
-      </c>
-      <c r="D44" s="17">
-        <f>B44-C44</f>
-        <v/>
-      </c>
-      <c r="E44" s="24">
-        <f>IF(B44=0,"Sin limite",IF(C44&lt;=B44,"OK","EXCEDIDO"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="B45" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="C45" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D45" s="17">
+        <f>B45-C45</f>
+        <v/>
+      </c>
+      <c r="E45" s="24">
+        <f>IF(B45=0,"Sin limite",IF(C45&lt;=B45*0.8,"OK",IF(C45&lt;=B45,"AVISO","EXCEDIDO")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>Cafeteria/Bar</t>
         </is>
       </c>
-      <c r="B45" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C45" s="19">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
-        <v/>
-      </c>
-      <c r="D45" s="19">
-        <f>B45-C45</f>
-        <v/>
-      </c>
-      <c r="E45" s="23">
-        <f>IF(B45=0,"Sin limite",IF(C45&lt;=B45,"OK","EXCEDIDO"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="9" t="inlineStr">
+      <c r="B46" s="25" t="n">
+        <v>40</v>
+      </c>
+      <c r="C46" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D46" s="19">
+        <f>B46-C46</f>
+        <v/>
+      </c>
+      <c r="E46" s="23">
+        <f>IF(B46=0,"Sin limite",IF(C46&lt;=B46*0.8,"OK",IF(C46&lt;=B46,"AVISO","EXCEDIDO")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
         <is>
           <t>Ocio/Entretenimiento</t>
         </is>
       </c>
-      <c r="B46" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="C46" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
-        <v/>
-      </c>
-      <c r="D46" s="17">
-        <f>B46-C46</f>
-        <v/>
-      </c>
-      <c r="E46" s="24">
-        <f>IF(B46=0,"Sin limite",IF(C46&lt;=B46,"OK","EXCEDIDO"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="B47" s="25" t="n">
+        <v>80</v>
+      </c>
+      <c r="C47" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D47" s="17">
+        <f>B47-C47</f>
+        <v/>
+      </c>
+      <c r="E47" s="24">
+        <f>IF(B47=0,"Sin limite",IF(C47&lt;=B47*0.8,"OK",IF(C47&lt;=B47,"AVISO","EXCEDIDO")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>Ropa/Calzado</t>
         </is>
       </c>
-      <c r="B47" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C47" s="19">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
-        <v/>
-      </c>
-      <c r="D47" s="19">
-        <f>B47-C47</f>
-        <v/>
-      </c>
-      <c r="E47" s="23">
-        <f>IF(B47=0,"Sin limite",IF(C47&lt;=B47,"OK","EXCEDIDO"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="9" t="inlineStr">
+      <c r="B48" s="25" t="n">
+        <v>60</v>
+      </c>
+      <c r="C48" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D48" s="19">
+        <f>B48-C48</f>
+        <v/>
+      </c>
+      <c r="E48" s="23">
+        <f>IF(B48=0,"Sin limite",IF(C48&lt;=B48*0.8,"OK",IF(C48&lt;=B48,"AVISO","EXCEDIDO")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="9" t="inlineStr">
         <is>
           <t>Farmacia/Salud</t>
         </is>
       </c>
-      <c r="B48" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="C48" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
-        <v/>
-      </c>
-      <c r="D48" s="17">
-        <f>B48-C48</f>
-        <v/>
-      </c>
-      <c r="E48" s="24">
-        <f>IF(B48=0,"Sin limite",IF(C48&lt;=B48,"OK","EXCEDIDO"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="B49" s="25" t="n">
+        <v>40</v>
+      </c>
+      <c r="C49" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D49" s="17">
+        <f>B49-C49</f>
+        <v/>
+      </c>
+      <c r="E49" s="24">
+        <f>IF(B49=0,"Sin limite",IF(C49&lt;=B49*0.8,"OK",IF(C49&lt;=B49,"AVISO","EXCEDIDO")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>Deporte/Gimnasio</t>
         </is>
       </c>
-      <c r="B49" s="19">
+      <c r="B50" s="19">
         <f>C10</f>
         <v/>
       </c>
-      <c r="C49" s="19">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Deporte/Gimnasio")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
-        <v/>
-      </c>
-      <c r="D49" s="19">
-        <f>B49-C49</f>
-        <v/>
-      </c>
-      <c r="E49" s="23">
-        <f>IF(B49=0,"Sin limite",IF(C49&lt;=B49,"OK","EXCEDIDO"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="9" t="inlineStr">
+      <c r="C50" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Deporte/Gimnasio")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D50" s="19">
+        <f>B50-C50</f>
+        <v/>
+      </c>
+      <c r="E50" s="23">
+        <f>IF(B50=0,"Sin limite",IF(C50&lt;=B50*0.8,"OK",IF(C50&lt;=B50,"AVISO","EXCEDIDO")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="9" t="inlineStr">
         <is>
           <t>Formacion/Suscripciones</t>
         </is>
       </c>
-      <c r="B50" s="17">
+      <c r="B51" s="17">
         <f>C11</f>
         <v/>
       </c>
-      <c r="C50" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
-        <v/>
-      </c>
-      <c r="D50" s="17">
-        <f>B50-C50</f>
-        <v/>
-      </c>
-      <c r="E50" s="24">
-        <f>IF(B50=0,"Sin limite",IF(C50&lt;=B50,"OK","EXCEDIDO"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="C51" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D51" s="17">
+        <f>B51-C51</f>
+        <v/>
+      </c>
+      <c r="E51" s="24">
+        <f>IF(B51=0,"Sin limite",IF(C51&lt;=B51*0.8,"OK",IF(C51&lt;=B51,"AVISO","EXCEDIDO")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>Ahorro</t>
         </is>
       </c>
-      <c r="B51" s="19">
+      <c r="B52" s="19">
         <f>B18</f>
         <v/>
       </c>
-      <c r="C51" s="19">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
-        <v/>
-      </c>
-      <c r="D51" s="19">
-        <f>B51-C51</f>
-        <v/>
-      </c>
-      <c r="E51" s="23">
-        <f>IF(B51=0,"Sin limite",IF(C51&lt;=B51,"OK","EXCEDIDO"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="9" t="inlineStr">
+      <c r="C52" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D52" s="19">
+        <f>B52-C52</f>
+        <v/>
+      </c>
+      <c r="E52" s="23">
+        <f>IF(B52=0,"Sin limite",IF(C52&lt;=B52*0.8,"OK",IF(C52&lt;=B52,"AVISO","EXCEDIDO")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="9" t="inlineStr">
         <is>
           <t>Bankroll</t>
         </is>
       </c>
-      <c r="B52" s="17">
+      <c r="B53" s="17">
         <f>B17</f>
         <v/>
       </c>
-      <c r="C52" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
-        <v/>
-      </c>
-      <c r="D52" s="17">
-        <f>B52-C52</f>
-        <v/>
-      </c>
-      <c r="E52" s="24">
-        <f>IF(B52=0,"Sin limite",IF(C52&lt;=B52,"OK","EXCEDIDO"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="inlineStr">
+      <c r="C53" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D53" s="17">
+        <f>B53-C53</f>
+        <v/>
+      </c>
+      <c r="E53" s="24">
+        <f>IF(B53=0,"Sin limite",IF(C53&lt;=B53*0.8,"OK",IF(C53&lt;=B53,"AVISO","EXCEDIDO")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>Otros</t>
         </is>
       </c>
-      <c r="B53" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C53" s="19">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
-        <v/>
-      </c>
-      <c r="D53" s="19">
-        <f>B53-C53</f>
-        <v/>
-      </c>
-      <c r="E53" s="23">
-        <f>IF(B53=0,"Sin limite",IF(C53&lt;=B53,"OK","EXCEDIDO"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="4" t="inlineStr">
+      <c r="B54" s="25" t="n">
+        <v>50</v>
+      </c>
+      <c r="C54" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D54" s="19">
+        <f>B54-C54</f>
+        <v/>
+      </c>
+      <c r="E54" s="23">
+        <f>IF(B54=0,"Sin limite",IF(C54&lt;=B54*0.8,"OK",IF(C54&lt;=B54,"AVISO","EXCEDIDO")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
         <is>
           <t>TOTAL GASTOS REALES DEL MES</t>
         </is>
       </c>
-      <c r="C54" s="21">
+      <c r="C55" s="21">
         <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
-      <c r="D54" s="21">
-        <f>$D$3-C54</f>
-        <v/>
-      </c>
-      <c r="E54" s="4">
-        <f>IF(C54&lt;=$D$3,"Dentro del ingreso","SUPERA EL INGRESO")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="9" t="inlineStr">
-        <is>
-          <t>TOTAL INGRESOS REGISTRADOS DEL MES</t>
-        </is>
-      </c>
-      <c r="C55" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+      <c r="D55" s="21">
+        <f>$D$3-C55</f>
+        <v/>
+      </c>
+      <c r="E55" s="4">
+        <f>IF(C55&lt;=$D$3,"Dentro del ingreso","SUPERA EL INGRESO")</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="9" t="inlineStr">
         <is>
+          <t>TOTAL INGRESOS REGISTRADOS DEL MES</t>
+        </is>
+      </c>
+      <c r="C56" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="9" t="inlineStr">
+        <is>
           <t>% del presupuesto ejecutado (gastos / ingreso)</t>
         </is>
       </c>
-      <c r="C56" s="18">
-        <f>IFERROR(C54/$D$3,0)</f>
+      <c r="C57" s="18">
+        <f>IFERROR(C55/$D$3,0)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
+    <mergeCell ref="A39:E39"/>
     <mergeCell ref="B35:E35"/>
     <mergeCell ref="A38:E38"/>
     <mergeCell ref="A14:F14"/>
@@ -8685,23 +9882,34 @@
     <mergeCell ref="A21:F21"/>
     <mergeCell ref="B36:E36"/>
   </mergeCells>
+  <conditionalFormatting sqref="A41:E54">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND($B41&gt;0,$C41&gt;$B41)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>AND($B41&gt;0,$C41&gt;$B41*0.8,$C41&lt;=$B41)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2">
+      <formula>AND($B41&gt;0,$C41&gt;0,$C41&lt;=$B41*0.8)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C28">
-    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
+    <cfRule type="cellIs" priority="4" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="lessThanOrEqual" dxfId="1">
+    <cfRule type="cellIs" priority="5" operator="lessThanOrEqual" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C29">
-    <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="6" operator="greaterThan" dxfId="3">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="between" dxfId="3">
+    <cfRule type="cellIs" priority="7" operator="between" dxfId="4">
       <formula>0.9</formula>
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="lessThanOrEqual" dxfId="4">
+    <cfRule type="cellIs" priority="8" operator="lessThanOrEqual" dxfId="5">
       <formula>0.9</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9186,10 +10394,10 @@
     <mergeCell ref="A502:E502"/>
   </mergeCells>
   <conditionalFormatting sqref="C3:C1000">
-    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="1">
+    <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9299,10 +10507,10 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <conditionalFormatting sqref="D3:D1000">
-    <cfRule type="expression" priority="1" dxfId="0">
+    <cfRule type="expression" priority="1" dxfId="2">
       <formula>D3="Cobrado"</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="5">
+    <cfRule type="expression" priority="2" dxfId="1">
       <formula>D3="Pendiente"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Selector de mes/año + formulas REGISTRO extendidas a fila 500
- PRESUPUESTO MENSUAL fila 5: selector B5 (mes 1-12) y E5 (año).
  Celda C5 muestra el nombre del mes/año seleccionado (ej. junio 2026).
  Validacion: B5 solo acepta numeros 1-12 con mensaje de error.
- Todas las formulas SUMPRODUCT del sistema filtran por B5/E5 en vez
  de MONTH(TODAY()). Cambiar B5=7 muestra julio sin tocar nada mas.
- REGISTRO DE MOVIMIENTOS: formulas Mes(auto)/Anio(auto)/Tipo(auto)
  extendidas de fila 300 a fila 500 (498 filas de datos disponibles).

https://claude.ai/code/session_01EdLrBe1U3fRxvoA6PYaJVC
</commit_message>
<xml_diff>
--- a/sistema_financiero.xlsx
+++ b/sistema_financiero.xlsx
@@ -30,7 +30,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">'GUIA DE USO'!$A$1:$J$42</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'DASHBOARD EJECUTIVO'!$A$1:$N$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'REGISTRO DE MOVIMIENTOS'!$A$2:$J$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'REGISTRO DE MOVIMIENTOS'!$A$1:$L$305</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'REGISTRO DE MOVIMIENTOS'!$A$1:$L$505</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'PRESUPUESTO MENSUAL'!$A$1:$H$62</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'CONTROL DE AHORRO'!$A$1:$H$19</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'CONTROL DE BANKROLL'!$A$1:$G$17</definedName>
@@ -271,7 +271,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -346,6 +346,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="21">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="21">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="21">
@@ -1322,6 +1325,13 @@
         <t>Cambia este valor cada mes. Todo el sistema se actualiza automaticamente.</t>
       </text>
     </comment>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>Cambia B5 (mes 1-12) y E5 (anio) para ver los datos de cualquier mes.
+Ejemplo: B5=7, E5=2026 muestra julio 2026.
+Todo el seguimiento y dashboard se actualizan solos.</t>
+      </text>
+    </comment>
     <comment ref="B17" authorId="0" shapeId="0">
       <text>
         <t>Importe fijo minimo para bankroll. Aumentalo en meses buenos.</t>
@@ -2252,7 +2262,7 @@
           <t>Meses cubiertos actualmente</t>
         </is>
       </c>
-      <c r="B10" s="30">
+      <c r="B10" s="31">
         <f>B9/1575</f>
         <v/>
       </c>
@@ -2809,7 +2819,7 @@
         </is>
       </c>
       <c r="B514" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="C514" s="18">
@@ -2832,7 +2842,7 @@
         </is>
       </c>
       <c r="B515" s="19">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="C515" s="20">
@@ -2855,7 +2865,7 @@
         </is>
       </c>
       <c r="B516" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="C516" s="18">
@@ -2878,7 +2888,7 @@
         </is>
       </c>
       <c r="B517" s="19">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="C517" s="20">
@@ -2901,7 +2911,7 @@
         </is>
       </c>
       <c r="B518" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="C518" s="18">
@@ -2924,7 +2934,7 @@
         </is>
       </c>
       <c r="B519" s="19">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Electronica/Amazon")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Electronica/Amazon")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="C519" s="20">
@@ -2947,7 +2957,7 @@
         </is>
       </c>
       <c r="B520" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="C520" s="18">
@@ -2970,7 +2980,7 @@
         </is>
       </c>
       <c r="B521" s="19">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Peluqueria/Estetica")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Peluqueria/Estetica")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="C521" s="20">
@@ -2993,7 +3003,7 @@
         </is>
       </c>
       <c r="B522" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Hogar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Hogar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="C522" s="18">
@@ -3016,7 +3026,7 @@
         </is>
       </c>
       <c r="B523" s="19">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="C523" s="20">
@@ -3039,7 +3049,7 @@
         </is>
       </c>
       <c r="B524" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Software/Apps")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Software/Apps")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="C524" s="18">
@@ -3062,7 +3072,7 @@
         </is>
       </c>
       <c r="B525" s="19">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="C525" s="20">
@@ -3085,7 +3095,7 @@
         </is>
       </c>
       <c r="B526" s="21">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="C526" s="22">
@@ -3216,7 +3226,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C5" s="31" t="n">
+      <c r="C5" s="32" t="n">
         <v>0</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -3229,7 +3239,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F5" s="31" t="n">
+      <c r="F5" s="32" t="n">
         <v>0</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -3242,7 +3252,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I5" s="31" t="n">
+      <c r="I5" s="32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3257,7 +3267,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C6" s="32" t="n">
+      <c r="C6" s="33" t="n">
         <v>0</v>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -3270,7 +3280,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F6" s="32" t="n">
+      <c r="F6" s="33" t="n">
         <v>0</v>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -3283,7 +3293,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I6" s="32" t="n">
+      <c r="I6" s="33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3298,7 +3308,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C7" s="33" t="n">
+      <c r="C7" s="34" t="n">
         <v>0</v>
       </c>
       <c r="D7" s="10" t="inlineStr">
@@ -3311,7 +3321,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F7" s="33" t="n">
+      <c r="F7" s="34" t="n">
         <v>0</v>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -3324,7 +3334,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I7" s="33" t="n">
+      <c r="I7" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3339,7 +3349,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C8" s="32" t="n">
+      <c r="C8" s="33" t="n">
         <v>0</v>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -3352,7 +3362,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F8" s="32" t="n">
+      <c r="F8" s="33" t="n">
         <v>0</v>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -3365,7 +3375,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I8" s="32" t="n">
+      <c r="I8" s="33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3380,7 +3390,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C9" s="33" t="n">
+      <c r="C9" s="34" t="n">
         <v>0</v>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -3393,7 +3403,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F9" s="33" t="n">
+      <c r="F9" s="34" t="n">
         <v>0</v>
       </c>
       <c r="G9" s="10" t="inlineStr">
@@ -3406,7 +3416,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I9" s="33" t="n">
+      <c r="I9" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3489,7 +3499,7 @@
           <t>Meses con datos de trading</t>
         </is>
       </c>
-      <c r="B6" s="34" t="n">
+      <c r="B6" s="35" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3505,12 +3515,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="35" t="inlineStr">
+      <c r="A9" s="36" t="inlineStr">
         <is>
           <t>Estado actual:</t>
         </is>
       </c>
-      <c r="B9" s="35">
+      <c r="B9" s="36">
         <f>"El trading cubre el "&amp;TEXT(B5,"0.0%")&amp;" de tus gastos mensuales fijos"</f>
         <v/>
       </c>
@@ -3658,7 +3668,7 @@
           <t>Rentabilidad anual inversion %</t>
         </is>
       </c>
-      <c r="B8" s="26" t="n">
+      <c r="B8" s="27" t="n">
         <v>0.05</v>
       </c>
     </row>
@@ -3916,7 +3926,7 @@
           <t>Actualiza con % cumplimiento ahorro</t>
         </is>
       </c>
-      <c r="D5" s="30" t="n">
+      <c r="D5" s="31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3936,7 +3946,7 @@
           <t>Actualiza con % cumplimiento bankroll</t>
         </is>
       </c>
-      <c r="D6" s="36" t="n">
+      <c r="D6" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3956,7 +3966,7 @@
           <t>Actualiza segun control de gastos</t>
         </is>
       </c>
-      <c r="D7" s="30" t="n">
+      <c r="D7" s="31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3976,7 +3986,7 @@
           <t>Actualiza con crecimiento patrimonio</t>
         </is>
       </c>
-      <c r="D8" s="36" t="n">
+      <c r="D8" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3996,7 +4006,7 @@
           <t>Actualiza con resultados de trading</t>
         </is>
       </c>
-      <c r="D9" s="30" t="n">
+      <c r="D9" s="31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4006,7 +4016,7 @@
           <t>SCORE TOTAL DEL TRADER (sobre 100)</t>
         </is>
       </c>
-      <c r="D10" s="37">
+      <c r="D10" s="38">
         <f>ROUND(SUM(D5:D9),1)</f>
         <v/>
       </c>
@@ -4346,11 +4356,11 @@
         <v/>
       </c>
       <c r="C7" s="14">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="E7" s="14">
-        <f>'PRESUPUESTO MENSUAL'!$D$3-(SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500)))</f>
+        <f>'PRESUPUESTO MENSUAL'!$D$3-(SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500)))</f>
         <v/>
       </c>
       <c r="G7" s="14">
@@ -4581,27 +4591,27 @@
     </row>
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="14">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Vivienda/Alquiler")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Vivienda/Alquiler")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="C24" s="14">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Coche/Transporte")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Coche/Transporte")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="E24" s="14">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Gasolina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Gasolina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="G24" s="14">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="I24" s="14">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="K24" s="14">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
     </row>
@@ -4640,27 +4650,27 @@
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="14">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="C27" s="14">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="E27" s="14">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="G27" s="14">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="I27" s="14">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="K27" s="14">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
     </row>
@@ -4742,7 +4752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J300"/>
+  <dimension ref="A1:J500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -8985,6 +8995,2806 @@
       </c>
       <c r="D300" s="24">
         <f>IF(A300="","",IF(OR(E300="Nomina",E300="Trading/Payout",E300="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="301">
+      <c r="B301" s="23">
+        <f>IF(A301="","",TEXT(A301,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C301" s="23">
+        <f>IF(A301="","",YEAR(A301))</f>
+        <v/>
+      </c>
+      <c r="D301" s="23">
+        <f>IF(A301="","",IF(OR(E301="Nomina",E301="Trading/Payout",E301="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="302">
+      <c r="B302" s="24">
+        <f>IF(A302="","",TEXT(A302,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C302" s="24">
+        <f>IF(A302="","",YEAR(A302))</f>
+        <v/>
+      </c>
+      <c r="D302" s="24">
+        <f>IF(A302="","",IF(OR(E302="Nomina",E302="Trading/Payout",E302="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="303">
+      <c r="B303" s="23">
+        <f>IF(A303="","",TEXT(A303,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C303" s="23">
+        <f>IF(A303="","",YEAR(A303))</f>
+        <v/>
+      </c>
+      <c r="D303" s="23">
+        <f>IF(A303="","",IF(OR(E303="Nomina",E303="Trading/Payout",E303="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="304">
+      <c r="B304" s="24">
+        <f>IF(A304="","",TEXT(A304,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C304" s="24">
+        <f>IF(A304="","",YEAR(A304))</f>
+        <v/>
+      </c>
+      <c r="D304" s="24">
+        <f>IF(A304="","",IF(OR(E304="Nomina",E304="Trading/Payout",E304="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="305">
+      <c r="B305" s="23">
+        <f>IF(A305="","",TEXT(A305,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C305" s="23">
+        <f>IF(A305="","",YEAR(A305))</f>
+        <v/>
+      </c>
+      <c r="D305" s="23">
+        <f>IF(A305="","",IF(OR(E305="Nomina",E305="Trading/Payout",E305="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="306">
+      <c r="B306" s="24">
+        <f>IF(A306="","",TEXT(A306,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C306" s="24">
+        <f>IF(A306="","",YEAR(A306))</f>
+        <v/>
+      </c>
+      <c r="D306" s="24">
+        <f>IF(A306="","",IF(OR(E306="Nomina",E306="Trading/Payout",E306="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="307">
+      <c r="B307" s="23">
+        <f>IF(A307="","",TEXT(A307,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C307" s="23">
+        <f>IF(A307="","",YEAR(A307))</f>
+        <v/>
+      </c>
+      <c r="D307" s="23">
+        <f>IF(A307="","",IF(OR(E307="Nomina",E307="Trading/Payout",E307="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="308">
+      <c r="B308" s="24">
+        <f>IF(A308="","",TEXT(A308,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C308" s="24">
+        <f>IF(A308="","",YEAR(A308))</f>
+        <v/>
+      </c>
+      <c r="D308" s="24">
+        <f>IF(A308="","",IF(OR(E308="Nomina",E308="Trading/Payout",E308="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="309">
+      <c r="B309" s="23">
+        <f>IF(A309="","",TEXT(A309,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C309" s="23">
+        <f>IF(A309="","",YEAR(A309))</f>
+        <v/>
+      </c>
+      <c r="D309" s="23">
+        <f>IF(A309="","",IF(OR(E309="Nomina",E309="Trading/Payout",E309="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="310">
+      <c r="B310" s="24">
+        <f>IF(A310="","",TEXT(A310,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C310" s="24">
+        <f>IF(A310="","",YEAR(A310))</f>
+        <v/>
+      </c>
+      <c r="D310" s="24">
+        <f>IF(A310="","",IF(OR(E310="Nomina",E310="Trading/Payout",E310="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="311">
+      <c r="B311" s="23">
+        <f>IF(A311="","",TEXT(A311,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C311" s="23">
+        <f>IF(A311="","",YEAR(A311))</f>
+        <v/>
+      </c>
+      <c r="D311" s="23">
+        <f>IF(A311="","",IF(OR(E311="Nomina",E311="Trading/Payout",E311="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="312">
+      <c r="B312" s="24">
+        <f>IF(A312="","",TEXT(A312,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C312" s="24">
+        <f>IF(A312="","",YEAR(A312))</f>
+        <v/>
+      </c>
+      <c r="D312" s="24">
+        <f>IF(A312="","",IF(OR(E312="Nomina",E312="Trading/Payout",E312="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="313">
+      <c r="B313" s="23">
+        <f>IF(A313="","",TEXT(A313,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C313" s="23">
+        <f>IF(A313="","",YEAR(A313))</f>
+        <v/>
+      </c>
+      <c r="D313" s="23">
+        <f>IF(A313="","",IF(OR(E313="Nomina",E313="Trading/Payout",E313="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="314">
+      <c r="B314" s="24">
+        <f>IF(A314="","",TEXT(A314,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C314" s="24">
+        <f>IF(A314="","",YEAR(A314))</f>
+        <v/>
+      </c>
+      <c r="D314" s="24">
+        <f>IF(A314="","",IF(OR(E314="Nomina",E314="Trading/Payout",E314="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="315">
+      <c r="B315" s="23">
+        <f>IF(A315="","",TEXT(A315,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C315" s="23">
+        <f>IF(A315="","",YEAR(A315))</f>
+        <v/>
+      </c>
+      <c r="D315" s="23">
+        <f>IF(A315="","",IF(OR(E315="Nomina",E315="Trading/Payout",E315="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="316">
+      <c r="B316" s="24">
+        <f>IF(A316="","",TEXT(A316,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C316" s="24">
+        <f>IF(A316="","",YEAR(A316))</f>
+        <v/>
+      </c>
+      <c r="D316" s="24">
+        <f>IF(A316="","",IF(OR(E316="Nomina",E316="Trading/Payout",E316="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="317">
+      <c r="B317" s="23">
+        <f>IF(A317="","",TEXT(A317,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C317" s="23">
+        <f>IF(A317="","",YEAR(A317))</f>
+        <v/>
+      </c>
+      <c r="D317" s="23">
+        <f>IF(A317="","",IF(OR(E317="Nomina",E317="Trading/Payout",E317="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="318">
+      <c r="B318" s="24">
+        <f>IF(A318="","",TEXT(A318,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C318" s="24">
+        <f>IF(A318="","",YEAR(A318))</f>
+        <v/>
+      </c>
+      <c r="D318" s="24">
+        <f>IF(A318="","",IF(OR(E318="Nomina",E318="Trading/Payout",E318="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="319">
+      <c r="B319" s="23">
+        <f>IF(A319="","",TEXT(A319,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C319" s="23">
+        <f>IF(A319="","",YEAR(A319))</f>
+        <v/>
+      </c>
+      <c r="D319" s="23">
+        <f>IF(A319="","",IF(OR(E319="Nomina",E319="Trading/Payout",E319="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="320">
+      <c r="B320" s="24">
+        <f>IF(A320="","",TEXT(A320,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C320" s="24">
+        <f>IF(A320="","",YEAR(A320))</f>
+        <v/>
+      </c>
+      <c r="D320" s="24">
+        <f>IF(A320="","",IF(OR(E320="Nomina",E320="Trading/Payout",E320="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="321">
+      <c r="B321" s="23">
+        <f>IF(A321="","",TEXT(A321,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C321" s="23">
+        <f>IF(A321="","",YEAR(A321))</f>
+        <v/>
+      </c>
+      <c r="D321" s="23">
+        <f>IF(A321="","",IF(OR(E321="Nomina",E321="Trading/Payout",E321="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="322">
+      <c r="B322" s="24">
+        <f>IF(A322="","",TEXT(A322,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C322" s="24">
+        <f>IF(A322="","",YEAR(A322))</f>
+        <v/>
+      </c>
+      <c r="D322" s="24">
+        <f>IF(A322="","",IF(OR(E322="Nomina",E322="Trading/Payout",E322="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="323">
+      <c r="B323" s="23">
+        <f>IF(A323="","",TEXT(A323,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C323" s="23">
+        <f>IF(A323="","",YEAR(A323))</f>
+        <v/>
+      </c>
+      <c r="D323" s="23">
+        <f>IF(A323="","",IF(OR(E323="Nomina",E323="Trading/Payout",E323="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="324">
+      <c r="B324" s="24">
+        <f>IF(A324="","",TEXT(A324,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C324" s="24">
+        <f>IF(A324="","",YEAR(A324))</f>
+        <v/>
+      </c>
+      <c r="D324" s="24">
+        <f>IF(A324="","",IF(OR(E324="Nomina",E324="Trading/Payout",E324="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="325">
+      <c r="B325" s="23">
+        <f>IF(A325="","",TEXT(A325,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C325" s="23">
+        <f>IF(A325="","",YEAR(A325))</f>
+        <v/>
+      </c>
+      <c r="D325" s="23">
+        <f>IF(A325="","",IF(OR(E325="Nomina",E325="Trading/Payout",E325="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="326">
+      <c r="B326" s="24">
+        <f>IF(A326="","",TEXT(A326,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C326" s="24">
+        <f>IF(A326="","",YEAR(A326))</f>
+        <v/>
+      </c>
+      <c r="D326" s="24">
+        <f>IF(A326="","",IF(OR(E326="Nomina",E326="Trading/Payout",E326="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="327">
+      <c r="B327" s="23">
+        <f>IF(A327="","",TEXT(A327,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C327" s="23">
+        <f>IF(A327="","",YEAR(A327))</f>
+        <v/>
+      </c>
+      <c r="D327" s="23">
+        <f>IF(A327="","",IF(OR(E327="Nomina",E327="Trading/Payout",E327="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="328">
+      <c r="B328" s="24">
+        <f>IF(A328="","",TEXT(A328,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C328" s="24">
+        <f>IF(A328="","",YEAR(A328))</f>
+        <v/>
+      </c>
+      <c r="D328" s="24">
+        <f>IF(A328="","",IF(OR(E328="Nomina",E328="Trading/Payout",E328="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="329">
+      <c r="B329" s="23">
+        <f>IF(A329="","",TEXT(A329,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C329" s="23">
+        <f>IF(A329="","",YEAR(A329))</f>
+        <v/>
+      </c>
+      <c r="D329" s="23">
+        <f>IF(A329="","",IF(OR(E329="Nomina",E329="Trading/Payout",E329="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="330">
+      <c r="B330" s="24">
+        <f>IF(A330="","",TEXT(A330,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C330" s="24">
+        <f>IF(A330="","",YEAR(A330))</f>
+        <v/>
+      </c>
+      <c r="D330" s="24">
+        <f>IF(A330="","",IF(OR(E330="Nomina",E330="Trading/Payout",E330="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="331">
+      <c r="B331" s="23">
+        <f>IF(A331="","",TEXT(A331,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C331" s="23">
+        <f>IF(A331="","",YEAR(A331))</f>
+        <v/>
+      </c>
+      <c r="D331" s="23">
+        <f>IF(A331="","",IF(OR(E331="Nomina",E331="Trading/Payout",E331="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="332">
+      <c r="B332" s="24">
+        <f>IF(A332="","",TEXT(A332,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C332" s="24">
+        <f>IF(A332="","",YEAR(A332))</f>
+        <v/>
+      </c>
+      <c r="D332" s="24">
+        <f>IF(A332="","",IF(OR(E332="Nomina",E332="Trading/Payout",E332="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="333">
+      <c r="B333" s="23">
+        <f>IF(A333="","",TEXT(A333,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C333" s="23">
+        <f>IF(A333="","",YEAR(A333))</f>
+        <v/>
+      </c>
+      <c r="D333" s="23">
+        <f>IF(A333="","",IF(OR(E333="Nomina",E333="Trading/Payout",E333="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="334">
+      <c r="B334" s="24">
+        <f>IF(A334="","",TEXT(A334,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C334" s="24">
+        <f>IF(A334="","",YEAR(A334))</f>
+        <v/>
+      </c>
+      <c r="D334" s="24">
+        <f>IF(A334="","",IF(OR(E334="Nomina",E334="Trading/Payout",E334="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="335">
+      <c r="B335" s="23">
+        <f>IF(A335="","",TEXT(A335,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C335" s="23">
+        <f>IF(A335="","",YEAR(A335))</f>
+        <v/>
+      </c>
+      <c r="D335" s="23">
+        <f>IF(A335="","",IF(OR(E335="Nomina",E335="Trading/Payout",E335="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="336">
+      <c r="B336" s="24">
+        <f>IF(A336="","",TEXT(A336,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C336" s="24">
+        <f>IF(A336="","",YEAR(A336))</f>
+        <v/>
+      </c>
+      <c r="D336" s="24">
+        <f>IF(A336="","",IF(OR(E336="Nomina",E336="Trading/Payout",E336="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="337">
+      <c r="B337" s="23">
+        <f>IF(A337="","",TEXT(A337,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C337" s="23">
+        <f>IF(A337="","",YEAR(A337))</f>
+        <v/>
+      </c>
+      <c r="D337" s="23">
+        <f>IF(A337="","",IF(OR(E337="Nomina",E337="Trading/Payout",E337="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="338">
+      <c r="B338" s="24">
+        <f>IF(A338="","",TEXT(A338,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C338" s="24">
+        <f>IF(A338="","",YEAR(A338))</f>
+        <v/>
+      </c>
+      <c r="D338" s="24">
+        <f>IF(A338="","",IF(OR(E338="Nomina",E338="Trading/Payout",E338="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="339">
+      <c r="B339" s="23">
+        <f>IF(A339="","",TEXT(A339,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C339" s="23">
+        <f>IF(A339="","",YEAR(A339))</f>
+        <v/>
+      </c>
+      <c r="D339" s="23">
+        <f>IF(A339="","",IF(OR(E339="Nomina",E339="Trading/Payout",E339="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="340">
+      <c r="B340" s="24">
+        <f>IF(A340="","",TEXT(A340,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C340" s="24">
+        <f>IF(A340="","",YEAR(A340))</f>
+        <v/>
+      </c>
+      <c r="D340" s="24">
+        <f>IF(A340="","",IF(OR(E340="Nomina",E340="Trading/Payout",E340="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="341">
+      <c r="B341" s="23">
+        <f>IF(A341="","",TEXT(A341,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C341" s="23">
+        <f>IF(A341="","",YEAR(A341))</f>
+        <v/>
+      </c>
+      <c r="D341" s="23">
+        <f>IF(A341="","",IF(OR(E341="Nomina",E341="Trading/Payout",E341="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="342">
+      <c r="B342" s="24">
+        <f>IF(A342="","",TEXT(A342,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C342" s="24">
+        <f>IF(A342="","",YEAR(A342))</f>
+        <v/>
+      </c>
+      <c r="D342" s="24">
+        <f>IF(A342="","",IF(OR(E342="Nomina",E342="Trading/Payout",E342="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="343">
+      <c r="B343" s="23">
+        <f>IF(A343="","",TEXT(A343,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C343" s="23">
+        <f>IF(A343="","",YEAR(A343))</f>
+        <v/>
+      </c>
+      <c r="D343" s="23">
+        <f>IF(A343="","",IF(OR(E343="Nomina",E343="Trading/Payout",E343="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="344">
+      <c r="B344" s="24">
+        <f>IF(A344="","",TEXT(A344,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C344" s="24">
+        <f>IF(A344="","",YEAR(A344))</f>
+        <v/>
+      </c>
+      <c r="D344" s="24">
+        <f>IF(A344="","",IF(OR(E344="Nomina",E344="Trading/Payout",E344="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="345">
+      <c r="B345" s="23">
+        <f>IF(A345="","",TEXT(A345,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C345" s="23">
+        <f>IF(A345="","",YEAR(A345))</f>
+        <v/>
+      </c>
+      <c r="D345" s="23">
+        <f>IF(A345="","",IF(OR(E345="Nomina",E345="Trading/Payout",E345="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="346">
+      <c r="B346" s="24">
+        <f>IF(A346="","",TEXT(A346,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C346" s="24">
+        <f>IF(A346="","",YEAR(A346))</f>
+        <v/>
+      </c>
+      <c r="D346" s="24">
+        <f>IF(A346="","",IF(OR(E346="Nomina",E346="Trading/Payout",E346="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="347">
+      <c r="B347" s="23">
+        <f>IF(A347="","",TEXT(A347,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C347" s="23">
+        <f>IF(A347="","",YEAR(A347))</f>
+        <v/>
+      </c>
+      <c r="D347" s="23">
+        <f>IF(A347="","",IF(OR(E347="Nomina",E347="Trading/Payout",E347="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="348">
+      <c r="B348" s="24">
+        <f>IF(A348="","",TEXT(A348,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C348" s="24">
+        <f>IF(A348="","",YEAR(A348))</f>
+        <v/>
+      </c>
+      <c r="D348" s="24">
+        <f>IF(A348="","",IF(OR(E348="Nomina",E348="Trading/Payout",E348="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="349">
+      <c r="B349" s="23">
+        <f>IF(A349="","",TEXT(A349,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C349" s="23">
+        <f>IF(A349="","",YEAR(A349))</f>
+        <v/>
+      </c>
+      <c r="D349" s="23">
+        <f>IF(A349="","",IF(OR(E349="Nomina",E349="Trading/Payout",E349="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="350">
+      <c r="B350" s="24">
+        <f>IF(A350="","",TEXT(A350,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C350" s="24">
+        <f>IF(A350="","",YEAR(A350))</f>
+        <v/>
+      </c>
+      <c r="D350" s="24">
+        <f>IF(A350="","",IF(OR(E350="Nomina",E350="Trading/Payout",E350="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="351">
+      <c r="B351" s="23">
+        <f>IF(A351="","",TEXT(A351,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C351" s="23">
+        <f>IF(A351="","",YEAR(A351))</f>
+        <v/>
+      </c>
+      <c r="D351" s="23">
+        <f>IF(A351="","",IF(OR(E351="Nomina",E351="Trading/Payout",E351="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="352">
+      <c r="B352" s="24">
+        <f>IF(A352="","",TEXT(A352,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C352" s="24">
+        <f>IF(A352="","",YEAR(A352))</f>
+        <v/>
+      </c>
+      <c r="D352" s="24">
+        <f>IF(A352="","",IF(OR(E352="Nomina",E352="Trading/Payout",E352="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="353">
+      <c r="B353" s="23">
+        <f>IF(A353="","",TEXT(A353,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C353" s="23">
+        <f>IF(A353="","",YEAR(A353))</f>
+        <v/>
+      </c>
+      <c r="D353" s="23">
+        <f>IF(A353="","",IF(OR(E353="Nomina",E353="Trading/Payout",E353="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="354">
+      <c r="B354" s="24">
+        <f>IF(A354="","",TEXT(A354,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C354" s="24">
+        <f>IF(A354="","",YEAR(A354))</f>
+        <v/>
+      </c>
+      <c r="D354" s="24">
+        <f>IF(A354="","",IF(OR(E354="Nomina",E354="Trading/Payout",E354="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="355">
+      <c r="B355" s="23">
+        <f>IF(A355="","",TEXT(A355,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C355" s="23">
+        <f>IF(A355="","",YEAR(A355))</f>
+        <v/>
+      </c>
+      <c r="D355" s="23">
+        <f>IF(A355="","",IF(OR(E355="Nomina",E355="Trading/Payout",E355="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="356">
+      <c r="B356" s="24">
+        <f>IF(A356="","",TEXT(A356,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C356" s="24">
+        <f>IF(A356="","",YEAR(A356))</f>
+        <v/>
+      </c>
+      <c r="D356" s="24">
+        <f>IF(A356="","",IF(OR(E356="Nomina",E356="Trading/Payout",E356="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="357">
+      <c r="B357" s="23">
+        <f>IF(A357="","",TEXT(A357,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C357" s="23">
+        <f>IF(A357="","",YEAR(A357))</f>
+        <v/>
+      </c>
+      <c r="D357" s="23">
+        <f>IF(A357="","",IF(OR(E357="Nomina",E357="Trading/Payout",E357="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="358">
+      <c r="B358" s="24">
+        <f>IF(A358="","",TEXT(A358,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C358" s="24">
+        <f>IF(A358="","",YEAR(A358))</f>
+        <v/>
+      </c>
+      <c r="D358" s="24">
+        <f>IF(A358="","",IF(OR(E358="Nomina",E358="Trading/Payout",E358="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="359">
+      <c r="B359" s="23">
+        <f>IF(A359="","",TEXT(A359,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C359" s="23">
+        <f>IF(A359="","",YEAR(A359))</f>
+        <v/>
+      </c>
+      <c r="D359" s="23">
+        <f>IF(A359="","",IF(OR(E359="Nomina",E359="Trading/Payout",E359="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="360">
+      <c r="B360" s="24">
+        <f>IF(A360="","",TEXT(A360,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C360" s="24">
+        <f>IF(A360="","",YEAR(A360))</f>
+        <v/>
+      </c>
+      <c r="D360" s="24">
+        <f>IF(A360="","",IF(OR(E360="Nomina",E360="Trading/Payout",E360="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="361">
+      <c r="B361" s="23">
+        <f>IF(A361="","",TEXT(A361,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C361" s="23">
+        <f>IF(A361="","",YEAR(A361))</f>
+        <v/>
+      </c>
+      <c r="D361" s="23">
+        <f>IF(A361="","",IF(OR(E361="Nomina",E361="Trading/Payout",E361="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="362">
+      <c r="B362" s="24">
+        <f>IF(A362="","",TEXT(A362,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C362" s="24">
+        <f>IF(A362="","",YEAR(A362))</f>
+        <v/>
+      </c>
+      <c r="D362" s="24">
+        <f>IF(A362="","",IF(OR(E362="Nomina",E362="Trading/Payout",E362="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="363">
+      <c r="B363" s="23">
+        <f>IF(A363="","",TEXT(A363,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C363" s="23">
+        <f>IF(A363="","",YEAR(A363))</f>
+        <v/>
+      </c>
+      <c r="D363" s="23">
+        <f>IF(A363="","",IF(OR(E363="Nomina",E363="Trading/Payout",E363="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="364">
+      <c r="B364" s="24">
+        <f>IF(A364="","",TEXT(A364,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C364" s="24">
+        <f>IF(A364="","",YEAR(A364))</f>
+        <v/>
+      </c>
+      <c r="D364" s="24">
+        <f>IF(A364="","",IF(OR(E364="Nomina",E364="Trading/Payout",E364="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="365">
+      <c r="B365" s="23">
+        <f>IF(A365="","",TEXT(A365,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C365" s="23">
+        <f>IF(A365="","",YEAR(A365))</f>
+        <v/>
+      </c>
+      <c r="D365" s="23">
+        <f>IF(A365="","",IF(OR(E365="Nomina",E365="Trading/Payout",E365="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="366">
+      <c r="B366" s="24">
+        <f>IF(A366="","",TEXT(A366,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C366" s="24">
+        <f>IF(A366="","",YEAR(A366))</f>
+        <v/>
+      </c>
+      <c r="D366" s="24">
+        <f>IF(A366="","",IF(OR(E366="Nomina",E366="Trading/Payout",E366="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="367">
+      <c r="B367" s="23">
+        <f>IF(A367="","",TEXT(A367,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C367" s="23">
+        <f>IF(A367="","",YEAR(A367))</f>
+        <v/>
+      </c>
+      <c r="D367" s="23">
+        <f>IF(A367="","",IF(OR(E367="Nomina",E367="Trading/Payout",E367="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="368">
+      <c r="B368" s="24">
+        <f>IF(A368="","",TEXT(A368,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C368" s="24">
+        <f>IF(A368="","",YEAR(A368))</f>
+        <v/>
+      </c>
+      <c r="D368" s="24">
+        <f>IF(A368="","",IF(OR(E368="Nomina",E368="Trading/Payout",E368="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="369">
+      <c r="B369" s="23">
+        <f>IF(A369="","",TEXT(A369,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C369" s="23">
+        <f>IF(A369="","",YEAR(A369))</f>
+        <v/>
+      </c>
+      <c r="D369" s="23">
+        <f>IF(A369="","",IF(OR(E369="Nomina",E369="Trading/Payout",E369="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="370">
+      <c r="B370" s="24">
+        <f>IF(A370="","",TEXT(A370,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C370" s="24">
+        <f>IF(A370="","",YEAR(A370))</f>
+        <v/>
+      </c>
+      <c r="D370" s="24">
+        <f>IF(A370="","",IF(OR(E370="Nomina",E370="Trading/Payout",E370="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="371">
+      <c r="B371" s="23">
+        <f>IF(A371="","",TEXT(A371,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C371" s="23">
+        <f>IF(A371="","",YEAR(A371))</f>
+        <v/>
+      </c>
+      <c r="D371" s="23">
+        <f>IF(A371="","",IF(OR(E371="Nomina",E371="Trading/Payout",E371="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="372">
+      <c r="B372" s="24">
+        <f>IF(A372="","",TEXT(A372,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C372" s="24">
+        <f>IF(A372="","",YEAR(A372))</f>
+        <v/>
+      </c>
+      <c r="D372" s="24">
+        <f>IF(A372="","",IF(OR(E372="Nomina",E372="Trading/Payout",E372="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="373">
+      <c r="B373" s="23">
+        <f>IF(A373="","",TEXT(A373,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C373" s="23">
+        <f>IF(A373="","",YEAR(A373))</f>
+        <v/>
+      </c>
+      <c r="D373" s="23">
+        <f>IF(A373="","",IF(OR(E373="Nomina",E373="Trading/Payout",E373="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="374">
+      <c r="B374" s="24">
+        <f>IF(A374="","",TEXT(A374,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C374" s="24">
+        <f>IF(A374="","",YEAR(A374))</f>
+        <v/>
+      </c>
+      <c r="D374" s="24">
+        <f>IF(A374="","",IF(OR(E374="Nomina",E374="Trading/Payout",E374="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="375">
+      <c r="B375" s="23">
+        <f>IF(A375="","",TEXT(A375,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C375" s="23">
+        <f>IF(A375="","",YEAR(A375))</f>
+        <v/>
+      </c>
+      <c r="D375" s="23">
+        <f>IF(A375="","",IF(OR(E375="Nomina",E375="Trading/Payout",E375="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="376">
+      <c r="B376" s="24">
+        <f>IF(A376="","",TEXT(A376,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C376" s="24">
+        <f>IF(A376="","",YEAR(A376))</f>
+        <v/>
+      </c>
+      <c r="D376" s="24">
+        <f>IF(A376="","",IF(OR(E376="Nomina",E376="Trading/Payout",E376="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="377">
+      <c r="B377" s="23">
+        <f>IF(A377="","",TEXT(A377,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C377" s="23">
+        <f>IF(A377="","",YEAR(A377))</f>
+        <v/>
+      </c>
+      <c r="D377" s="23">
+        <f>IF(A377="","",IF(OR(E377="Nomina",E377="Trading/Payout",E377="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="378">
+      <c r="B378" s="24">
+        <f>IF(A378="","",TEXT(A378,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C378" s="24">
+        <f>IF(A378="","",YEAR(A378))</f>
+        <v/>
+      </c>
+      <c r="D378" s="24">
+        <f>IF(A378="","",IF(OR(E378="Nomina",E378="Trading/Payout",E378="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="379">
+      <c r="B379" s="23">
+        <f>IF(A379="","",TEXT(A379,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C379" s="23">
+        <f>IF(A379="","",YEAR(A379))</f>
+        <v/>
+      </c>
+      <c r="D379" s="23">
+        <f>IF(A379="","",IF(OR(E379="Nomina",E379="Trading/Payout",E379="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="380">
+      <c r="B380" s="24">
+        <f>IF(A380="","",TEXT(A380,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C380" s="24">
+        <f>IF(A380="","",YEAR(A380))</f>
+        <v/>
+      </c>
+      <c r="D380" s="24">
+        <f>IF(A380="","",IF(OR(E380="Nomina",E380="Trading/Payout",E380="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="381">
+      <c r="B381" s="23">
+        <f>IF(A381="","",TEXT(A381,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C381" s="23">
+        <f>IF(A381="","",YEAR(A381))</f>
+        <v/>
+      </c>
+      <c r="D381" s="23">
+        <f>IF(A381="","",IF(OR(E381="Nomina",E381="Trading/Payout",E381="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="382">
+      <c r="B382" s="24">
+        <f>IF(A382="","",TEXT(A382,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C382" s="24">
+        <f>IF(A382="","",YEAR(A382))</f>
+        <v/>
+      </c>
+      <c r="D382" s="24">
+        <f>IF(A382="","",IF(OR(E382="Nomina",E382="Trading/Payout",E382="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="383">
+      <c r="B383" s="23">
+        <f>IF(A383="","",TEXT(A383,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C383" s="23">
+        <f>IF(A383="","",YEAR(A383))</f>
+        <v/>
+      </c>
+      <c r="D383" s="23">
+        <f>IF(A383="","",IF(OR(E383="Nomina",E383="Trading/Payout",E383="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="384">
+      <c r="B384" s="24">
+        <f>IF(A384="","",TEXT(A384,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C384" s="24">
+        <f>IF(A384="","",YEAR(A384))</f>
+        <v/>
+      </c>
+      <c r="D384" s="24">
+        <f>IF(A384="","",IF(OR(E384="Nomina",E384="Trading/Payout",E384="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="385">
+      <c r="B385" s="23">
+        <f>IF(A385="","",TEXT(A385,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C385" s="23">
+        <f>IF(A385="","",YEAR(A385))</f>
+        <v/>
+      </c>
+      <c r="D385" s="23">
+        <f>IF(A385="","",IF(OR(E385="Nomina",E385="Trading/Payout",E385="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="386">
+      <c r="B386" s="24">
+        <f>IF(A386="","",TEXT(A386,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C386" s="24">
+        <f>IF(A386="","",YEAR(A386))</f>
+        <v/>
+      </c>
+      <c r="D386" s="24">
+        <f>IF(A386="","",IF(OR(E386="Nomina",E386="Trading/Payout",E386="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="387">
+      <c r="B387" s="23">
+        <f>IF(A387="","",TEXT(A387,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C387" s="23">
+        <f>IF(A387="","",YEAR(A387))</f>
+        <v/>
+      </c>
+      <c r="D387" s="23">
+        <f>IF(A387="","",IF(OR(E387="Nomina",E387="Trading/Payout",E387="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="388">
+      <c r="B388" s="24">
+        <f>IF(A388="","",TEXT(A388,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C388" s="24">
+        <f>IF(A388="","",YEAR(A388))</f>
+        <v/>
+      </c>
+      <c r="D388" s="24">
+        <f>IF(A388="","",IF(OR(E388="Nomina",E388="Trading/Payout",E388="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="389">
+      <c r="B389" s="23">
+        <f>IF(A389="","",TEXT(A389,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C389" s="23">
+        <f>IF(A389="","",YEAR(A389))</f>
+        <v/>
+      </c>
+      <c r="D389" s="23">
+        <f>IF(A389="","",IF(OR(E389="Nomina",E389="Trading/Payout",E389="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="390">
+      <c r="B390" s="24">
+        <f>IF(A390="","",TEXT(A390,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C390" s="24">
+        <f>IF(A390="","",YEAR(A390))</f>
+        <v/>
+      </c>
+      <c r="D390" s="24">
+        <f>IF(A390="","",IF(OR(E390="Nomina",E390="Trading/Payout",E390="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="391">
+      <c r="B391" s="23">
+        <f>IF(A391="","",TEXT(A391,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C391" s="23">
+        <f>IF(A391="","",YEAR(A391))</f>
+        <v/>
+      </c>
+      <c r="D391" s="23">
+        <f>IF(A391="","",IF(OR(E391="Nomina",E391="Trading/Payout",E391="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="392">
+      <c r="B392" s="24">
+        <f>IF(A392="","",TEXT(A392,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C392" s="24">
+        <f>IF(A392="","",YEAR(A392))</f>
+        <v/>
+      </c>
+      <c r="D392" s="24">
+        <f>IF(A392="","",IF(OR(E392="Nomina",E392="Trading/Payout",E392="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="393">
+      <c r="B393" s="23">
+        <f>IF(A393="","",TEXT(A393,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C393" s="23">
+        <f>IF(A393="","",YEAR(A393))</f>
+        <v/>
+      </c>
+      <c r="D393" s="23">
+        <f>IF(A393="","",IF(OR(E393="Nomina",E393="Trading/Payout",E393="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="394">
+      <c r="B394" s="24">
+        <f>IF(A394="","",TEXT(A394,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C394" s="24">
+        <f>IF(A394="","",YEAR(A394))</f>
+        <v/>
+      </c>
+      <c r="D394" s="24">
+        <f>IF(A394="","",IF(OR(E394="Nomina",E394="Trading/Payout",E394="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="395">
+      <c r="B395" s="23">
+        <f>IF(A395="","",TEXT(A395,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C395" s="23">
+        <f>IF(A395="","",YEAR(A395))</f>
+        <v/>
+      </c>
+      <c r="D395" s="23">
+        <f>IF(A395="","",IF(OR(E395="Nomina",E395="Trading/Payout",E395="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="396">
+      <c r="B396" s="24">
+        <f>IF(A396="","",TEXT(A396,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C396" s="24">
+        <f>IF(A396="","",YEAR(A396))</f>
+        <v/>
+      </c>
+      <c r="D396" s="24">
+        <f>IF(A396="","",IF(OR(E396="Nomina",E396="Trading/Payout",E396="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="397">
+      <c r="B397" s="23">
+        <f>IF(A397="","",TEXT(A397,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C397" s="23">
+        <f>IF(A397="","",YEAR(A397))</f>
+        <v/>
+      </c>
+      <c r="D397" s="23">
+        <f>IF(A397="","",IF(OR(E397="Nomina",E397="Trading/Payout",E397="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="398">
+      <c r="B398" s="24">
+        <f>IF(A398="","",TEXT(A398,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C398" s="24">
+        <f>IF(A398="","",YEAR(A398))</f>
+        <v/>
+      </c>
+      <c r="D398" s="24">
+        <f>IF(A398="","",IF(OR(E398="Nomina",E398="Trading/Payout",E398="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="399">
+      <c r="B399" s="23">
+        <f>IF(A399="","",TEXT(A399,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C399" s="23">
+        <f>IF(A399="","",YEAR(A399))</f>
+        <v/>
+      </c>
+      <c r="D399" s="23">
+        <f>IF(A399="","",IF(OR(E399="Nomina",E399="Trading/Payout",E399="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="400">
+      <c r="B400" s="24">
+        <f>IF(A400="","",TEXT(A400,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C400" s="24">
+        <f>IF(A400="","",YEAR(A400))</f>
+        <v/>
+      </c>
+      <c r="D400" s="24">
+        <f>IF(A400="","",IF(OR(E400="Nomina",E400="Trading/Payout",E400="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="401">
+      <c r="B401" s="23">
+        <f>IF(A401="","",TEXT(A401,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C401" s="23">
+        <f>IF(A401="","",YEAR(A401))</f>
+        <v/>
+      </c>
+      <c r="D401" s="23">
+        <f>IF(A401="","",IF(OR(E401="Nomina",E401="Trading/Payout",E401="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="402">
+      <c r="B402" s="24">
+        <f>IF(A402="","",TEXT(A402,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C402" s="24">
+        <f>IF(A402="","",YEAR(A402))</f>
+        <v/>
+      </c>
+      <c r="D402" s="24">
+        <f>IF(A402="","",IF(OR(E402="Nomina",E402="Trading/Payout",E402="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="403">
+      <c r="B403" s="23">
+        <f>IF(A403="","",TEXT(A403,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C403" s="23">
+        <f>IF(A403="","",YEAR(A403))</f>
+        <v/>
+      </c>
+      <c r="D403" s="23">
+        <f>IF(A403="","",IF(OR(E403="Nomina",E403="Trading/Payout",E403="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="404">
+      <c r="B404" s="24">
+        <f>IF(A404="","",TEXT(A404,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C404" s="24">
+        <f>IF(A404="","",YEAR(A404))</f>
+        <v/>
+      </c>
+      <c r="D404" s="24">
+        <f>IF(A404="","",IF(OR(E404="Nomina",E404="Trading/Payout",E404="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="405">
+      <c r="B405" s="23">
+        <f>IF(A405="","",TEXT(A405,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C405" s="23">
+        <f>IF(A405="","",YEAR(A405))</f>
+        <v/>
+      </c>
+      <c r="D405" s="23">
+        <f>IF(A405="","",IF(OR(E405="Nomina",E405="Trading/Payout",E405="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="406">
+      <c r="B406" s="24">
+        <f>IF(A406="","",TEXT(A406,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C406" s="24">
+        <f>IF(A406="","",YEAR(A406))</f>
+        <v/>
+      </c>
+      <c r="D406" s="24">
+        <f>IF(A406="","",IF(OR(E406="Nomina",E406="Trading/Payout",E406="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="407">
+      <c r="B407" s="23">
+        <f>IF(A407="","",TEXT(A407,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C407" s="23">
+        <f>IF(A407="","",YEAR(A407))</f>
+        <v/>
+      </c>
+      <c r="D407" s="23">
+        <f>IF(A407="","",IF(OR(E407="Nomina",E407="Trading/Payout",E407="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="408">
+      <c r="B408" s="24">
+        <f>IF(A408="","",TEXT(A408,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C408" s="24">
+        <f>IF(A408="","",YEAR(A408))</f>
+        <v/>
+      </c>
+      <c r="D408" s="24">
+        <f>IF(A408="","",IF(OR(E408="Nomina",E408="Trading/Payout",E408="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="409">
+      <c r="B409" s="23">
+        <f>IF(A409="","",TEXT(A409,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C409" s="23">
+        <f>IF(A409="","",YEAR(A409))</f>
+        <v/>
+      </c>
+      <c r="D409" s="23">
+        <f>IF(A409="","",IF(OR(E409="Nomina",E409="Trading/Payout",E409="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="410">
+      <c r="B410" s="24">
+        <f>IF(A410="","",TEXT(A410,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C410" s="24">
+        <f>IF(A410="","",YEAR(A410))</f>
+        <v/>
+      </c>
+      <c r="D410" s="24">
+        <f>IF(A410="","",IF(OR(E410="Nomina",E410="Trading/Payout",E410="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="411">
+      <c r="B411" s="23">
+        <f>IF(A411="","",TEXT(A411,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C411" s="23">
+        <f>IF(A411="","",YEAR(A411))</f>
+        <v/>
+      </c>
+      <c r="D411" s="23">
+        <f>IF(A411="","",IF(OR(E411="Nomina",E411="Trading/Payout",E411="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="412">
+      <c r="B412" s="24">
+        <f>IF(A412="","",TEXT(A412,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C412" s="24">
+        <f>IF(A412="","",YEAR(A412))</f>
+        <v/>
+      </c>
+      <c r="D412" s="24">
+        <f>IF(A412="","",IF(OR(E412="Nomina",E412="Trading/Payout",E412="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="413">
+      <c r="B413" s="23">
+        <f>IF(A413="","",TEXT(A413,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C413" s="23">
+        <f>IF(A413="","",YEAR(A413))</f>
+        <v/>
+      </c>
+      <c r="D413" s="23">
+        <f>IF(A413="","",IF(OR(E413="Nomina",E413="Trading/Payout",E413="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="414">
+      <c r="B414" s="24">
+        <f>IF(A414="","",TEXT(A414,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C414" s="24">
+        <f>IF(A414="","",YEAR(A414))</f>
+        <v/>
+      </c>
+      <c r="D414" s="24">
+        <f>IF(A414="","",IF(OR(E414="Nomina",E414="Trading/Payout",E414="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="415">
+      <c r="B415" s="23">
+        <f>IF(A415="","",TEXT(A415,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C415" s="23">
+        <f>IF(A415="","",YEAR(A415))</f>
+        <v/>
+      </c>
+      <c r="D415" s="23">
+        <f>IF(A415="","",IF(OR(E415="Nomina",E415="Trading/Payout",E415="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="416">
+      <c r="B416" s="24">
+        <f>IF(A416="","",TEXT(A416,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C416" s="24">
+        <f>IF(A416="","",YEAR(A416))</f>
+        <v/>
+      </c>
+      <c r="D416" s="24">
+        <f>IF(A416="","",IF(OR(E416="Nomina",E416="Trading/Payout",E416="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="417">
+      <c r="B417" s="23">
+        <f>IF(A417="","",TEXT(A417,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C417" s="23">
+        <f>IF(A417="","",YEAR(A417))</f>
+        <v/>
+      </c>
+      <c r="D417" s="23">
+        <f>IF(A417="","",IF(OR(E417="Nomina",E417="Trading/Payout",E417="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="418">
+      <c r="B418" s="24">
+        <f>IF(A418="","",TEXT(A418,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C418" s="24">
+        <f>IF(A418="","",YEAR(A418))</f>
+        <v/>
+      </c>
+      <c r="D418" s="24">
+        <f>IF(A418="","",IF(OR(E418="Nomina",E418="Trading/Payout",E418="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="419">
+      <c r="B419" s="23">
+        <f>IF(A419="","",TEXT(A419,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C419" s="23">
+        <f>IF(A419="","",YEAR(A419))</f>
+        <v/>
+      </c>
+      <c r="D419" s="23">
+        <f>IF(A419="","",IF(OR(E419="Nomina",E419="Trading/Payout",E419="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="420">
+      <c r="B420" s="24">
+        <f>IF(A420="","",TEXT(A420,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C420" s="24">
+        <f>IF(A420="","",YEAR(A420))</f>
+        <v/>
+      </c>
+      <c r="D420" s="24">
+        <f>IF(A420="","",IF(OR(E420="Nomina",E420="Trading/Payout",E420="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="421">
+      <c r="B421" s="23">
+        <f>IF(A421="","",TEXT(A421,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C421" s="23">
+        <f>IF(A421="","",YEAR(A421))</f>
+        <v/>
+      </c>
+      <c r="D421" s="23">
+        <f>IF(A421="","",IF(OR(E421="Nomina",E421="Trading/Payout",E421="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="422">
+      <c r="B422" s="24">
+        <f>IF(A422="","",TEXT(A422,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C422" s="24">
+        <f>IF(A422="","",YEAR(A422))</f>
+        <v/>
+      </c>
+      <c r="D422" s="24">
+        <f>IF(A422="","",IF(OR(E422="Nomina",E422="Trading/Payout",E422="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="423">
+      <c r="B423" s="23">
+        <f>IF(A423="","",TEXT(A423,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C423" s="23">
+        <f>IF(A423="","",YEAR(A423))</f>
+        <v/>
+      </c>
+      <c r="D423" s="23">
+        <f>IF(A423="","",IF(OR(E423="Nomina",E423="Trading/Payout",E423="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="424">
+      <c r="B424" s="24">
+        <f>IF(A424="","",TEXT(A424,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C424" s="24">
+        <f>IF(A424="","",YEAR(A424))</f>
+        <v/>
+      </c>
+      <c r="D424" s="24">
+        <f>IF(A424="","",IF(OR(E424="Nomina",E424="Trading/Payout",E424="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="425">
+      <c r="B425" s="23">
+        <f>IF(A425="","",TEXT(A425,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C425" s="23">
+        <f>IF(A425="","",YEAR(A425))</f>
+        <v/>
+      </c>
+      <c r="D425" s="23">
+        <f>IF(A425="","",IF(OR(E425="Nomina",E425="Trading/Payout",E425="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="426">
+      <c r="B426" s="24">
+        <f>IF(A426="","",TEXT(A426,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C426" s="24">
+        <f>IF(A426="","",YEAR(A426))</f>
+        <v/>
+      </c>
+      <c r="D426" s="24">
+        <f>IF(A426="","",IF(OR(E426="Nomina",E426="Trading/Payout",E426="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="427">
+      <c r="B427" s="23">
+        <f>IF(A427="","",TEXT(A427,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C427" s="23">
+        <f>IF(A427="","",YEAR(A427))</f>
+        <v/>
+      </c>
+      <c r="D427" s="23">
+        <f>IF(A427="","",IF(OR(E427="Nomina",E427="Trading/Payout",E427="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="428">
+      <c r="B428" s="24">
+        <f>IF(A428="","",TEXT(A428,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C428" s="24">
+        <f>IF(A428="","",YEAR(A428))</f>
+        <v/>
+      </c>
+      <c r="D428" s="24">
+        <f>IF(A428="","",IF(OR(E428="Nomina",E428="Trading/Payout",E428="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="429">
+      <c r="B429" s="23">
+        <f>IF(A429="","",TEXT(A429,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C429" s="23">
+        <f>IF(A429="","",YEAR(A429))</f>
+        <v/>
+      </c>
+      <c r="D429" s="23">
+        <f>IF(A429="","",IF(OR(E429="Nomina",E429="Trading/Payout",E429="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="430">
+      <c r="B430" s="24">
+        <f>IF(A430="","",TEXT(A430,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C430" s="24">
+        <f>IF(A430="","",YEAR(A430))</f>
+        <v/>
+      </c>
+      <c r="D430" s="24">
+        <f>IF(A430="","",IF(OR(E430="Nomina",E430="Trading/Payout",E430="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="431">
+      <c r="B431" s="23">
+        <f>IF(A431="","",TEXT(A431,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C431" s="23">
+        <f>IF(A431="","",YEAR(A431))</f>
+        <v/>
+      </c>
+      <c r="D431" s="23">
+        <f>IF(A431="","",IF(OR(E431="Nomina",E431="Trading/Payout",E431="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="432">
+      <c r="B432" s="24">
+        <f>IF(A432="","",TEXT(A432,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C432" s="24">
+        <f>IF(A432="","",YEAR(A432))</f>
+        <v/>
+      </c>
+      <c r="D432" s="24">
+        <f>IF(A432="","",IF(OR(E432="Nomina",E432="Trading/Payout",E432="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="433">
+      <c r="B433" s="23">
+        <f>IF(A433="","",TEXT(A433,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C433" s="23">
+        <f>IF(A433="","",YEAR(A433))</f>
+        <v/>
+      </c>
+      <c r="D433" s="23">
+        <f>IF(A433="","",IF(OR(E433="Nomina",E433="Trading/Payout",E433="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="434">
+      <c r="B434" s="24">
+        <f>IF(A434="","",TEXT(A434,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C434" s="24">
+        <f>IF(A434="","",YEAR(A434))</f>
+        <v/>
+      </c>
+      <c r="D434" s="24">
+        <f>IF(A434="","",IF(OR(E434="Nomina",E434="Trading/Payout",E434="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="435">
+      <c r="B435" s="23">
+        <f>IF(A435="","",TEXT(A435,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C435" s="23">
+        <f>IF(A435="","",YEAR(A435))</f>
+        <v/>
+      </c>
+      <c r="D435" s="23">
+        <f>IF(A435="","",IF(OR(E435="Nomina",E435="Trading/Payout",E435="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="436">
+      <c r="B436" s="24">
+        <f>IF(A436="","",TEXT(A436,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C436" s="24">
+        <f>IF(A436="","",YEAR(A436))</f>
+        <v/>
+      </c>
+      <c r="D436" s="24">
+        <f>IF(A436="","",IF(OR(E436="Nomina",E436="Trading/Payout",E436="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="437">
+      <c r="B437" s="23">
+        <f>IF(A437="","",TEXT(A437,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C437" s="23">
+        <f>IF(A437="","",YEAR(A437))</f>
+        <v/>
+      </c>
+      <c r="D437" s="23">
+        <f>IF(A437="","",IF(OR(E437="Nomina",E437="Trading/Payout",E437="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="438">
+      <c r="B438" s="24">
+        <f>IF(A438="","",TEXT(A438,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C438" s="24">
+        <f>IF(A438="","",YEAR(A438))</f>
+        <v/>
+      </c>
+      <c r="D438" s="24">
+        <f>IF(A438="","",IF(OR(E438="Nomina",E438="Trading/Payout",E438="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="439">
+      <c r="B439" s="23">
+        <f>IF(A439="","",TEXT(A439,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C439" s="23">
+        <f>IF(A439="","",YEAR(A439))</f>
+        <v/>
+      </c>
+      <c r="D439" s="23">
+        <f>IF(A439="","",IF(OR(E439="Nomina",E439="Trading/Payout",E439="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="440">
+      <c r="B440" s="24">
+        <f>IF(A440="","",TEXT(A440,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C440" s="24">
+        <f>IF(A440="","",YEAR(A440))</f>
+        <v/>
+      </c>
+      <c r="D440" s="24">
+        <f>IF(A440="","",IF(OR(E440="Nomina",E440="Trading/Payout",E440="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="441">
+      <c r="B441" s="23">
+        <f>IF(A441="","",TEXT(A441,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C441" s="23">
+        <f>IF(A441="","",YEAR(A441))</f>
+        <v/>
+      </c>
+      <c r="D441" s="23">
+        <f>IF(A441="","",IF(OR(E441="Nomina",E441="Trading/Payout",E441="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="442">
+      <c r="B442" s="24">
+        <f>IF(A442="","",TEXT(A442,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C442" s="24">
+        <f>IF(A442="","",YEAR(A442))</f>
+        <v/>
+      </c>
+      <c r="D442" s="24">
+        <f>IF(A442="","",IF(OR(E442="Nomina",E442="Trading/Payout",E442="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="443">
+      <c r="B443" s="23">
+        <f>IF(A443="","",TEXT(A443,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C443" s="23">
+        <f>IF(A443="","",YEAR(A443))</f>
+        <v/>
+      </c>
+      <c r="D443" s="23">
+        <f>IF(A443="","",IF(OR(E443="Nomina",E443="Trading/Payout",E443="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="444">
+      <c r="B444" s="24">
+        <f>IF(A444="","",TEXT(A444,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C444" s="24">
+        <f>IF(A444="","",YEAR(A444))</f>
+        <v/>
+      </c>
+      <c r="D444" s="24">
+        <f>IF(A444="","",IF(OR(E444="Nomina",E444="Trading/Payout",E444="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="445">
+      <c r="B445" s="23">
+        <f>IF(A445="","",TEXT(A445,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C445" s="23">
+        <f>IF(A445="","",YEAR(A445))</f>
+        <v/>
+      </c>
+      <c r="D445" s="23">
+        <f>IF(A445="","",IF(OR(E445="Nomina",E445="Trading/Payout",E445="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="446">
+      <c r="B446" s="24">
+        <f>IF(A446="","",TEXT(A446,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C446" s="24">
+        <f>IF(A446="","",YEAR(A446))</f>
+        <v/>
+      </c>
+      <c r="D446" s="24">
+        <f>IF(A446="","",IF(OR(E446="Nomina",E446="Trading/Payout",E446="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="447">
+      <c r="B447" s="23">
+        <f>IF(A447="","",TEXT(A447,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C447" s="23">
+        <f>IF(A447="","",YEAR(A447))</f>
+        <v/>
+      </c>
+      <c r="D447" s="23">
+        <f>IF(A447="","",IF(OR(E447="Nomina",E447="Trading/Payout",E447="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="448">
+      <c r="B448" s="24">
+        <f>IF(A448="","",TEXT(A448,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C448" s="24">
+        <f>IF(A448="","",YEAR(A448))</f>
+        <v/>
+      </c>
+      <c r="D448" s="24">
+        <f>IF(A448="","",IF(OR(E448="Nomina",E448="Trading/Payout",E448="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="449">
+      <c r="B449" s="23">
+        <f>IF(A449="","",TEXT(A449,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C449" s="23">
+        <f>IF(A449="","",YEAR(A449))</f>
+        <v/>
+      </c>
+      <c r="D449" s="23">
+        <f>IF(A449="","",IF(OR(E449="Nomina",E449="Trading/Payout",E449="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="450">
+      <c r="B450" s="24">
+        <f>IF(A450="","",TEXT(A450,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C450" s="24">
+        <f>IF(A450="","",YEAR(A450))</f>
+        <v/>
+      </c>
+      <c r="D450" s="24">
+        <f>IF(A450="","",IF(OR(E450="Nomina",E450="Trading/Payout",E450="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="451">
+      <c r="B451" s="23">
+        <f>IF(A451="","",TEXT(A451,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C451" s="23">
+        <f>IF(A451="","",YEAR(A451))</f>
+        <v/>
+      </c>
+      <c r="D451" s="23">
+        <f>IF(A451="","",IF(OR(E451="Nomina",E451="Trading/Payout",E451="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="452">
+      <c r="B452" s="24">
+        <f>IF(A452="","",TEXT(A452,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C452" s="24">
+        <f>IF(A452="","",YEAR(A452))</f>
+        <v/>
+      </c>
+      <c r="D452" s="24">
+        <f>IF(A452="","",IF(OR(E452="Nomina",E452="Trading/Payout",E452="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="453">
+      <c r="B453" s="23">
+        <f>IF(A453="","",TEXT(A453,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C453" s="23">
+        <f>IF(A453="","",YEAR(A453))</f>
+        <v/>
+      </c>
+      <c r="D453" s="23">
+        <f>IF(A453="","",IF(OR(E453="Nomina",E453="Trading/Payout",E453="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="454">
+      <c r="B454" s="24">
+        <f>IF(A454="","",TEXT(A454,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C454" s="24">
+        <f>IF(A454="","",YEAR(A454))</f>
+        <v/>
+      </c>
+      <c r="D454" s="24">
+        <f>IF(A454="","",IF(OR(E454="Nomina",E454="Trading/Payout",E454="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="455">
+      <c r="B455" s="23">
+        <f>IF(A455="","",TEXT(A455,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C455" s="23">
+        <f>IF(A455="","",YEAR(A455))</f>
+        <v/>
+      </c>
+      <c r="D455" s="23">
+        <f>IF(A455="","",IF(OR(E455="Nomina",E455="Trading/Payout",E455="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="456">
+      <c r="B456" s="24">
+        <f>IF(A456="","",TEXT(A456,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C456" s="24">
+        <f>IF(A456="","",YEAR(A456))</f>
+        <v/>
+      </c>
+      <c r="D456" s="24">
+        <f>IF(A456="","",IF(OR(E456="Nomina",E456="Trading/Payout",E456="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="457">
+      <c r="B457" s="23">
+        <f>IF(A457="","",TEXT(A457,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C457" s="23">
+        <f>IF(A457="","",YEAR(A457))</f>
+        <v/>
+      </c>
+      <c r="D457" s="23">
+        <f>IF(A457="","",IF(OR(E457="Nomina",E457="Trading/Payout",E457="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="458">
+      <c r="B458" s="24">
+        <f>IF(A458="","",TEXT(A458,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C458" s="24">
+        <f>IF(A458="","",YEAR(A458))</f>
+        <v/>
+      </c>
+      <c r="D458" s="24">
+        <f>IF(A458="","",IF(OR(E458="Nomina",E458="Trading/Payout",E458="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="459">
+      <c r="B459" s="23">
+        <f>IF(A459="","",TEXT(A459,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C459" s="23">
+        <f>IF(A459="","",YEAR(A459))</f>
+        <v/>
+      </c>
+      <c r="D459" s="23">
+        <f>IF(A459="","",IF(OR(E459="Nomina",E459="Trading/Payout",E459="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="460">
+      <c r="B460" s="24">
+        <f>IF(A460="","",TEXT(A460,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C460" s="24">
+        <f>IF(A460="","",YEAR(A460))</f>
+        <v/>
+      </c>
+      <c r="D460" s="24">
+        <f>IF(A460="","",IF(OR(E460="Nomina",E460="Trading/Payout",E460="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="461">
+      <c r="B461" s="23">
+        <f>IF(A461="","",TEXT(A461,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C461" s="23">
+        <f>IF(A461="","",YEAR(A461))</f>
+        <v/>
+      </c>
+      <c r="D461" s="23">
+        <f>IF(A461="","",IF(OR(E461="Nomina",E461="Trading/Payout",E461="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="462">
+      <c r="B462" s="24">
+        <f>IF(A462="","",TEXT(A462,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C462" s="24">
+        <f>IF(A462="","",YEAR(A462))</f>
+        <v/>
+      </c>
+      <c r="D462" s="24">
+        <f>IF(A462="","",IF(OR(E462="Nomina",E462="Trading/Payout",E462="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="463">
+      <c r="B463" s="23">
+        <f>IF(A463="","",TEXT(A463,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C463" s="23">
+        <f>IF(A463="","",YEAR(A463))</f>
+        <v/>
+      </c>
+      <c r="D463" s="23">
+        <f>IF(A463="","",IF(OR(E463="Nomina",E463="Trading/Payout",E463="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="464">
+      <c r="B464" s="24">
+        <f>IF(A464="","",TEXT(A464,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C464" s="24">
+        <f>IF(A464="","",YEAR(A464))</f>
+        <v/>
+      </c>
+      <c r="D464" s="24">
+        <f>IF(A464="","",IF(OR(E464="Nomina",E464="Trading/Payout",E464="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="465">
+      <c r="B465" s="23">
+        <f>IF(A465="","",TEXT(A465,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C465" s="23">
+        <f>IF(A465="","",YEAR(A465))</f>
+        <v/>
+      </c>
+      <c r="D465" s="23">
+        <f>IF(A465="","",IF(OR(E465="Nomina",E465="Trading/Payout",E465="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="466">
+      <c r="B466" s="24">
+        <f>IF(A466="","",TEXT(A466,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C466" s="24">
+        <f>IF(A466="","",YEAR(A466))</f>
+        <v/>
+      </c>
+      <c r="D466" s="24">
+        <f>IF(A466="","",IF(OR(E466="Nomina",E466="Trading/Payout",E466="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="467">
+      <c r="B467" s="23">
+        <f>IF(A467="","",TEXT(A467,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C467" s="23">
+        <f>IF(A467="","",YEAR(A467))</f>
+        <v/>
+      </c>
+      <c r="D467" s="23">
+        <f>IF(A467="","",IF(OR(E467="Nomina",E467="Trading/Payout",E467="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="468">
+      <c r="B468" s="24">
+        <f>IF(A468="","",TEXT(A468,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C468" s="24">
+        <f>IF(A468="","",YEAR(A468))</f>
+        <v/>
+      </c>
+      <c r="D468" s="24">
+        <f>IF(A468="","",IF(OR(E468="Nomina",E468="Trading/Payout",E468="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="469">
+      <c r="B469" s="23">
+        <f>IF(A469="","",TEXT(A469,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C469" s="23">
+        <f>IF(A469="","",YEAR(A469))</f>
+        <v/>
+      </c>
+      <c r="D469" s="23">
+        <f>IF(A469="","",IF(OR(E469="Nomina",E469="Trading/Payout",E469="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="470">
+      <c r="B470" s="24">
+        <f>IF(A470="","",TEXT(A470,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C470" s="24">
+        <f>IF(A470="","",YEAR(A470))</f>
+        <v/>
+      </c>
+      <c r="D470" s="24">
+        <f>IF(A470="","",IF(OR(E470="Nomina",E470="Trading/Payout",E470="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="471">
+      <c r="B471" s="23">
+        <f>IF(A471="","",TEXT(A471,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C471" s="23">
+        <f>IF(A471="","",YEAR(A471))</f>
+        <v/>
+      </c>
+      <c r="D471" s="23">
+        <f>IF(A471="","",IF(OR(E471="Nomina",E471="Trading/Payout",E471="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="472">
+      <c r="B472" s="24">
+        <f>IF(A472="","",TEXT(A472,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C472" s="24">
+        <f>IF(A472="","",YEAR(A472))</f>
+        <v/>
+      </c>
+      <c r="D472" s="24">
+        <f>IF(A472="","",IF(OR(E472="Nomina",E472="Trading/Payout",E472="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="473">
+      <c r="B473" s="23">
+        <f>IF(A473="","",TEXT(A473,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C473" s="23">
+        <f>IF(A473="","",YEAR(A473))</f>
+        <v/>
+      </c>
+      <c r="D473" s="23">
+        <f>IF(A473="","",IF(OR(E473="Nomina",E473="Trading/Payout",E473="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="474">
+      <c r="B474" s="24">
+        <f>IF(A474="","",TEXT(A474,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C474" s="24">
+        <f>IF(A474="","",YEAR(A474))</f>
+        <v/>
+      </c>
+      <c r="D474" s="24">
+        <f>IF(A474="","",IF(OR(E474="Nomina",E474="Trading/Payout",E474="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="475">
+      <c r="B475" s="23">
+        <f>IF(A475="","",TEXT(A475,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C475" s="23">
+        <f>IF(A475="","",YEAR(A475))</f>
+        <v/>
+      </c>
+      <c r="D475" s="23">
+        <f>IF(A475="","",IF(OR(E475="Nomina",E475="Trading/Payout",E475="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="476">
+      <c r="B476" s="24">
+        <f>IF(A476="","",TEXT(A476,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C476" s="24">
+        <f>IF(A476="","",YEAR(A476))</f>
+        <v/>
+      </c>
+      <c r="D476" s="24">
+        <f>IF(A476="","",IF(OR(E476="Nomina",E476="Trading/Payout",E476="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="477">
+      <c r="B477" s="23">
+        <f>IF(A477="","",TEXT(A477,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C477" s="23">
+        <f>IF(A477="","",YEAR(A477))</f>
+        <v/>
+      </c>
+      <c r="D477" s="23">
+        <f>IF(A477="","",IF(OR(E477="Nomina",E477="Trading/Payout",E477="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="478">
+      <c r="B478" s="24">
+        <f>IF(A478="","",TEXT(A478,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C478" s="24">
+        <f>IF(A478="","",YEAR(A478))</f>
+        <v/>
+      </c>
+      <c r="D478" s="24">
+        <f>IF(A478="","",IF(OR(E478="Nomina",E478="Trading/Payout",E478="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="479">
+      <c r="B479" s="23">
+        <f>IF(A479="","",TEXT(A479,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C479" s="23">
+        <f>IF(A479="","",YEAR(A479))</f>
+        <v/>
+      </c>
+      <c r="D479" s="23">
+        <f>IF(A479="","",IF(OR(E479="Nomina",E479="Trading/Payout",E479="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="480">
+      <c r="B480" s="24">
+        <f>IF(A480="","",TEXT(A480,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C480" s="24">
+        <f>IF(A480="","",YEAR(A480))</f>
+        <v/>
+      </c>
+      <c r="D480" s="24">
+        <f>IF(A480="","",IF(OR(E480="Nomina",E480="Trading/Payout",E480="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="481">
+      <c r="B481" s="23">
+        <f>IF(A481="","",TEXT(A481,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C481" s="23">
+        <f>IF(A481="","",YEAR(A481))</f>
+        <v/>
+      </c>
+      <c r="D481" s="23">
+        <f>IF(A481="","",IF(OR(E481="Nomina",E481="Trading/Payout",E481="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="482">
+      <c r="B482" s="24">
+        <f>IF(A482="","",TEXT(A482,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C482" s="24">
+        <f>IF(A482="","",YEAR(A482))</f>
+        <v/>
+      </c>
+      <c r="D482" s="24">
+        <f>IF(A482="","",IF(OR(E482="Nomina",E482="Trading/Payout",E482="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="483">
+      <c r="B483" s="23">
+        <f>IF(A483="","",TEXT(A483,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C483" s="23">
+        <f>IF(A483="","",YEAR(A483))</f>
+        <v/>
+      </c>
+      <c r="D483" s="23">
+        <f>IF(A483="","",IF(OR(E483="Nomina",E483="Trading/Payout",E483="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="484">
+      <c r="B484" s="24">
+        <f>IF(A484="","",TEXT(A484,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C484" s="24">
+        <f>IF(A484="","",YEAR(A484))</f>
+        <v/>
+      </c>
+      <c r="D484" s="24">
+        <f>IF(A484="","",IF(OR(E484="Nomina",E484="Trading/Payout",E484="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="485">
+      <c r="B485" s="23">
+        <f>IF(A485="","",TEXT(A485,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C485" s="23">
+        <f>IF(A485="","",YEAR(A485))</f>
+        <v/>
+      </c>
+      <c r="D485" s="23">
+        <f>IF(A485="","",IF(OR(E485="Nomina",E485="Trading/Payout",E485="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="486">
+      <c r="B486" s="24">
+        <f>IF(A486="","",TEXT(A486,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C486" s="24">
+        <f>IF(A486="","",YEAR(A486))</f>
+        <v/>
+      </c>
+      <c r="D486" s="24">
+        <f>IF(A486="","",IF(OR(E486="Nomina",E486="Trading/Payout",E486="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="487">
+      <c r="B487" s="23">
+        <f>IF(A487="","",TEXT(A487,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C487" s="23">
+        <f>IF(A487="","",YEAR(A487))</f>
+        <v/>
+      </c>
+      <c r="D487" s="23">
+        <f>IF(A487="","",IF(OR(E487="Nomina",E487="Trading/Payout",E487="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="488">
+      <c r="B488" s="24">
+        <f>IF(A488="","",TEXT(A488,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C488" s="24">
+        <f>IF(A488="","",YEAR(A488))</f>
+        <v/>
+      </c>
+      <c r="D488" s="24">
+        <f>IF(A488="","",IF(OR(E488="Nomina",E488="Trading/Payout",E488="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="489">
+      <c r="B489" s="23">
+        <f>IF(A489="","",TEXT(A489,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C489" s="23">
+        <f>IF(A489="","",YEAR(A489))</f>
+        <v/>
+      </c>
+      <c r="D489" s="23">
+        <f>IF(A489="","",IF(OR(E489="Nomina",E489="Trading/Payout",E489="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="490">
+      <c r="B490" s="24">
+        <f>IF(A490="","",TEXT(A490,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C490" s="24">
+        <f>IF(A490="","",YEAR(A490))</f>
+        <v/>
+      </c>
+      <c r="D490" s="24">
+        <f>IF(A490="","",IF(OR(E490="Nomina",E490="Trading/Payout",E490="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="491">
+      <c r="B491" s="23">
+        <f>IF(A491="","",TEXT(A491,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C491" s="23">
+        <f>IF(A491="","",YEAR(A491))</f>
+        <v/>
+      </c>
+      <c r="D491" s="23">
+        <f>IF(A491="","",IF(OR(E491="Nomina",E491="Trading/Payout",E491="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="492">
+      <c r="B492" s="24">
+        <f>IF(A492="","",TEXT(A492,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C492" s="24">
+        <f>IF(A492="","",YEAR(A492))</f>
+        <v/>
+      </c>
+      <c r="D492" s="24">
+        <f>IF(A492="","",IF(OR(E492="Nomina",E492="Trading/Payout",E492="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="493">
+      <c r="B493" s="23">
+        <f>IF(A493="","",TEXT(A493,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C493" s="23">
+        <f>IF(A493="","",YEAR(A493))</f>
+        <v/>
+      </c>
+      <c r="D493" s="23">
+        <f>IF(A493="","",IF(OR(E493="Nomina",E493="Trading/Payout",E493="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="494">
+      <c r="B494" s="24">
+        <f>IF(A494="","",TEXT(A494,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C494" s="24">
+        <f>IF(A494="","",YEAR(A494))</f>
+        <v/>
+      </c>
+      <c r="D494" s="24">
+        <f>IF(A494="","",IF(OR(E494="Nomina",E494="Trading/Payout",E494="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="495">
+      <c r="B495" s="23">
+        <f>IF(A495="","",TEXT(A495,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C495" s="23">
+        <f>IF(A495="","",YEAR(A495))</f>
+        <v/>
+      </c>
+      <c r="D495" s="23">
+        <f>IF(A495="","",IF(OR(E495="Nomina",E495="Trading/Payout",E495="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="496">
+      <c r="B496" s="24">
+        <f>IF(A496="","",TEXT(A496,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C496" s="24">
+        <f>IF(A496="","",YEAR(A496))</f>
+        <v/>
+      </c>
+      <c r="D496" s="24">
+        <f>IF(A496="","",IF(OR(E496="Nomina",E496="Trading/Payout",E496="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="497">
+      <c r="B497" s="23">
+        <f>IF(A497="","",TEXT(A497,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C497" s="23">
+        <f>IF(A497="","",YEAR(A497))</f>
+        <v/>
+      </c>
+      <c r="D497" s="23">
+        <f>IF(A497="","",IF(OR(E497="Nomina",E497="Trading/Payout",E497="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="498">
+      <c r="B498" s="24">
+        <f>IF(A498="","",TEXT(A498,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C498" s="24">
+        <f>IF(A498="","",YEAR(A498))</f>
+        <v/>
+      </c>
+      <c r="D498" s="24">
+        <f>IF(A498="","",IF(OR(E498="Nomina",E498="Trading/Payout",E498="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="499">
+      <c r="B499" s="23">
+        <f>IF(A499="","",TEXT(A499,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C499" s="23">
+        <f>IF(A499="","",YEAR(A499))</f>
+        <v/>
+      </c>
+      <c r="D499" s="23">
+        <f>IF(A499="","",IF(OR(E499="Nomina",E499="Trading/Payout",E499="Otro ingreso"),"Ingreso","Gasto"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="500">
+      <c r="B500" s="24">
+        <f>IF(A500="","",TEXT(A500,"MMMM"))</f>
+        <v/>
+      </c>
+      <c r="C500" s="24">
+        <f>IF(A500="","",YEAR(A500))</f>
+        <v/>
+      </c>
+      <c r="D500" s="24">
+        <f>IF(A500="","",IF(OR(E500="Nomina",E500="Trading/Payout",E500="Otro ingreso"),"Ingreso","Gasto"))</f>
         <v/>
       </c>
     </row>
@@ -9047,6 +11857,28 @@
         </is>
       </c>
     </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>PERIODO A ANALIZAR:</t>
+        </is>
+      </c>
+      <c r="B5" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="C5" s="2">
+        <f>TEXT(DATE($E$5,$B$5,1),"MMMM YYYY")</f>
+        <v/>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Ano:</t>
+        </is>
+      </c>
+      <c r="E5" s="26" t="n">
+        <v>2026</v>
+      </c>
+    </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -9295,7 +12127,7 @@
           <t>Caprichos y ocio (% del sobrante)</t>
         </is>
       </c>
-      <c r="B19" s="26" t="n">
+      <c r="B19" s="27" t="n">
         <v>0.2</v>
       </c>
       <c r="C19" s="19">
@@ -9522,7 +12354,7 @@
         <v/>
       </c>
       <c r="C41" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Vivienda/Alquiler")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Vivienda/Alquiler")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="D41" s="17">
@@ -9545,7 +12377,7 @@
         <v/>
       </c>
       <c r="C42" s="19">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Coche/Transporte")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Coche/Transporte")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="D42" s="19">
@@ -9567,7 +12399,7 @@
         <v>80</v>
       </c>
       <c r="C43" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Gasolina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Gasolina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="D43" s="17">
@@ -9589,7 +12421,7 @@
         <v>200</v>
       </c>
       <c r="C44" s="19">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="D44" s="19">
@@ -9611,7 +12443,7 @@
         <v>100</v>
       </c>
       <c r="C45" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="D45" s="17">
@@ -9633,7 +12465,7 @@
         <v>40</v>
       </c>
       <c r="C46" s="19">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="D46" s="19">
@@ -9655,7 +12487,7 @@
         <v>80</v>
       </c>
       <c r="C47" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="D47" s="17">
@@ -9677,7 +12509,7 @@
         <v>60</v>
       </c>
       <c r="C48" s="19">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="D48" s="19">
@@ -9699,7 +12531,7 @@
         <v>40</v>
       </c>
       <c r="C49" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="D49" s="17">
@@ -9722,7 +12554,7 @@
         <v/>
       </c>
       <c r="C50" s="19">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Deporte/Gimnasio")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Deporte/Gimnasio")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="D50" s="19">
@@ -9745,7 +12577,7 @@
         <v/>
       </c>
       <c r="C51" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="D51" s="17">
@@ -9768,7 +12600,7 @@
         <v/>
       </c>
       <c r="C52" s="19">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="D52" s="19">
@@ -9791,7 +12623,7 @@
         <v/>
       </c>
       <c r="C53" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="D53" s="17">
@@ -9813,7 +12645,7 @@
         <v>50</v>
       </c>
       <c r="C54" s="19">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="D54" s="19">
@@ -9832,7 +12664,7 @@
         </is>
       </c>
       <c r="C55" s="21">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="D55" s="21">
@@ -9851,7 +12683,7 @@
         </is>
       </c>
       <c r="C56" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
     </row>
@@ -9913,6 +12745,12 @@
       <formula>0.9</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Mes invalido" error="Introduce un numero entre 1 y 12" type="whole" operator="between">
+      <formula1>1</formula1>
+      <formula2>12</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -10052,7 +12890,7 @@
         </is>
       </c>
       <c r="B13" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="C13" s="10" t="inlineStr">
@@ -10205,7 +13043,7 @@
         </is>
       </c>
       <c r="B11" s="17">
-        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=MONTH(TODAY()))*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=YEAR(TODAY()))*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$B$5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))='PRESUPUESTO MENSUAL'!$E$5)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
         <v/>
       </c>
       <c r="C11" s="10" t="inlineStr">
@@ -10383,7 +13221,7 @@
           <t>Numero de entradas</t>
         </is>
       </c>
-      <c r="B510" s="27">
+      <c r="B510" s="28">
         <f>COUNTA(B3:B500)</f>
         <v/>
       </c>
@@ -10653,7 +13491,7 @@
           <t>TOTAL ACTIVOS</t>
         </is>
       </c>
-      <c r="B10" s="28">
+      <c r="B10" s="29">
         <f>SUM(B5:B9)</f>
         <v/>
       </c>
@@ -10721,7 +13559,7 @@
           <t>TOTAL PASIVOS</t>
         </is>
       </c>
-      <c r="B17" s="29">
+      <c r="B17" s="30">
         <f>SUM(B14:B16)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Nueva hoja COMPARATIVA MENSUAL - resumen automatico enero-diciembre
Muestra en una sola tabla todos los meses del año 2026 con:
- Ingresos por categoria (Nomina, Trading, Otros)
- Gastos fijos por categoria (Vivienda, Coche, Gimnasio...)
- Gastos variables por categoria (Supermercado, Restaurante, Ocio...)
- Inversion/Ahorro (Ahorro, Bankroll, TraderLab)
- Fila resumen: Total Gastos | Total Ingresos | Ahorro Real | % Ahorro
- Verde si ahorro real > 0, rojo si negativo
- Grafico de barras Ingresos vs Gastos vs Ahorro por mes
- Columnas TOTAL 2026 y MEDIA/mes para vision anual
Los datos se rellenan solos cuando introduces registros con la fecha
correcta en REGISTRO DE MOVIMIENTOS. Cada mes es independiente.

https://claude.ai/code/session_01EdLrBe1U3fRxvoA6PYaJVC
</commit_message>
<xml_diff>
--- a/sistema_financiero.xlsx
+++ b/sistema_financiero.xlsx
@@ -19,11 +19,12 @@
     <sheet name="FONDO DE EMERGENCIA" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="OBJETIVOS" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="GASTOS HORMIGA" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="RANKING MEJORES MESES" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="LIBERTAD FINANCIERA" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="PROYECCIONES FUTURAS" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="SCORE DEL TRADER" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="_LISTAS" sheetId="17" state="hidden" r:id="rId17"/>
+    <sheet name="COMPARATIVA MENSUAL" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="RANKING MEJORES MESES" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="LIBERTAD FINANCIERA" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="PROYECCIONES FUTURAS" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="SCORE DEL TRADER" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="_LISTAS" sheetId="18" state="hidden" r:id="rId18"/>
   </sheets>
   <definedNames>
     <definedName name="ListaCategorias">_LISTAS!$A$1:$A$25</definedName>
@@ -40,11 +41,12 @@
     <definedName name="_xlnm.Print_Area" localSheetId="9">'FONDO DE EMERGENCIA'!$A$1:$F$28</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="10">'OBJETIVOS'!$A$1:$H$11</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="11">'GASTOS HORMIGA'!$A$1:$I$531</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="12">'RANKING MEJORES MESES'!$A$1:$K$17</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="13">'LIBERTAD FINANCIERA'!$A$1:$F$20</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="14">'PROYECCIONES FUTURAS'!$A$1:$H$21</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="15">'SCORE DEL TRADER'!$A$1:$F$22</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="16">'_LISTAS'!$A$1:$C$30</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="12">'COMPARATIVA MENSUAL'!$A$1:$Q$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="13">'RANKING MEJORES MESES'!$A$1:$K$17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="14">'LIBERTAD FINANCIERA'!$A$1:$F$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="15">'PROYECCIONES FUTURAS'!$A$1:$H$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="16">'SCORE DEL TRADER'!$A$1:$F$22</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="17">'_LISTAS'!$A$1:$C$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -271,7 +273,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -364,6 +366,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="17">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="26">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="23">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
@@ -1132,6 +1143,782 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:t>Ingresos vs Gastos por Mes 2026</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>Ingresos</v>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="28A745"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$41</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Gastos</v>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="DC3545"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$C$41</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>Ahorro Real</v>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="007BFF"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$D$41</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$E$41</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$F$41</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$G$41</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$H$41</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="7"/>
+          <order val="7"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$I$41</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="8"/>
+          <order val="8"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$J$41</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="9"/>
+          <order val="9"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$K$41</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="10"/>
+          <order val="10"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$L$41</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="11"/>
+          <order val="11"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$M$41</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="12"/>
+          <order val="12"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="13"/>
+          <order val="13"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$C$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="14"/>
+          <order val="14"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$D$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="15"/>
+          <order val="15"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$E$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="16"/>
+          <order val="16"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$F$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="17"/>
+          <order val="17"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$G$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="18"/>
+          <order val="18"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$H$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="19"/>
+          <order val="19"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$I$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="20"/>
+          <order val="20"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$J$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="21"/>
+          <order val="21"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$K$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="22"/>
+          <order val="22"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$L$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="23"/>
+          <order val="23"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$M$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="24"/>
+          <order val="24"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$42</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="25"/>
+          <order val="25"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$C$42</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="26"/>
+          <order val="26"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$D$42</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="27"/>
+          <order val="27"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$E$42</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="28"/>
+          <order val="28"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$F$42</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="29"/>
+          <order val="29"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$G$42</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="30"/>
+          <order val="30"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$H$42</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="31"/>
+          <order val="31"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$I$42</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="32"/>
+          <order val="32"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$J$42</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="33"/>
+          <order val="33"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$K$42</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="34"/>
+          <order val="34"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$L$42</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="35"/>
+          <order val="35"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$B$4:$M$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'COMPARATIVA MENSUAL'!$M$42</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>EUR</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
               <a:t>Proyeccion Patrimonial a 5 Anos</a:t>
             </a:r>
           </a:p>
@@ -1517,6 +2304,33 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>45</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10080000" cy="5040000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
       <col>7</col>
       <colOff>0</colOff>
       <row>3</row>
@@ -2057,46 +2871,58 @@
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>RANKING MEJORES MESES</t>
+          <t>COMPARATIVA MENSUAL</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Ranking de mejores meses. Actualiza con tus datos.</t>
+          <t>Tabla automatica mes a mes: ingresos, gastos y ahorro real enero-diciembre.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>LIBERTAD FINANCIERA</t>
+          <t>RANKING MEJORES MESES</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Mide el porcentaje de cobertura de gastos con ingresos de trading.</t>
+          <t>Ranking de mejores meses. Actualiza con tus datos.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>PROYECCIONES FUTURAS</t>
+          <t>LIBERTAD FINANCIERA</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>Proyecciones a 1, 3 y 5 anos basadas en parametros actuales.</t>
+          <t>Mide el porcentaje de cobertura de gastos con ingresos de trading.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
         <is>
+          <t>PROYECCIONES FUTURAS</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Proyecciones a 1, 3 y 5 anos basadas en parametros actuales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
           <t>SCORE DEL TRADER</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B30" s="10" t="inlineStr">
         <is>
           <t>Puntuacion 0-100 que evalua tu desempeno financiero.</t>
         </is>
@@ -3127,6 +3953,2073 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00007BFF"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:O43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>COMPARATIVA MENSUAL 2026 - EVOLUCION MES A MES (automatico desde REGISTRO DE MOVIMIENTOS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cada columna es un mes. Los datos se rellenan solos cuando introduces registros con la fecha correcta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Categoria / Concepto</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Ene</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Abr</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>Ago</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="M4" s="7" t="inlineStr">
+        <is>
+          <t>Dic</t>
+        </is>
+      </c>
+      <c r="N4" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL 2026</t>
+        </is>
+      </c>
+      <c r="O4" s="7" t="inlineStr">
+        <is>
+          <t>MEDIA/mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>INGRESOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Nomina</t>
+        </is>
+      </c>
+      <c r="B6" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Nomina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C6" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Nomina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D6" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Nomina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E6" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Nomina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F6" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Nomina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G6" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Nomina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H6" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Nomina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I6" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Nomina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J6" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Nomina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K6" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Nomina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L6" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Nomina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M6" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Nomina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N6" s="32">
+        <f>SUM(B6:M6)</f>
+        <v/>
+      </c>
+      <c r="O6" s="32">
+        <f>IFERROR(N6/COUNTIF(B6:M6,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Trading/Payout</t>
+        </is>
+      </c>
+      <c r="B7" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Trading/Payout")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C7" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Trading/Payout")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D7" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Trading/Payout")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E7" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Trading/Payout")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F7" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Trading/Payout")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G7" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Trading/Payout")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H7" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Trading/Payout")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I7" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Trading/Payout")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J7" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Trading/Payout")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K7" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Trading/Payout")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L7" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Trading/Payout")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M7" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Trading/Payout")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N7" s="32">
+        <f>SUM(B7:M7)</f>
+        <v/>
+      </c>
+      <c r="O7" s="32">
+        <f>IFERROR(N7/COUNTIF(B7:M7,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Otro ingreso</t>
+        </is>
+      </c>
+      <c r="B8" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otro ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C8" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otro ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D8" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otro ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E8" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otro ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F8" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otro ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G8" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otro ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H8" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otro ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I8" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otro ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J8" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otro ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K8" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otro ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L8" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otro ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M8" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otro ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N8" s="32">
+        <f>SUM(B8:M8)</f>
+        <v/>
+      </c>
+      <c r="O8" s="32">
+        <f>IFERROR(N8/COUNTIF(B8:M8,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL INGRESOS</t>
+        </is>
+      </c>
+      <c r="B9" s="21">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C9" s="21">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D9" s="21">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E9" s="21">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F9" s="21">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G9" s="21">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H9" s="21">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I9" s="21">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J9" s="21">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K9" s="21">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L9" s="21">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M9" s="21">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N9" s="21">
+        <f>SUM(B9:M9)</f>
+        <v/>
+      </c>
+      <c r="O9" s="21">
+        <f>IFERROR(N9/12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>GASTOS FIJOS (mensuales constantes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Vivienda/Alquiler</t>
+        </is>
+      </c>
+      <c r="B12" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Vivienda/Alquiler")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C12" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Vivienda/Alquiler")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D12" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Vivienda/Alquiler")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E12" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Vivienda/Alquiler")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F12" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Vivienda/Alquiler")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G12" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Vivienda/Alquiler")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H12" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Vivienda/Alquiler")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I12" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Vivienda/Alquiler")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J12" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Vivienda/Alquiler")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K12" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Vivienda/Alquiler")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L12" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Vivienda/Alquiler")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M12" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Vivienda/Alquiler")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N12" s="33">
+        <f>SUM(B12:M12)</f>
+        <v/>
+      </c>
+      <c r="O12" s="33">
+        <f>IFERROR(N12/COUNTIF(B12:M12,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Coche/Transporte</t>
+        </is>
+      </c>
+      <c r="B13" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Coche/Transporte")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C13" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Coche/Transporte")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D13" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Coche/Transporte")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E13" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Coche/Transporte")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F13" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Coche/Transporte")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G13" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Coche/Transporte")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H13" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Coche/Transporte")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I13" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Coche/Transporte")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J13" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Coche/Transporte")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K13" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Coche/Transporte")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L13" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Coche/Transporte")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M13" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Coche/Transporte")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N13" s="34">
+        <f>SUM(B13:M13)</f>
+        <v/>
+      </c>
+      <c r="O13" s="34">
+        <f>IFERROR(N13/COUNTIF(B13:M13,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Gasolina</t>
+        </is>
+      </c>
+      <c r="B14" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Gasolina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C14" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Gasolina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D14" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Gasolina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E14" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Gasolina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F14" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Gasolina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G14" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Gasolina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H14" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Gasolina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I14" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Gasolina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J14" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Gasolina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K14" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Gasolina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L14" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Gasolina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M14" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Gasolina")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N14" s="33">
+        <f>SUM(B14:M14)</f>
+        <v/>
+      </c>
+      <c r="O14" s="33">
+        <f>IFERROR(N14/COUNTIF(B14:M14,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Deporte/Gimnasio</t>
+        </is>
+      </c>
+      <c r="B15" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Deporte/Gimnasio")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C15" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Deporte/Gimnasio")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D15" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Deporte/Gimnasio")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E15" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Deporte/Gimnasio")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F15" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Deporte/Gimnasio")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G15" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Deporte/Gimnasio")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H15" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Deporte/Gimnasio")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I15" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Deporte/Gimnasio")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J15" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Deporte/Gimnasio")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K15" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Deporte/Gimnasio")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L15" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Deporte/Gimnasio")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M15" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Deporte/Gimnasio")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N15" s="34">
+        <f>SUM(B15:M15)</f>
+        <v/>
+      </c>
+      <c r="O15" s="34">
+        <f>IFERROR(N15/COUNTIF(B15:M15,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Formacion/Suscripciones</t>
+        </is>
+      </c>
+      <c r="B16" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C16" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D16" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E16" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F16" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G16" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H16" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I16" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J16" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K16" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L16" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M16" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Formacion/Suscripciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N16" s="33">
+        <f>SUM(B16:M16)</f>
+        <v/>
+      </c>
+      <c r="O16" s="33">
+        <f>IFERROR(N16/COUNTIF(B16:M16,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL GASTOS FIJOS</t>
+        </is>
+      </c>
+      <c r="B17" s="21">
+        <f>SUM(B12:B16)</f>
+        <v/>
+      </c>
+      <c r="C17" s="21">
+        <f>SUM(C12:C16)</f>
+        <v/>
+      </c>
+      <c r="D17" s="21">
+        <f>SUM(D12:D16)</f>
+        <v/>
+      </c>
+      <c r="E17" s="21">
+        <f>SUM(E12:E16)</f>
+        <v/>
+      </c>
+      <c r="F17" s="21">
+        <f>SUM(F12:F16)</f>
+        <v/>
+      </c>
+      <c r="G17" s="21">
+        <f>SUM(G12:G16)</f>
+        <v/>
+      </c>
+      <c r="H17" s="21">
+        <f>SUM(H12:H16)</f>
+        <v/>
+      </c>
+      <c r="I17" s="21">
+        <f>SUM(I12:I16)</f>
+        <v/>
+      </c>
+      <c r="J17" s="21">
+        <f>SUM(J12:J16)</f>
+        <v/>
+      </c>
+      <c r="K17" s="21">
+        <f>SUM(K12:K16)</f>
+        <v/>
+      </c>
+      <c r="L17" s="21">
+        <f>SUM(L12:L16)</f>
+        <v/>
+      </c>
+      <c r="M17" s="21">
+        <f>SUM(M12:M16)</f>
+        <v/>
+      </c>
+      <c r="N17" s="21">
+        <f>SUM(B17:M17)</f>
+        <v/>
+      </c>
+      <c r="O17" s="21">
+        <f>IFERROR(N17/12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>GASTOS VARIABLES (lo que gastas de mas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Supermercado</t>
+        </is>
+      </c>
+      <c r="B20" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C20" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D20" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E20" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F20" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G20" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H20" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I20" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J20" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K20" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L20" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M20" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Supermercado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N20" s="33">
+        <f>SUM(B20:M20)</f>
+        <v/>
+      </c>
+      <c r="O20" s="33">
+        <f>IFERROR(N20/COUNTIF(B20:M20,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Restaurante</t>
+        </is>
+      </c>
+      <c r="B21" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C21" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D21" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E21" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F21" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G21" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H21" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I21" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J21" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K21" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L21" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M21" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Restaurante")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N21" s="34">
+        <f>SUM(B21:M21)</f>
+        <v/>
+      </c>
+      <c r="O21" s="34">
+        <f>IFERROR(N21/COUNTIF(B21:M21,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>Cafeteria/Bar</t>
+        </is>
+      </c>
+      <c r="B22" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C22" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D22" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E22" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F22" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G22" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H22" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I22" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J22" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K22" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L22" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M22" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Cafeteria/Bar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N22" s="33">
+        <f>SUM(B22:M22)</f>
+        <v/>
+      </c>
+      <c r="O22" s="33">
+        <f>IFERROR(N22/COUNTIF(B22:M22,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Ocio/Entretenimiento</t>
+        </is>
+      </c>
+      <c r="B23" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C23" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D23" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E23" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F23" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G23" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H23" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I23" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J23" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K23" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L23" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M23" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ocio/Entretenimiento")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N23" s="34">
+        <f>SUM(B23:M23)</f>
+        <v/>
+      </c>
+      <c r="O23" s="34">
+        <f>IFERROR(N23/COUNTIF(B23:M23,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>Ropa/Calzado</t>
+        </is>
+      </c>
+      <c r="B24" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C24" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D24" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E24" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F24" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G24" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H24" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I24" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J24" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K24" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L24" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M24" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ropa/Calzado")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N24" s="33">
+        <f>SUM(B24:M24)</f>
+        <v/>
+      </c>
+      <c r="O24" s="33">
+        <f>IFERROR(N24/COUNTIF(B24:M24,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Farmacia/Salud</t>
+        </is>
+      </c>
+      <c r="B25" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C25" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D25" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E25" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F25" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G25" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H25" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I25" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J25" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K25" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L25" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M25" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Farmacia/Salud")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N25" s="34">
+        <f>SUM(B25:M25)</f>
+        <v/>
+      </c>
+      <c r="O25" s="34">
+        <f>IFERROR(N25/COUNTIF(B25:M25,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>Peluqueria/Estetica</t>
+        </is>
+      </c>
+      <c r="B26" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Peluqueria/Estetica")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C26" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Peluqueria/Estetica")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D26" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Peluqueria/Estetica")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E26" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Peluqueria/Estetica")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F26" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Peluqueria/Estetica")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G26" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Peluqueria/Estetica")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H26" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Peluqueria/Estetica")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I26" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Peluqueria/Estetica")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J26" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Peluqueria/Estetica")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K26" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Peluqueria/Estetica")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L26" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Peluqueria/Estetica")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M26" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Peluqueria/Estetica")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N26" s="33">
+        <f>SUM(B26:M26)</f>
+        <v/>
+      </c>
+      <c r="O26" s="33">
+        <f>IFERROR(N26/COUNTIF(B26:M26,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Electronica/Amazon</t>
+        </is>
+      </c>
+      <c r="B27" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Electronica/Amazon")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C27" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Electronica/Amazon")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D27" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Electronica/Amazon")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E27" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Electronica/Amazon")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F27" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Electronica/Amazon")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G27" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Electronica/Amazon")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H27" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Electronica/Amazon")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I27" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Electronica/Amazon")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J27" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Electronica/Amazon")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K27" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Electronica/Amazon")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L27" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Electronica/Amazon")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M27" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Electronica/Amazon")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N27" s="34">
+        <f>SUM(B27:M27)</f>
+        <v/>
+      </c>
+      <c r="O27" s="34">
+        <f>IFERROR(N27/COUNTIF(B27:M27,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>Hogar</t>
+        </is>
+      </c>
+      <c r="B28" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Hogar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C28" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Hogar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D28" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Hogar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E28" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Hogar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F28" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Hogar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G28" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Hogar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H28" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Hogar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I28" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Hogar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J28" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Hogar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K28" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Hogar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L28" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Hogar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M28" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Hogar")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N28" s="33">
+        <f>SUM(B28:M28)</f>
+        <v/>
+      </c>
+      <c r="O28" s="33">
+        <f>IFERROR(N28/COUNTIF(B28:M28,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Software/Apps</t>
+        </is>
+      </c>
+      <c r="B29" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Software/Apps")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C29" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Software/Apps")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D29" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Software/Apps")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E29" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Software/Apps")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F29" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Software/Apps")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G29" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Software/Apps")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H29" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Software/Apps")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I29" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Software/Apps")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J29" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Software/Apps")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K29" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Software/Apps")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L29" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Software/Apps")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M29" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Software/Apps")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N29" s="34">
+        <f>SUM(B29:M29)</f>
+        <v/>
+      </c>
+      <c r="O29" s="34">
+        <f>IFERROR(N29/COUNTIF(B29:M29,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>Viajes/Vacaciones</t>
+        </is>
+      </c>
+      <c r="B30" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Viajes/Vacaciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C30" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Viajes/Vacaciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D30" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Viajes/Vacaciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E30" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Viajes/Vacaciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F30" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Viajes/Vacaciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G30" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Viajes/Vacaciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H30" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Viajes/Vacaciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I30" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Viajes/Vacaciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J30" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Viajes/Vacaciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K30" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Viajes/Vacaciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L30" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Viajes/Vacaciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M30" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Viajes/Vacaciones")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N30" s="33">
+        <f>SUM(B30:M30)</f>
+        <v/>
+      </c>
+      <c r="O30" s="33">
+        <f>IFERROR(N30/COUNTIF(B30:M30,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
+      <c r="B31" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C31" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D31" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E31" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F31" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G31" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H31" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I31" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J31" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K31" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L31" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M31" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Otros")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N31" s="34">
+        <f>SUM(B31:M31)</f>
+        <v/>
+      </c>
+      <c r="O31" s="34">
+        <f>IFERROR(N31/COUNTIF(B31:M31,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL GASTOS VARIABLES</t>
+        </is>
+      </c>
+      <c r="B32" s="21">
+        <f>SUM(B20:B31)</f>
+        <v/>
+      </c>
+      <c r="C32" s="21">
+        <f>SUM(C20:C31)</f>
+        <v/>
+      </c>
+      <c r="D32" s="21">
+        <f>SUM(D20:D31)</f>
+        <v/>
+      </c>
+      <c r="E32" s="21">
+        <f>SUM(E20:E31)</f>
+        <v/>
+      </c>
+      <c r="F32" s="21">
+        <f>SUM(F20:F31)</f>
+        <v/>
+      </c>
+      <c r="G32" s="21">
+        <f>SUM(G20:G31)</f>
+        <v/>
+      </c>
+      <c r="H32" s="21">
+        <f>SUM(H20:H31)</f>
+        <v/>
+      </c>
+      <c r="I32" s="21">
+        <f>SUM(I20:I31)</f>
+        <v/>
+      </c>
+      <c r="J32" s="21">
+        <f>SUM(J20:J31)</f>
+        <v/>
+      </c>
+      <c r="K32" s="21">
+        <f>SUM(K20:K31)</f>
+        <v/>
+      </c>
+      <c r="L32" s="21">
+        <f>SUM(L20:L31)</f>
+        <v/>
+      </c>
+      <c r="M32" s="21">
+        <f>SUM(M20:M31)</f>
+        <v/>
+      </c>
+      <c r="N32" s="21">
+        <f>SUM(B32:M32)</f>
+        <v/>
+      </c>
+      <c r="O32" s="21">
+        <f>IFERROR(N32/12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>INVERSION Y AHORRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Ahorro</t>
+        </is>
+      </c>
+      <c r="B35" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C35" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D35" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E35" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F35" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G35" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H35" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I35" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J35" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K35" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L35" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M35" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Ahorro")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N35" s="34">
+        <f>SUM(B35:M35)</f>
+        <v/>
+      </c>
+      <c r="O35" s="34">
+        <f>IFERROR(N35/COUNTIF(B35:M35,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>Bankroll</t>
+        </is>
+      </c>
+      <c r="B36" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C36" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D36" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E36" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F36" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G36" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H36" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I36" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J36" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K36" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L36" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M36" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="Bankroll")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N36" s="33">
+        <f>SUM(B36:M36)</f>
+        <v/>
+      </c>
+      <c r="O36" s="33">
+        <f>IFERROR(N36/COUNTIF(B36:M36,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>TraderLab</t>
+        </is>
+      </c>
+      <c r="B37" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="TraderLab")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C37" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="TraderLab")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D37" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="TraderLab")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E37" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="TraderLab")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F37" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="TraderLab")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G37" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="TraderLab")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H37" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="TraderLab")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I37" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="TraderLab")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J37" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="TraderLab")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K37" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="TraderLab")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L37" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="TraderLab")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M37" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$E$3:$E$500="TraderLab")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N37" s="34">
+        <f>SUM(B37:M37)</f>
+        <v/>
+      </c>
+      <c r="O37" s="34">
+        <f>IFERROR(N37/COUNTIF(B37:M37,"&gt;0"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>RESUMEN FINAL POR MES</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL GASTOS DEL MES</t>
+        </is>
+      </c>
+      <c r="B40" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C40" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D40" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E40" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F40" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G40" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H40" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I40" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J40" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K40" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L40" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M40" s="19">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Gasto")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N40" s="32">
+        <f>SUM(B40:M40)</f>
+        <v/>
+      </c>
+      <c r="O40" s="32">
+        <f>IFERROR(N40/12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL INGRESOS DEL MES</t>
+        </is>
+      </c>
+      <c r="B41" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=1)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="C41" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="D41" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=3)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="E41" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=4)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="F41" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=5)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="G41" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=6)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="H41" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=7)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="I41" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=8)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="J41" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=9)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="K41" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=10)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="L41" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=11)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="M41" s="17">
+        <f>SUMPRODUCT((ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500))*(MONTH(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=12)*(YEAR(IF(ISNUMBER('REGISTRO DE MOVIMIENTOS'!$A$3:$A$500),'REGISTRO DE MOVIMIENTOS'!$A$3:$A$500,TODAY()))=2026)*('REGISTRO DE MOVIMIENTOS'!$D$3:$D$500="Ingreso")*('REGISTRO DE MOVIMIENTOS'!$H$3:$H$500))</f>
+        <v/>
+      </c>
+      <c r="N41" s="33">
+        <f>SUM(B41:M41)</f>
+        <v/>
+      </c>
+      <c r="O41" s="33">
+        <f>IFERROR(N41/12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>AHORRO REAL (Ingresos - Gastos)</t>
+        </is>
+      </c>
+      <c r="B42" s="21">
+        <f>B41-B40</f>
+        <v/>
+      </c>
+      <c r="C42" s="21">
+        <f>C41-C40</f>
+        <v/>
+      </c>
+      <c r="D42" s="21">
+        <f>D41-D40</f>
+        <v/>
+      </c>
+      <c r="E42" s="21">
+        <f>E41-E40</f>
+        <v/>
+      </c>
+      <c r="F42" s="21">
+        <f>F41-F40</f>
+        <v/>
+      </c>
+      <c r="G42" s="21">
+        <f>G41-G40</f>
+        <v/>
+      </c>
+      <c r="H42" s="21">
+        <f>H41-H40</f>
+        <v/>
+      </c>
+      <c r="I42" s="21">
+        <f>I41-I40</f>
+        <v/>
+      </c>
+      <c r="J42" s="21">
+        <f>J41-J40</f>
+        <v/>
+      </c>
+      <c r="K42" s="21">
+        <f>K41-K40</f>
+        <v/>
+      </c>
+      <c r="L42" s="21">
+        <f>L41-L40</f>
+        <v/>
+      </c>
+      <c r="M42" s="21">
+        <f>M41-M40</f>
+        <v/>
+      </c>
+      <c r="N42" s="21">
+        <f>SUM(B42:M42)</f>
+        <v/>
+      </c>
+      <c r="O42" s="21">
+        <f>IFERROR(N42/12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>% Ahorro real / Ingresos</t>
+        </is>
+      </c>
+      <c r="B43" s="18">
+        <f>IFERROR(B42/B41,0)</f>
+        <v/>
+      </c>
+      <c r="C43" s="18">
+        <f>IFERROR(C42/C41,0)</f>
+        <v/>
+      </c>
+      <c r="D43" s="18">
+        <f>IFERROR(D42/D41,0)</f>
+        <v/>
+      </c>
+      <c r="E43" s="18">
+        <f>IFERROR(E42/E41,0)</f>
+        <v/>
+      </c>
+      <c r="F43" s="18">
+        <f>IFERROR(F42/F41,0)</f>
+        <v/>
+      </c>
+      <c r="G43" s="18">
+        <f>IFERROR(G42/G41,0)</f>
+        <v/>
+      </c>
+      <c r="H43" s="18">
+        <f>IFERROR(H42/H41,0)</f>
+        <v/>
+      </c>
+      <c r="I43" s="18">
+        <f>IFERROR(I42/I41,0)</f>
+        <v/>
+      </c>
+      <c r="J43" s="18">
+        <f>IFERROR(J42/J41,0)</f>
+        <v/>
+      </c>
+      <c r="K43" s="18">
+        <f>IFERROR(K42/K41,0)</f>
+        <v/>
+      </c>
+      <c r="L43" s="18">
+        <f>IFERROR(L42/L41,0)</f>
+        <v/>
+      </c>
+      <c r="M43" s="18">
+        <f>IFERROR(M42/M41,0)</f>
+        <v/>
+      </c>
+      <c r="N43" s="18">
+        <f>IFERROR(N42/N41,0)</f>
+        <v/>
+      </c>
+      <c r="O43" s="18">
+        <f>IFERROR(AVERAGE(B43:M43),0)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A2:O2"/>
+    <mergeCell ref="A19:O19"/>
+    <mergeCell ref="A11:O11"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A5:O5"/>
+    <mergeCell ref="A34:O34"/>
+    <mergeCell ref="A39:O39"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B42:M42">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="lessThanOrEqual" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="0020C997"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
@@ -3226,7 +6119,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C5" s="32" t="n">
+      <c r="C5" s="35" t="n">
         <v>0</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -3239,7 +6132,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F5" s="32" t="n">
+      <c r="F5" s="35" t="n">
         <v>0</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -3252,7 +6145,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I5" s="32" t="n">
+      <c r="I5" s="35" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3267,7 +6160,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C6" s="33" t="n">
+      <c r="C6" s="36" t="n">
         <v>0</v>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -3280,7 +6173,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F6" s="33" t="n">
+      <c r="F6" s="36" t="n">
         <v>0</v>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -3293,7 +6186,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I6" s="33" t="n">
+      <c r="I6" s="36" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3308,7 +6201,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C7" s="34" t="n">
+      <c r="C7" s="37" t="n">
         <v>0</v>
       </c>
       <c r="D7" s="10" t="inlineStr">
@@ -3321,7 +6214,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F7" s="34" t="n">
+      <c r="F7" s="37" t="n">
         <v>0</v>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -3334,7 +6227,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I7" s="34" t="n">
+      <c r="I7" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3349,7 +6242,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C8" s="33" t="n">
+      <c r="C8" s="36" t="n">
         <v>0</v>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -3362,7 +6255,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F8" s="33" t="n">
+      <c r="F8" s="36" t="n">
         <v>0</v>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -3375,7 +6268,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I8" s="33" t="n">
+      <c r="I8" s="36" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3390,7 +6283,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C9" s="34" t="n">
+      <c r="C9" s="37" t="n">
         <v>0</v>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -3403,7 +6296,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F9" s="34" t="n">
+      <c r="F9" s="37" t="n">
         <v>0</v>
       </c>
       <c r="G9" s="10" t="inlineStr">
@@ -3416,7 +6309,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I9" s="34" t="n">
+      <c r="I9" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3440,7 +6333,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="0020C997"/>
@@ -3499,7 +6392,7 @@
           <t>Meses con datos de trading</t>
         </is>
       </c>
-      <c r="B6" s="35" t="n">
+      <c r="B6" s="38" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3515,12 +6408,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="36" t="inlineStr">
+      <c r="A9" s="39" t="inlineStr">
         <is>
           <t>Estado actual:</t>
         </is>
       </c>
-      <c r="B9" s="36">
+      <c r="B9" s="39">
         <f>"El trading cubre el "&amp;TEXT(B5,"0.0%")&amp;" de tus gastos mensuales fijos"</f>
         <v/>
       </c>
@@ -3590,7 +6483,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="0020C997"/>
@@ -3858,7 +6751,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00FD7E14"/>
@@ -3946,7 +6839,7 @@
           <t>Actualiza con % cumplimiento bankroll</t>
         </is>
       </c>
-      <c r="D6" s="37" t="n">
+      <c r="D6" s="40" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3986,7 +6879,7 @@
           <t>Actualiza con crecimiento patrimonio</t>
         </is>
       </c>
-      <c r="D8" s="37" t="n">
+      <c r="D8" s="40" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4016,7 +6909,7 @@
           <t>SCORE TOTAL DEL TRADER (sobre 100)</t>
         </is>
       </c>
-      <c r="D10" s="38">
+      <c r="D10" s="41">
         <f>ROUND(SUM(D5:D9),1)</f>
         <v/>
       </c>
@@ -4076,7 +6969,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>